<commit_message>
feat: add explicit run paces and split sessions
</commit_message>
<xml_diff>
--- a/source_plan_v2.xlsx
+++ b/source_plan_v2.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAZA 1 - OSLO V2" sheetId="1" r:id="R985a4829a39a41b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TYGODNIE I BRAMKI" sheetId="2" r:id="Ra80e8a5e080f4020"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STRATEGIA STARTOWA" sheetId="3" r:id="Rc674b31e67a74dbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAZA 1 - OSLO V2" sheetId="1" r:id="Rce6f739af7a5444c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TYGODNIE I BRAMKI" sheetId="2" r:id="R0aa656e5b50f4164"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STRATEGIA STARTOWA" sheetId="3" r:id="R0b51aa4b9f9443c7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -163,7 +163,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="42">
+  <x:cellXfs count="44">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -225,7 +225,13 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -476,20 +482,22 @@
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="13" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="13" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="13" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="14" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="70" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="13" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="42" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="13" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="42" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="42" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="42" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="38" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="42" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="38" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="10" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="38" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="55" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="10" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -527,33 +535,39 @@
         <x:v>Intensywność</x:v>
       </x:c>
       <x:c r="L1" s="8" t="str">
-        <x:v>Tempo</x:v>
+        <x:v>Tempo — skrót</x:v>
       </x:c>
       <x:c r="M1" s="8" t="str">
+        <x:v>Tempo i RPE — wszystkie bloki</x:v>
+      </x:c>
+      <x:c r="N1" s="8" t="str">
         <x:v>RPE</x:v>
       </x:c>
-      <x:c r="N1" s="8" t="str">
+      <x:c r="O1" s="8" t="str">
         <x:v>Przewyższenie m</x:v>
       </x:c>
-      <x:c r="O1" s="8" t="str">
+      <x:c r="P1" s="8" t="str">
         <x:v>Część główna</x:v>
       </x:c>
-      <x:c r="P1" s="8" t="str">
+      <x:c r="Q1" s="8" t="str">
         <x:v>Plan B</x:v>
       </x:c>
-      <x:c r="Q1" s="8" t="str">
+      <x:c r="R1" s="8" t="str">
         <x:v>Warunki</x:v>
       </x:c>
-      <x:c r="R1" s="8" t="str">
+      <x:c r="S1" s="8" t="str">
         <x:v>Paliwo</x:v>
       </x:c>
-      <x:c r="S1" s="8" t="str">
+      <x:c r="T1" s="8" t="str">
         <x:v>parentId</x:v>
       </x:c>
-      <x:c r="T1" s="8" t="str">
+      <x:c r="U1" s="8" t="str">
         <x:v>external_id</x:v>
       </x:c>
-      <x:c r="U1" s="9" t="str">
+      <x:c r="V1" s="8" t="str">
+        <x:v>Structured workout</x:v>
+      </x:c>
+      <x:c r="W1" s="9" t="str">
         <x:v>Long</x:v>
       </x:c>
     </x:row>
@@ -586,23 +600,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L2" s="21"/>
-      <x:c r="M2" s="21"/>
-      <x:c r="N2" s="23"/>
-      <x:c r="O2" s="30" t="str"/>
-      <x:c r="P2" s="30" t="str">
+      <x:c r="M2" s="30"/>
+      <x:c r="N2" s="30"/>
+      <x:c r="O2" s="31"/>
+      <x:c r="P2" s="30" t="str"/>
+      <x:c r="Q2" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q2" s="30" t="str"/>
-      <x:c r="R2" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S2" s="21" t="str">
+      <x:c r="R2" s="30" t="str"/>
+      <x:c r="S2" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T2" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-15</x:v>
       </x:c>
-      <x:c r="T2" s="21" t="str">
+      <x:c r="U2" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-15-note-1</x:v>
       </x:c>
-      <x:c r="U2" s="24" t="n">
+      <x:c r="V2" s="30" t="str">
+        <x:v>Pełne wolne</x:v>
+      </x:c>
+      <x:c r="W2" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -636,30 +654,38 @@
       <x:c r="K3" s="21" t="str">
         <x:v>REGENERACJA</x:v>
       </x:c>
-      <x:c r="L3" s="21"/>
-      <x:c r="M3" s="21" t="str">
-        <x:v>2–3</x:v>
-      </x:c>
-      <x:c r="N3" s="23"/>
-      <x:c r="O3" s="30" t="str">
+      <x:c r="L3" s="21" t="str">
+        <x:v>Z2 • RPE 3</x:v>
+      </x:c>
+      <x:c r="M3" s="30" t="str">
+        <x:v>Rower Z2, RPE 3; bez tempa biegowego. Wybierz tylko jedną opcję ALT.</x:v>
+      </x:c>
+      <x:c r="N3" s="30" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O3" s="31"/>
+      <x:c r="P3" s="30" t="str">
         <x:v>40 min spokojnego Z2, kadencja 85–95; bez sweet spotu.</x:v>
       </x:c>
-      <x:c r="P3" s="30" t="str">
+      <x:c r="Q3" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q3" s="30" t="str">
-        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem.</x:v>
-      </x:c>
       <x:c r="R3" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S3" s="21" t="str">
+        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem. Wybierz tylko jedną opcję z grupy alt-2026-07-15.</x:v>
+      </x:c>
+      <x:c r="S3" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T3" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-15</x:v>
       </x:c>
-      <x:c r="T3" s="21" t="str">
+      <x:c r="U3" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-15-ride-alt</x:v>
       </x:c>
-      <x:c r="U3" s="24" t="n">
+      <x:c r="V3" s="30" t="str">
+        <x:v>- Easy spin 40m 55-70% 85-95rpm</x:v>
+      </x:c>
+      <x:c r="W3" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -696,31 +722,42 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L4" s="21" t="str">
-        <x:v>5:50–6:25/km</x:v>
-      </x:c>
-      <x:c r="M4" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+      </x:c>
+      <x:c r="M4" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 5 km easy 5:50–6:25/km, RPE 3–4 + 6 × 20 s rytmu technicznego, RPE 7–8, bez targetu tempa. Przerwy: 90 s pełnego truchtu lub marszu, target otwarty. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Rytmy wykonuj luźno i technicznie; Garmin bez alarmu tempa. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N4" s="30" t="str">
         <x:v>3–4</x:v>
       </x:c>
-      <x:c r="N4" s="23" t="n">
+      <x:c r="O4" s="31" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="O4" s="30" t="str">
+      <x:c r="P4" s="30" t="str">
         <x:v>6 × 20 s rytmu luźno, nie sprint</x:v>
       </x:c>
-      <x:c r="P4" s="30" t="str">
+      <x:c r="Q4" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q4" s="30" t="str"/>
-      <x:c r="R4" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S4" s="21" t="str">
+      <x:c r="R4" s="30" t="str"/>
+      <x:c r="S4" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T4" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-16</x:v>
       </x:c>
-      <x:c r="T4" s="21" t="str">
+      <x:c r="U4" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-16-run-1</x:v>
       </x:c>
-      <x:c r="U4" s="24" t="n">
+      <x:c r="V4" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Easy 5km 5:50/km-6:25/km Pace
+Strides 6x
+- Fast relaxed 20s 7-8 RPE
+- Full recovery 90s open
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W4" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -755,29 +792,33 @@
         <x:v>LEKKA</x:v>
       </x:c>
       <x:c r="L5" s="21"/>
-      <x:c r="M5" s="21" t="str">
+      <x:c r="M5" s="30"/>
+      <x:c r="N5" s="30" t="str">
         <x:v>2–4</x:v>
       </x:c>
-      <x:c r="N5" s="23"/>
-      <x:c r="O5" s="30" t="str">
+      <x:c r="O5" s="31"/>
+      <x:c r="P5" s="30" t="str">
         <x:v>Technika: split squat do ławki, wspięcia łydki, hip hinge bez ciężaru, side plank; 1–2 serie, zostaw 4–5 powtórzeń w zapasie.</x:v>
       </x:c>
-      <x:c r="P5" s="30" t="str">
+      <x:c r="Q5" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q5" s="30" t="str">
+      <x:c r="R5" s="30" t="str">
         <x:v>Bez DOMS i bez pracy do upadku. Przerwij przy bólu &gt;2/10.</x:v>
       </x:c>
-      <x:c r="R5" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S5" s="21" t="str">
+      <x:c r="S5" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T5" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-16</x:v>
       </x:c>
-      <x:c r="T5" s="21" t="str">
+      <x:c r="U5" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-16-strength-1</x:v>
       </x:c>
-      <x:c r="U5" s="24" t="n">
+      <x:c r="V5" s="30" t="str">
+        <x:v>- Technika i stabilizacja 12m 2-4 RPE</x:v>
+      </x:c>
+      <x:c r="W5" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -810,23 +851,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L6" s="21"/>
-      <x:c r="M6" s="21"/>
-      <x:c r="N6" s="23"/>
-      <x:c r="O6" s="30" t="str"/>
-      <x:c r="P6" s="30" t="str">
+      <x:c r="M6" s="30"/>
+      <x:c r="N6" s="30"/>
+      <x:c r="O6" s="31"/>
+      <x:c r="P6" s="30" t="str"/>
+      <x:c r="Q6" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q6" s="30" t="str"/>
-      <x:c r="R6" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S6" s="21" t="str">
+      <x:c r="R6" s="30" t="str"/>
+      <x:c r="S6" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T6" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-17</x:v>
       </x:c>
-      <x:c r="T6" s="21" t="str">
+      <x:c r="U6" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-17-note-1</x:v>
       </x:c>
-      <x:c r="U6" s="24" t="n">
+      <x:c r="V6" s="30" t="str">
+        <x:v>WOLNE przed long runem</x:v>
+      </x:c>
+      <x:c r="W6" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -863,33 +908,41 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L7" s="21" t="str">
-        <x:v>5:55–6:25/km</x:v>
-      </x:c>
-      <x:c r="M7" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M7" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 10 km easy 5:50–6:25/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N7" s="30" t="str">
         <x:v>3–4</x:v>
       </x:c>
-      <x:c r="N7" s="23" t="n">
+      <x:c r="O7" s="31" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="O7" s="30" t="str">
+      <x:c r="P7" s="30" t="str">
         <x:v>12 km easy na łagodnie pofałdowanej trasie; bez MP.</x:v>
       </x:c>
-      <x:c r="P7" s="30" t="str">
+      <x:c r="Q7" s="30" t="str">
         <x:v>8–10 km easy albo przerwanie przy narastającym bólu; nie nadrabiaj.</x:v>
       </x:c>
-      <x:c r="Q7" s="30" t="str">
+      <x:c r="R7" s="30" t="str">
         <x:v>Ból 0–2/10 i brak zmiany kroku. W innym przypadku 8–10 km easy.</x:v>
       </x:c>
-      <x:c r="R7" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S7" s="21" t="str">
+      <x:c r="S7" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T7" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-18</x:v>
       </x:c>
-      <x:c r="T7" s="21" t="str">
+      <x:c r="U7" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-18-run-1</x:v>
       </x:c>
-      <x:c r="U7" s="24" t="n">
+      <x:c r="V7" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Long easy 10km 5:50/km-6:25/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W7" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -926,31 +979,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L8" s="21" t="str">
-        <x:v>6:15–6:45/km</x:v>
-      </x:c>
-      <x:c r="M8" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M8" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N8" s="30" t="str">
         <x:v>2–3</x:v>
       </x:c>
-      <x:c r="N8" s="23" t="n">
+      <x:c r="O8" s="31" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="O8" s="30" t="str">
+      <x:c r="P8" s="30" t="str">
         <x:v>5 km bardzo lekko.</x:v>
       </x:c>
-      <x:c r="P8" s="30" t="str">
+      <x:c r="Q8" s="30" t="str">
         <x:v>Pełne wolne, jeśli po longu jest ból albo sztywność.</x:v>
       </x:c>
-      <x:c r="Q8" s="30" t="str"/>
-      <x:c r="R8" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S8" s="21" t="str">
+      <x:c r="R8" s="30" t="str"/>
+      <x:c r="S8" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T8" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-19</x:v>
       </x:c>
-      <x:c r="T8" s="21" t="str">
+      <x:c r="U8" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-19-run-1</x:v>
       </x:c>
-      <x:c r="U8" s="24" t="n">
+      <x:c r="V8" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Recovery 3km 6:15/km-6:45/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W8" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -983,23 +1044,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L9" s="21"/>
-      <x:c r="M9" s="21"/>
-      <x:c r="N9" s="23"/>
-      <x:c r="O9" s="30" t="str"/>
-      <x:c r="P9" s="30" t="str">
+      <x:c r="M9" s="30"/>
+      <x:c r="N9" s="30"/>
+      <x:c r="O9" s="31"/>
+      <x:c r="P9" s="30" t="str"/>
+      <x:c r="Q9" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q9" s="30" t="str"/>
-      <x:c r="R9" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S9" s="21" t="str">
+      <x:c r="R9" s="30" t="str"/>
+      <x:c r="S9" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T9" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-20</x:v>
       </x:c>
-      <x:c r="T9" s="21" t="str">
+      <x:c r="U9" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-20-note-1</x:v>
       </x:c>
-      <x:c r="U9" s="24" t="n">
+      <x:c r="V9" s="30" t="str">
+        <x:v>Regeneracja</x:v>
+      </x:c>
+      <x:c r="W9" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1034,29 +1099,33 @@
         <x:v>LEKKA</x:v>
       </x:c>
       <x:c r="L10" s="21"/>
-      <x:c r="M10" s="21" t="str">
+      <x:c r="M10" s="30"/>
+      <x:c r="N10" s="30" t="str">
         <x:v>2–4</x:v>
       </x:c>
-      <x:c r="N10" s="23"/>
-      <x:c r="O10" s="30" t="str">
+      <x:c r="O10" s="31"/>
+      <x:c r="P10" s="30" t="str">
         <x:v>Technika: split squat do ławki, wspięcia łydki, hip hinge bez ciężaru, side plank; 1–2 serie, zostaw 4–5 powtórzeń w zapasie.</x:v>
       </x:c>
-      <x:c r="P10" s="30" t="str">
+      <x:c r="Q10" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q10" s="30" t="str">
+      <x:c r="R10" s="30" t="str">
         <x:v>Bez DOMS i bez pracy do upadku. Przerwij przy bólu &gt;2/10.</x:v>
       </x:c>
-      <x:c r="R10" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S10" s="21" t="str">
+      <x:c r="S10" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T10" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-20</x:v>
       </x:c>
-      <x:c r="T10" s="21" t="str">
+      <x:c r="U10" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-20-strength-1</x:v>
       </x:c>
-      <x:c r="U10" s="24" t="n">
+      <x:c r="V10" s="30" t="str">
+        <x:v>- Technika i stabilizacja 15m 2-4 RPE</x:v>
+      </x:c>
+      <x:c r="W10" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1093,31 +1162,41 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L11" s="21" t="str">
-        <x:v>odcinki 4:58–5:05/km</x:v>
-      </x:c>
-      <x:c r="M11" s="21" t="str">
-        <x:v>6–7</x:v>
-      </x:c>
-      <x:c r="N11" s="23" t="n">
+        <x:v>6:00–6:30/km albo wolniej • 4:58–5:05/km • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M11" s="30" t="str">
+        <x:v>Rozgrzewka: 2 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 3 × 1 km 4:58–5:05/km, RPE 7, na płaskim. Przerwy: 2 min truchtu 6:15–6:45/km, RPE 2–3. Schłodzenie: 2 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N11" s="30" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="O11" s="31" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="O11" s="30" t="str">
+      <x:c r="P11" s="30" t="str">
         <x:v>3 × 1 km w tempie progowym</x:v>
       </x:c>
-      <x:c r="P11" s="30" t="str">
+      <x:c r="Q11" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q11" s="30" t="str"/>
-      <x:c r="R11" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S11" s="21" t="str">
+      <x:c r="R11" s="30" t="str"/>
+      <x:c r="S11" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T11" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-21</x:v>
       </x:c>
-      <x:c r="T11" s="21" t="str">
+      <x:c r="U11" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-21-run-1</x:v>
       </x:c>
-      <x:c r="U11" s="24" t="n">
+      <x:c r="V11" s="30" t="str">
+        <x:v>- Warmup 2km 6:00/km-6:30/km Pace
+Threshold 3x
+- Threshold 1km 4:58/km-5:05/km Pace
+- Recovery 2m 6:15/km-6:45/km Pace
+- Cooldown 2km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W11" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1150,23 +1229,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L12" s="21"/>
-      <x:c r="M12" s="21"/>
-      <x:c r="N12" s="23"/>
-      <x:c r="O12" s="30" t="str"/>
-      <x:c r="P12" s="30" t="str">
+      <x:c r="M12" s="30"/>
+      <x:c r="N12" s="30"/>
+      <x:c r="O12" s="31"/>
+      <x:c r="P12" s="30" t="str"/>
+      <x:c r="Q12" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q12" s="30" t="str"/>
-      <x:c r="R12" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S12" s="21" t="str">
+      <x:c r="R12" s="30" t="str"/>
+      <x:c r="S12" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T12" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-22</x:v>
       </x:c>
-      <x:c r="T12" s="21" t="str">
+      <x:c r="U12" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-22-note-1</x:v>
       </x:c>
-      <x:c r="U12" s="24" t="n">
+      <x:c r="V12" s="30" t="str">
+        <x:v>Pełne wolne</x:v>
+      </x:c>
+      <x:c r="W12" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1200,30 +1283,38 @@
       <x:c r="K13" s="21" t="str">
         <x:v>REGENERACJA</x:v>
       </x:c>
-      <x:c r="L13" s="21"/>
-      <x:c r="M13" s="21" t="str">
-        <x:v>2–3</x:v>
-      </x:c>
-      <x:c r="N13" s="23"/>
-      <x:c r="O13" s="30" t="str">
+      <x:c r="L13" s="21" t="str">
+        <x:v>Z2 • RPE 3</x:v>
+      </x:c>
+      <x:c r="M13" s="30" t="str">
+        <x:v>Rower Z2, RPE 3; bez tempa biegowego. Wybierz tylko jedną opcję ALT.</x:v>
+      </x:c>
+      <x:c r="N13" s="30" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O13" s="31"/>
+      <x:c r="P13" s="30" t="str">
         <x:v>45 min spokojnego Z2, kadencja 85–95; bez sweet spotu.</x:v>
       </x:c>
-      <x:c r="P13" s="30" t="str">
+      <x:c r="Q13" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q13" s="30" t="str">
-        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem.</x:v>
-      </x:c>
       <x:c r="R13" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S13" s="21" t="str">
+        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem. Wybierz tylko jedną opcję z grupy alt-2026-07-22.</x:v>
+      </x:c>
+      <x:c r="S13" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T13" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-22</x:v>
       </x:c>
-      <x:c r="T13" s="21" t="str">
+      <x:c r="U13" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-22-ride-alt</x:v>
       </x:c>
-      <x:c r="U13" s="24" t="n">
+      <x:c r="V13" s="30" t="str">
+        <x:v>- Easy spin 45m 55-70% 85-95rpm</x:v>
+      </x:c>
+      <x:c r="W13" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1260,33 +1351,44 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L14" s="21" t="str">
-        <x:v>5:50–6:20/km</x:v>
-      </x:c>
-      <x:c r="M14" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:45–6:15/km • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+      </x:c>
+      <x:c r="M14" s="30" t="str">
+        <x:v>Rozgrzewka: 2 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 7 km średnio-długiego easy 5:45–6:15/km, RPE 3–4 + 6 × 8 s hill sprint techniczny, nachylenie 4–6%, RPE 8, bez targetu tempa. Przerwy: 2 min pełnego marszu/truchtu w dół, target otwarty. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Podbieg wykonywany na wysiłek — nie kontroluj tempa chwilowego. Garmin bez alarmu tempa na hill sprintach.</x:v>
+      </x:c>
+      <x:c r="N14" s="30" t="str">
         <x:v>3–4</x:v>
       </x:c>
-      <x:c r="N14" s="23" t="n">
+      <x:c r="O14" s="31" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O14" s="30" t="str">
+      <x:c r="P14" s="30" t="str">
         <x:v>6 × 8 s sprężystego podbiegu, nie maksymalnie</x:v>
       </x:c>
-      <x:c r="P14" s="30" t="str">
+      <x:c r="Q14" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q14" s="30" t="str">
+      <x:c r="R14" s="30" t="str">
         <x:v>Hill sprints są dodatkiem nerwowo-mięśniowym; pełna regeneracja, bez celu tempa na stromym podbiegu.</x:v>
       </x:c>
-      <x:c r="R14" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S14" s="21" t="str">
+      <x:c r="S14" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T14" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-23</x:v>
       </x:c>
-      <x:c r="T14" s="21" t="str">
+      <x:c r="U14" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-23-run-1</x:v>
       </x:c>
-      <x:c r="U14" s="24" t="n">
+      <x:c r="V14" s="30" t="str">
+        <x:v>- Warmup 2km 6:00/km-6:30/km Pace
+- Medium long easy 7km 5:45/km-6:15/km Pace
+Hill sprints 6x
+- Uphill fast relaxed 8s 8 RPE
+- Full walk-jog recovery 2m open
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W14" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1319,23 +1421,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L15" s="21"/>
-      <x:c r="M15" s="21"/>
-      <x:c r="N15" s="23"/>
-      <x:c r="O15" s="30" t="str"/>
-      <x:c r="P15" s="30" t="str">
+      <x:c r="M15" s="30"/>
+      <x:c r="N15" s="30"/>
+      <x:c r="O15" s="31"/>
+      <x:c r="P15" s="30" t="str"/>
+      <x:c r="Q15" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q15" s="30" t="str"/>
-      <x:c r="R15" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S15" s="21" t="str">
+      <x:c r="R15" s="30" t="str"/>
+      <x:c r="S15" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T15" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-24</x:v>
       </x:c>
-      <x:c r="T15" s="21" t="str">
+      <x:c r="U15" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-24-note-1</x:v>
       </x:c>
-      <x:c r="U15" s="24" t="n">
+      <x:c r="V15" s="30" t="str">
+        <x:v>WOLNE przed long runem</x:v>
+      </x:c>
+      <x:c r="W15" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1372,31 +1478,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L16" s="21" t="str">
-        <x:v>5:55–6:25/km</x:v>
-      </x:c>
-      <x:c r="M16" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M16" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 10 km easy 5:50–6:25/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N16" s="30" t="str">
         <x:v>3–4</x:v>
       </x:c>
-      <x:c r="N16" s="23" t="n">
+      <x:c r="O16" s="31" t="n">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="O16" s="30" t="str">
+      <x:c r="P16" s="30" t="str">
         <x:v>12 km easy na pofałdowanej trasie, równy wysiłek.</x:v>
       </x:c>
-      <x:c r="P16" s="30" t="str">
+      <x:c r="Q16" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q16" s="30" t="str"/>
-      <x:c r="R16" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S16" s="21" t="str">
+      <x:c r="R16" s="30" t="str"/>
+      <x:c r="S16" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T16" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-25</x:v>
       </x:c>
-      <x:c r="T16" s="21" t="str">
+      <x:c r="U16" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-25-run-1</x:v>
       </x:c>
-      <x:c r="U16" s="24" t="n">
+      <x:c r="V16" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Long easy 10km 5:50/km-6:25/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W16" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -1433,31 +1547,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L17" s="21" t="str">
-        <x:v>6:15–6:45/km</x:v>
-      </x:c>
-      <x:c r="M17" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M17" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N17" s="30" t="str">
         <x:v>2–3</x:v>
       </x:c>
-      <x:c r="N17" s="23" t="n">
+      <x:c r="O17" s="31" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="O17" s="30" t="str">
+      <x:c r="P17" s="30" t="str">
         <x:v>5 km bardzo lekko.</x:v>
       </x:c>
-      <x:c r="P17" s="30" t="str">
+      <x:c r="Q17" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q17" s="30" t="str"/>
-      <x:c r="R17" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S17" s="21" t="str">
+      <x:c r="R17" s="30" t="str"/>
+      <x:c r="S17" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T17" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-26</x:v>
       </x:c>
-      <x:c r="T17" s="21" t="str">
+      <x:c r="U17" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-26-run-1</x:v>
       </x:c>
-      <x:c r="U17" s="24" t="n">
+      <x:c r="V17" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Recovery 3km 6:15/km-6:45/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W17" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1490,23 +1612,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L18" s="21"/>
-      <x:c r="M18" s="21"/>
-      <x:c r="N18" s="23"/>
-      <x:c r="O18" s="30" t="str"/>
-      <x:c r="P18" s="30" t="str">
+      <x:c r="M18" s="30"/>
+      <x:c r="N18" s="30"/>
+      <x:c r="O18" s="31"/>
+      <x:c r="P18" s="30" t="str"/>
+      <x:c r="Q18" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q18" s="30" t="str"/>
-      <x:c r="R18" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S18" s="21" t="str">
+      <x:c r="R18" s="30" t="str"/>
+      <x:c r="S18" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T18" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-27</x:v>
       </x:c>
-      <x:c r="T18" s="21" t="str">
+      <x:c r="U18" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-27-note-1</x:v>
       </x:c>
-      <x:c r="U18" s="24" t="n">
+      <x:c r="V18" s="30" t="str">
+        <x:v>Regeneracja</x:v>
+      </x:c>
+      <x:c r="W18" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1541,29 +1667,33 @@
         <x:v>LEKKA</x:v>
       </x:c>
       <x:c r="L19" s="21"/>
-      <x:c r="M19" s="21" t="str">
+      <x:c r="M19" s="30"/>
+      <x:c r="N19" s="30" t="str">
         <x:v>2–4</x:v>
       </x:c>
-      <x:c r="N19" s="23"/>
-      <x:c r="O19" s="30" t="str">
+      <x:c r="O19" s="31"/>
+      <x:c r="P19" s="30" t="str">
         <x:v>Technika: split squat do ławki, wspięcia łydki, hip hinge bez ciężaru, side plank; 1–2 serie, zostaw 4–5 powtórzeń w zapasie.</x:v>
       </x:c>
-      <x:c r="P19" s="30" t="str">
+      <x:c r="Q19" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q19" s="30" t="str">
+      <x:c r="R19" s="30" t="str">
         <x:v>Bez DOMS i bez pracy do upadku. Przerwij przy bólu &gt;2/10.</x:v>
       </x:c>
-      <x:c r="R19" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S19" s="21" t="str">
+      <x:c r="S19" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T19" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-27</x:v>
       </x:c>
-      <x:c r="T19" s="21" t="str">
+      <x:c r="U19" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-27-strength-1</x:v>
       </x:c>
-      <x:c r="U19" s="24" t="n">
+      <x:c r="V19" s="30" t="str">
+        <x:v>- Technika i stabilizacja 18m 2-4 RPE</x:v>
+      </x:c>
+      <x:c r="W19" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1600,33 +1730,43 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L20" s="21" t="str">
-        <x:v>easy 5:55–6:25/km; podbieg wg RPE</x:v>
-      </x:c>
-      <x:c r="M20" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+      </x:c>
+      <x:c r="M20" s="30" t="str">
+        <x:v>Rozgrzewka: 2.5 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 6 × 60 s pod górę, nachylenie 4–7%, RPE 7; bez targetu tempa. Przerwy: pełny trucht w dół 2.5 min, target otwarty, RPE 2–3. Schłodzenie: 2 km 6:10–6:40/km, RPE 2–3. Podbieg wykonywany na wysiłek — nie kontroluj tempa chwilowego.</x:v>
+      </x:c>
+      <x:c r="N20" s="30" t="str">
         <x:v>7 na podbiegach</x:v>
       </x:c>
-      <x:c r="N20" s="23" t="n">
+      <x:c r="O20" s="31" t="n">
         <x:v>180</x:v>
       </x:c>
-      <x:c r="O20" s="30" t="str">
+      <x:c r="P20" s="30" t="str">
         <x:v>6 × 60 s pod górę w kontrolowanym mocnym wysiłku</x:v>
       </x:c>
-      <x:c r="P20" s="30" t="str">
+      <x:c r="Q20" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q20" s="30" t="str">
+      <x:c r="R20" s="30" t="str">
         <x:v>Bez celu tempa na podbiegu; technika i równy wysiłek.</x:v>
       </x:c>
-      <x:c r="R20" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S20" s="21" t="str">
+      <x:c r="S20" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T20" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-28</x:v>
       </x:c>
-      <x:c r="T20" s="21" t="str">
+      <x:c r="U20" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-28-run-1</x:v>
       </x:c>
-      <x:c r="U20" s="24" t="n">
+      <x:c r="V20" s="30" t="str">
+        <x:v>- Warmup 2.5km 6:00/km-6:30/km Pace
+Uphill effort 6x
+- Uphill 60s 7 RPE
+- Full jog-down recovery 150s open
+- Cooldown 2km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W20" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1659,23 +1799,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L21" s="21"/>
-      <x:c r="M21" s="21"/>
-      <x:c r="N21" s="23"/>
-      <x:c r="O21" s="30" t="str"/>
-      <x:c r="P21" s="30" t="str">
+      <x:c r="M21" s="30"/>
+      <x:c r="N21" s="30"/>
+      <x:c r="O21" s="31"/>
+      <x:c r="P21" s="30" t="str"/>
+      <x:c r="Q21" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q21" s="30" t="str"/>
-      <x:c r="R21" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S21" s="21" t="str">
+      <x:c r="R21" s="30" t="str"/>
+      <x:c r="S21" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T21" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-29</x:v>
       </x:c>
-      <x:c r="T21" s="21" t="str">
+      <x:c r="U21" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-29-note-1</x:v>
       </x:c>
-      <x:c r="U21" s="24" t="n">
+      <x:c r="V21" s="30" t="str">
+        <x:v>Pełne wolne</x:v>
+      </x:c>
+      <x:c r="W21" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1709,30 +1853,38 @@
       <x:c r="K22" s="21" t="str">
         <x:v>REGENERACJA</x:v>
       </x:c>
-      <x:c r="L22" s="21"/>
-      <x:c r="M22" s="21" t="str">
-        <x:v>2–3</x:v>
-      </x:c>
-      <x:c r="N22" s="23"/>
-      <x:c r="O22" s="30" t="str">
+      <x:c r="L22" s="21" t="str">
+        <x:v>Z2 • RPE 3</x:v>
+      </x:c>
+      <x:c r="M22" s="30" t="str">
+        <x:v>Rower Z2, RPE 3; bez tempa biegowego. Wybierz tylko jedną opcję ALT.</x:v>
+      </x:c>
+      <x:c r="N22" s="30" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O22" s="31"/>
+      <x:c r="P22" s="30" t="str">
         <x:v>45 min spokojnego Z2, kadencja 85–95; bez sweet spotu.</x:v>
       </x:c>
-      <x:c r="P22" s="30" t="str">
+      <x:c r="Q22" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q22" s="30" t="str">
-        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem.</x:v>
-      </x:c>
       <x:c r="R22" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S22" s="21" t="str">
+        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem. Wybierz tylko jedną opcję z grupy alt-2026-07-29.</x:v>
+      </x:c>
+      <x:c r="S22" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T22" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-29</x:v>
       </x:c>
-      <x:c r="T22" s="21" t="str">
+      <x:c r="U22" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-29-ride-alt</x:v>
       </x:c>
-      <x:c r="U22" s="24" t="n">
+      <x:c r="V22" s="30" t="str">
+        <x:v>- Easy spin 45m 55-70% 85-95rpm</x:v>
+      </x:c>
+      <x:c r="W22" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1769,31 +1921,40 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L23" s="21" t="str">
-        <x:v>8 km 5:50–6:15/km + 3 km 5:20–5:35/km</x:v>
-      </x:c>
-      <x:c r="M23" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:45–6:15/km • 5:20–5:35/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M23" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 6 km średnio-długiego easy 5:45–6:15/km, RPE 3–4 + 3 km steady 5:20–5:35/km, RPE 5–6. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N23" s="30" t="str">
         <x:v>3–5</x:v>
       </x:c>
-      <x:c r="N23" s="23" t="n">
+      <x:c r="O23" s="31" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O23" s="30" t="str">
+      <x:c r="P23" s="30" t="str">
         <x:v>Ostatnie 3 km steady, bez wejścia na próg</x:v>
       </x:c>
-      <x:c r="P23" s="30" t="str">
+      <x:c r="Q23" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q23" s="30" t="str"/>
-      <x:c r="R23" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S23" s="21" t="str">
+      <x:c r="R23" s="30" t="str"/>
+      <x:c r="S23" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T23" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-30</x:v>
       </x:c>
-      <x:c r="T23" s="21" t="str">
+      <x:c r="U23" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-30-run-1</x:v>
       </x:c>
-      <x:c r="U23" s="24" t="n">
+      <x:c r="V23" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Medium long easy 6km 5:45/km-6:15/km Pace
+- Steady 3km 5:20/km-5:35/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W23" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1826,23 +1987,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L24" s="21"/>
-      <x:c r="M24" s="21"/>
-      <x:c r="N24" s="23"/>
-      <x:c r="O24" s="30" t="str"/>
-      <x:c r="P24" s="30" t="str">
+      <x:c r="M24" s="30"/>
+      <x:c r="N24" s="30"/>
+      <x:c r="O24" s="31"/>
+      <x:c r="P24" s="30" t="str"/>
+      <x:c r="Q24" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q24" s="30" t="str"/>
-      <x:c r="R24" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S24" s="21" t="str">
+      <x:c r="R24" s="30" t="str"/>
+      <x:c r="S24" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T24" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-31</x:v>
       </x:c>
-      <x:c r="T24" s="21" t="str">
+      <x:c r="U24" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-07-31-note-1</x:v>
       </x:c>
-      <x:c r="U24" s="24" t="n">
+      <x:c r="V24" s="30" t="str">
+        <x:v>WOLNE przed long runem</x:v>
+      </x:c>
+      <x:c r="W24" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1879,33 +2044,41 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L25" s="21" t="str">
-        <x:v>5:55–6:30/km wg terenu</x:v>
-      </x:c>
-      <x:c r="M25" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M25" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 12 km easy 5:50–6:25/km na płaskich fragmentach; na podbiegach według wysiłku, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N25" s="30" t="str">
         <x:v>3–5</x:v>
       </x:c>
-      <x:c r="N25" s="23" t="n">
+      <x:c r="O25" s="31" t="n">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="O25" s="30" t="str">
+      <x:c r="P25" s="30" t="str">
         <x:v>14 km po pofałdowanej trasie, wysiłek easy; bez MP.</x:v>
       </x:c>
-      <x:c r="P25" s="30" t="str">
+      <x:c r="Q25" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q25" s="30" t="str">
+      <x:c r="R25" s="30" t="str">
         <x:v>Kontroluj wysiłek na podbiegach; tempo może spadać.</x:v>
       </x:c>
-      <x:c r="R25" s="30" t="str">
+      <x:c r="S25" s="30" t="str">
         <x:v>Śniadanie 2–3 h przed. 40–60 g węgli/h, płyny i sód według pogody; nic nowego.</x:v>
       </x:c>
-      <x:c r="S25" s="21" t="str">
+      <x:c r="T25" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-01</x:v>
       </x:c>
-      <x:c r="T25" s="21" t="str">
+      <x:c r="U25" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-01-run-1</x:v>
       </x:c>
-      <x:c r="U25" s="24" t="n">
+      <x:c r="V25" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Long easy 12km 5:50/km-6:25/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W25" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -1942,31 +2115,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L26" s="21" t="str">
-        <x:v>6:15–6:45/km</x:v>
-      </x:c>
-      <x:c r="M26" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M26" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N26" s="30" t="str">
         <x:v>2–3</x:v>
       </x:c>
-      <x:c r="N26" s="23" t="n">
+      <x:c r="O26" s="31" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="O26" s="30" t="str">
+      <x:c r="P26" s="30" t="str">
         <x:v>5 km bardzo lekko.</x:v>
       </x:c>
-      <x:c r="P26" s="30" t="str">
+      <x:c r="Q26" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q26" s="30" t="str"/>
-      <x:c r="R26" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S26" s="21" t="str">
+      <x:c r="R26" s="30" t="str"/>
+      <x:c r="S26" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T26" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-02</x:v>
       </x:c>
-      <x:c r="T26" s="21" t="str">
+      <x:c r="U26" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-02-run-1</x:v>
       </x:c>
-      <x:c r="U26" s="24" t="n">
+      <x:c r="V26" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Recovery 3km 6:15/km-6:45/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W26" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1999,23 +2180,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L27" s="21"/>
-      <x:c r="M27" s="21"/>
-      <x:c r="N27" s="23"/>
-      <x:c r="O27" s="30" t="str"/>
-      <x:c r="P27" s="30" t="str">
+      <x:c r="M27" s="30"/>
+      <x:c r="N27" s="30"/>
+      <x:c r="O27" s="31"/>
+      <x:c r="P27" s="30" t="str"/>
+      <x:c r="Q27" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q27" s="30" t="str"/>
-      <x:c r="R27" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S27" s="21" t="str">
+      <x:c r="R27" s="30" t="str"/>
+      <x:c r="S27" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T27" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-03</x:v>
       </x:c>
-      <x:c r="T27" s="21" t="str">
+      <x:c r="U27" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-03-note-1</x:v>
       </x:c>
-      <x:c r="U27" s="24" t="n">
+      <x:c r="V27" s="30" t="str">
+        <x:v>Regeneracja</x:v>
+      </x:c>
+      <x:c r="W27" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2050,29 +2235,33 @@
         <x:v>LEKKA</x:v>
       </x:c>
       <x:c r="L28" s="21"/>
-      <x:c r="M28" s="21" t="str">
+      <x:c r="M28" s="30"/>
+      <x:c r="N28" s="30" t="str">
         <x:v>2–4</x:v>
       </x:c>
-      <x:c r="N28" s="23"/>
-      <x:c r="O28" s="30" t="str">
+      <x:c r="O28" s="31"/>
+      <x:c r="P28" s="30" t="str">
         <x:v>Technika: split squat do ławki, wspięcia łydki, hip hinge bez ciężaru, side plank; 1–2 serie, zostaw 4–5 powtórzeń w zapasie.</x:v>
       </x:c>
-      <x:c r="P28" s="30" t="str">
+      <x:c r="Q28" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q28" s="30" t="str">
+      <x:c r="R28" s="30" t="str">
         <x:v>Bez DOMS i bez pracy do upadku. Przerwij przy bólu &gt;2/10.</x:v>
       </x:c>
-      <x:c r="R28" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S28" s="21" t="str">
+      <x:c r="S28" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T28" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-03</x:v>
       </x:c>
-      <x:c r="T28" s="21" t="str">
+      <x:c r="U28" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-03-strength-1</x:v>
       </x:c>
-      <x:c r="U28" s="24" t="n">
+      <x:c r="V28" s="30" t="str">
+        <x:v>- Technika i stabilizacja 20m 2-4 RPE</x:v>
+      </x:c>
+      <x:c r="W28" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2109,31 +2298,41 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L29" s="21" t="str">
-        <x:v>odcinki 4:58–5:05/km</x:v>
-      </x:c>
-      <x:c r="M29" s="21" t="str">
-        <x:v>6–7</x:v>
-      </x:c>
-      <x:c r="N29" s="23" t="n">
+        <x:v>6:00–6:30/km albo wolniej • 4:58–5:05/km • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M29" s="30" t="str">
+        <x:v>Rozgrzewka: 2 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 4 × 1 km 4:58–5:05/km, RPE 7, na płaskim. Przerwy: 2 min truchtu 6:15–6:45/km, RPE 2–3. Schłodzenie: 2 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N29" s="30" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="O29" s="31" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="O29" s="30" t="str">
+      <x:c r="P29" s="30" t="str">
         <x:v>4 × 1 km progowo</x:v>
       </x:c>
-      <x:c r="P29" s="30" t="str">
+      <x:c r="Q29" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q29" s="30" t="str"/>
-      <x:c r="R29" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S29" s="21" t="str">
+      <x:c r="R29" s="30" t="str"/>
+      <x:c r="S29" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T29" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-04</x:v>
       </x:c>
-      <x:c r="T29" s="21" t="str">
+      <x:c r="U29" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-04-run-1</x:v>
       </x:c>
-      <x:c r="U29" s="24" t="n">
+      <x:c r="V29" s="30" t="str">
+        <x:v>- Warmup 2km 6:00/km-6:30/km Pace
+Threshold 4x
+- Threshold 1km 4:58/km-5:05/km Pace
+- Recovery 2m 6:15/km-6:45/km Pace
+- Cooldown 2km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W29" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2166,23 +2365,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L30" s="21"/>
-      <x:c r="M30" s="21"/>
-      <x:c r="N30" s="23"/>
-      <x:c r="O30" s="30" t="str"/>
-      <x:c r="P30" s="30" t="str">
+      <x:c r="M30" s="30"/>
+      <x:c r="N30" s="30"/>
+      <x:c r="O30" s="31"/>
+      <x:c r="P30" s="30" t="str"/>
+      <x:c r="Q30" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q30" s="30" t="str"/>
-      <x:c r="R30" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S30" s="21" t="str">
+      <x:c r="R30" s="30" t="str"/>
+      <x:c r="S30" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T30" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-05</x:v>
       </x:c>
-      <x:c r="T30" s="21" t="str">
+      <x:c r="U30" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-05-note-1</x:v>
       </x:c>
-      <x:c r="U30" s="24" t="n">
+      <x:c r="V30" s="30" t="str">
+        <x:v>Pełne wolne</x:v>
+      </x:c>
+      <x:c r="W30" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2216,30 +2419,38 @@
       <x:c r="K31" s="21" t="str">
         <x:v>REGENERACJA</x:v>
       </x:c>
-      <x:c r="L31" s="21"/>
-      <x:c r="M31" s="21" t="str">
-        <x:v>2–3</x:v>
-      </x:c>
-      <x:c r="N31" s="23"/>
-      <x:c r="O31" s="30" t="str">
+      <x:c r="L31" s="21" t="str">
+        <x:v>Z2 • RPE 3</x:v>
+      </x:c>
+      <x:c r="M31" s="30" t="str">
+        <x:v>Rower Z2, RPE 3; bez tempa biegowego. Wybierz tylko jedną opcję ALT.</x:v>
+      </x:c>
+      <x:c r="N31" s="30" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O31" s="31"/>
+      <x:c r="P31" s="30" t="str">
         <x:v>40 min spokojnego Z2, kadencja 85–95; bez sweet spotu.</x:v>
       </x:c>
-      <x:c r="P31" s="30" t="str">
+      <x:c r="Q31" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q31" s="30" t="str">
-        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem.</x:v>
-      </x:c>
       <x:c r="R31" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S31" s="21" t="str">
+        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem. Wybierz tylko jedną opcję z grupy alt-2026-08-05.</x:v>
+      </x:c>
+      <x:c r="S31" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T31" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-05</x:v>
       </x:c>
-      <x:c r="T31" s="21" t="str">
+      <x:c r="U31" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-05-ride-alt</x:v>
       </x:c>
-      <x:c r="U31" s="24" t="n">
+      <x:c r="V31" s="30" t="str">
+        <x:v>- Easy spin 40m 55-70% 85-95rpm</x:v>
+      </x:c>
+      <x:c r="W31" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2276,31 +2487,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L32" s="21" t="str">
-        <x:v>5:50–6:20/km</x:v>
-      </x:c>
-      <x:c r="M32" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:45–6:15/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M32" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Średnio-długi easy: 8 km 5:45–6:15/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N32" s="30" t="str">
         <x:v>3–4</x:v>
       </x:c>
-      <x:c r="N32" s="23" t="n">
+      <x:c r="O32" s="31" t="n">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="O32" s="30" t="str">
+      <x:c r="P32" s="30" t="str">
         <x:v>10 km spokojnie.</x:v>
       </x:c>
-      <x:c r="P32" s="30" t="str">
+      <x:c r="Q32" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q32" s="30" t="str"/>
-      <x:c r="R32" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S32" s="21" t="str">
+      <x:c r="R32" s="30" t="str"/>
+      <x:c r="S32" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T32" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-06</x:v>
       </x:c>
-      <x:c r="T32" s="21" t="str">
+      <x:c r="U32" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-06-run-1</x:v>
       </x:c>
-      <x:c r="U32" s="24" t="n">
+      <x:c r="V32" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Średnio-długi easy 8km 5:45/km-6:15/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W32" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2333,23 +2552,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L33" s="21"/>
-      <x:c r="M33" s="21"/>
-      <x:c r="N33" s="23"/>
-      <x:c r="O33" s="30" t="str"/>
-      <x:c r="P33" s="30" t="str">
+      <x:c r="M33" s="30"/>
+      <x:c r="N33" s="30"/>
+      <x:c r="O33" s="31"/>
+      <x:c r="P33" s="30" t="str"/>
+      <x:c r="Q33" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q33" s="30" t="str"/>
-      <x:c r="R33" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S33" s="21" t="str">
+      <x:c r="R33" s="30" t="str"/>
+      <x:c r="S33" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T33" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-07</x:v>
       </x:c>
-      <x:c r="T33" s="21" t="str">
+      <x:c r="U33" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-07-note-1</x:v>
       </x:c>
-      <x:c r="U33" s="24" t="n">
+      <x:c r="V33" s="30" t="str">
+        <x:v>WOLNE przed long runem</x:v>
+      </x:c>
+      <x:c r="W33" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2386,31 +2609,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L34" s="21" t="str">
-        <x:v>5:55–6:25/km</x:v>
-      </x:c>
-      <x:c r="M34" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M34" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 10 km easy 5:50–6:25/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N34" s="30" t="str">
         <x:v>3–4</x:v>
       </x:c>
-      <x:c r="N34" s="23" t="n">
+      <x:c r="O34" s="31" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="O34" s="30" t="str">
+      <x:c r="P34" s="30" t="str">
         <x:v>12 km easy, bez MP.</x:v>
       </x:c>
-      <x:c r="P34" s="30" t="str">
+      <x:c r="Q34" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q34" s="30" t="str"/>
-      <x:c r="R34" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S34" s="21" t="str">
+      <x:c r="R34" s="30" t="str"/>
+      <x:c r="S34" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T34" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-08</x:v>
       </x:c>
-      <x:c r="T34" s="21" t="str">
+      <x:c r="U34" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-08-run-1</x:v>
       </x:c>
-      <x:c r="U34" s="24" t="n">
+      <x:c r="V34" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Long easy 10km 5:50/km-6:25/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W34" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2447,31 +2678,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L35" s="21" t="str">
-        <x:v>6:15–6:45/km</x:v>
-      </x:c>
-      <x:c r="M35" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M35" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N35" s="30" t="str">
         <x:v>2–3</x:v>
       </x:c>
-      <x:c r="N35" s="23" t="n">
+      <x:c r="O35" s="31" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="O35" s="30" t="str">
+      <x:c r="P35" s="30" t="str">
         <x:v>5 km bardzo lekko.</x:v>
       </x:c>
-      <x:c r="P35" s="30" t="str">
+      <x:c r="Q35" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q35" s="30" t="str"/>
-      <x:c r="R35" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S35" s="21" t="str">
+      <x:c r="R35" s="30" t="str"/>
+      <x:c r="S35" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T35" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-09</x:v>
       </x:c>
-      <x:c r="T35" s="21" t="str">
+      <x:c r="U35" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-09-run-1</x:v>
       </x:c>
-      <x:c r="U35" s="24" t="n">
+      <x:c r="V35" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Recovery 3km 6:15/km-6:45/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W35" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2504,23 +2743,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L36" s="21"/>
-      <x:c r="M36" s="21"/>
-      <x:c r="N36" s="23"/>
-      <x:c r="O36" s="30" t="str"/>
-      <x:c r="P36" s="30" t="str">
+      <x:c r="M36" s="30"/>
+      <x:c r="N36" s="30"/>
+      <x:c r="O36" s="31"/>
+      <x:c r="P36" s="30" t="str"/>
+      <x:c r="Q36" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q36" s="30" t="str"/>
-      <x:c r="R36" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S36" s="21" t="str">
+      <x:c r="R36" s="30" t="str"/>
+      <x:c r="S36" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T36" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-10</x:v>
       </x:c>
-      <x:c r="T36" s="21" t="str">
+      <x:c r="U36" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-10-note-1</x:v>
       </x:c>
-      <x:c r="U36" s="24" t="n">
+      <x:c r="V36" s="30" t="str">
+        <x:v>Regeneracja</x:v>
+      </x:c>
+      <x:c r="W36" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2555,29 +2798,33 @@
         <x:v>LEKKA</x:v>
       </x:c>
       <x:c r="L37" s="21"/>
-      <x:c r="M37" s="21" t="str">
+      <x:c r="M37" s="30"/>
+      <x:c r="N37" s="30" t="str">
         <x:v>2–4</x:v>
       </x:c>
-      <x:c r="N37" s="23"/>
-      <x:c r="O37" s="30" t="str">
+      <x:c r="O37" s="31"/>
+      <x:c r="P37" s="30" t="str">
         <x:v>Technika: split squat do ławki, wspięcia łydki, hip hinge bez ciężaru, side plank; 1–2 serie, zostaw 4–5 powtórzeń w zapasie.</x:v>
       </x:c>
-      <x:c r="P37" s="30" t="str">
+      <x:c r="Q37" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q37" s="30" t="str">
+      <x:c r="R37" s="30" t="str">
         <x:v>Bez DOMS i bez pracy do upadku. Przerwij przy bólu &gt;2/10.</x:v>
       </x:c>
-      <x:c r="R37" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S37" s="21" t="str">
+      <x:c r="S37" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T37" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-10</x:v>
       </x:c>
-      <x:c r="T37" s="21" t="str">
+      <x:c r="U37" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-10-strength-1</x:v>
       </x:c>
-      <x:c r="U37" s="24" t="n">
+      <x:c r="V37" s="30" t="str">
+        <x:v>- Technika i stabilizacja 20m 2-4 RPE</x:v>
+      </x:c>
+      <x:c r="W37" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2614,33 +2861,43 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L38" s="21" t="str">
-        <x:v>easy 5:55–6:25/km; podbieg wg RPE</x:v>
-      </x:c>
-      <x:c r="M38" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+      </x:c>
+      <x:c r="M38" s="30" t="str">
+        <x:v>Rozgrzewka: 2.5 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 4 × 3 min pod górę, nachylenie 4–7%, RPE 7; bez targetu tempa. Przerwy: pełny trucht w dół 3 min, target otwarty, RPE 2–3. Schłodzenie: 2 km 6:10–6:40/km, RPE 2–3. Podbieg wykonywany na wysiłek — nie kontroluj tempa chwilowego.</x:v>
+      </x:c>
+      <x:c r="N38" s="30" t="str">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="N38" s="23" t="n">
+      <x:c r="O38" s="31" t="n">
         <x:v>240</x:v>
       </x:c>
-      <x:c r="O38" s="30" t="str">
+      <x:c r="P38" s="30" t="str">
         <x:v>4 × 3 min pod górę równo, bez finiszu</x:v>
       </x:c>
-      <x:c r="P38" s="30" t="str">
+      <x:c r="Q38" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q38" s="30" t="str">
+      <x:c r="R38" s="30" t="str">
         <x:v>Nie utrzymuj konkretnego tempa na stromym podbiegu.</x:v>
       </x:c>
-      <x:c r="R38" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S38" s="21" t="str">
+      <x:c r="S38" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T38" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-11</x:v>
       </x:c>
-      <x:c r="T38" s="21" t="str">
+      <x:c r="U38" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-11-run-1</x:v>
       </x:c>
-      <x:c r="U38" s="24" t="n">
+      <x:c r="V38" s="30" t="str">
+        <x:v>- Warmup 2.5km 6:00/km-6:30/km Pace
+Uphill effort 4x
+- Uphill 180s 7 RPE
+- Full jog-down recovery 180s open
+- Cooldown 2km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W38" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2673,23 +2930,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L39" s="21"/>
-      <x:c r="M39" s="21"/>
-      <x:c r="N39" s="23"/>
-      <x:c r="O39" s="30" t="str"/>
-      <x:c r="P39" s="30" t="str">
+      <x:c r="M39" s="30"/>
+      <x:c r="N39" s="30"/>
+      <x:c r="O39" s="31"/>
+      <x:c r="P39" s="30" t="str"/>
+      <x:c r="Q39" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q39" s="30" t="str"/>
-      <x:c r="R39" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S39" s="21" t="str">
+      <x:c r="R39" s="30" t="str"/>
+      <x:c r="S39" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T39" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-12</x:v>
       </x:c>
-      <x:c r="T39" s="21" t="str">
+      <x:c r="U39" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-12-note-1</x:v>
       </x:c>
-      <x:c r="U39" s="24" t="n">
+      <x:c r="V39" s="30" t="str">
+        <x:v>Pełne wolne</x:v>
+      </x:c>
+      <x:c r="W39" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2726,31 +2987,39 @@
         <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L40" s="21" t="str">
-        <x:v>6:15–6:45/km</x:v>
-      </x:c>
-      <x:c r="M40" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M40" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N40" s="30" t="str">
         <x:v>2–3</x:v>
       </x:c>
-      <x:c r="N40" s="23"/>
-      <x:c r="O40" s="30" t="str">
+      <x:c r="O40" s="31"/>
+      <x:c r="P40" s="30" t="str">
         <x:v>5 km bardzo swobodnie, bez dokładania kilometrów.</x:v>
       </x:c>
-      <x:c r="P40" s="30" t="str">
+      <x:c r="Q40" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q40" s="30" t="str">
-        <x:v>Dostępne dopiero od 10.08; wybierz albo ten bieg, albo rower Z2, albo wolne.</x:v>
-      </x:c>
       <x:c r="R40" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S40" s="21" t="str">
+        <x:v>Dostępne dopiero od 10.08; wybierz albo ten bieg, albo rower Z2, albo wolne. Wybierz tylko jedną opcję z grupy alt-2026-08-12.</x:v>
+      </x:c>
+      <x:c r="S40" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T40" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-12</x:v>
       </x:c>
-      <x:c r="T40" s="21" t="str">
+      <x:c r="U40" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-12-run-alt</x:v>
       </x:c>
-      <x:c r="U40" s="24" t="n">
+      <x:c r="V40" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Recovery 3km 6:15/km-6:45/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W40" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2784,30 +3053,38 @@
       <x:c r="K41" s="21" t="str">
         <x:v>REGENERACJA</x:v>
       </x:c>
-      <x:c r="L41" s="21"/>
-      <x:c r="M41" s="21" t="str">
-        <x:v>2–3</x:v>
-      </x:c>
-      <x:c r="N41" s="23"/>
-      <x:c r="O41" s="30" t="str">
+      <x:c r="L41" s="21" t="str">
+        <x:v>Z2 • RPE 3</x:v>
+      </x:c>
+      <x:c r="M41" s="30" t="str">
+        <x:v>Rower Z2, RPE 3; bez tempa biegowego. Wybierz tylko jedną opcję ALT.</x:v>
+      </x:c>
+      <x:c r="N41" s="30" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O41" s="31"/>
+      <x:c r="P41" s="30" t="str">
         <x:v>45 min spokojnego Z2, kadencja 85–95; bez sweet spotu.</x:v>
       </x:c>
-      <x:c r="P41" s="30" t="str">
+      <x:c r="Q41" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q41" s="30" t="str">
-        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem.</x:v>
-      </x:c>
       <x:c r="R41" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S41" s="21" t="str">
+        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem. Wybierz tylko jedną opcję z grupy alt-2026-08-12.</x:v>
+      </x:c>
+      <x:c r="S41" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T41" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-12</x:v>
       </x:c>
-      <x:c r="T41" s="21" t="str">
+      <x:c r="U41" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-12-ride-alt</x:v>
       </x:c>
-      <x:c r="U41" s="24" t="n">
+      <x:c r="V41" s="30" t="str">
+        <x:v>- Easy spin 45m 55-70% 85-95rpm</x:v>
+      </x:c>
+      <x:c r="W41" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2844,31 +3121,40 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L42" s="21" t="str">
-        <x:v>8 km 5:50–6:15/km + 3 km 5:20–5:35/km</x:v>
-      </x:c>
-      <x:c r="M42" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:45–6:15/km • 5:20–5:35/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M42" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 6 km średnio-długiego easy 5:45–6:15/km, RPE 3–4 + 3 km steady 5:20–5:35/km, RPE 5–6. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N42" s="30" t="str">
         <x:v>3–5</x:v>
       </x:c>
-      <x:c r="N42" s="23" t="n">
+      <x:c r="O42" s="31" t="n">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="O42" s="30" t="str">
+      <x:c r="P42" s="30" t="str">
         <x:v>3 km steady</x:v>
       </x:c>
-      <x:c r="P42" s="30" t="str">
+      <x:c r="Q42" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q42" s="30" t="str"/>
-      <x:c r="R42" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S42" s="21" t="str">
+      <x:c r="R42" s="30" t="str"/>
+      <x:c r="S42" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T42" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-13</x:v>
       </x:c>
-      <x:c r="T42" s="21" t="str">
+      <x:c r="U42" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-13-run-1</x:v>
       </x:c>
-      <x:c r="U42" s="24" t="n">
+      <x:c r="V42" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Medium long easy 6km 5:45/km-6:15/km Pace
+- Steady 3km 5:20/km-5:35/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W42" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2901,23 +3187,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L43" s="21"/>
-      <x:c r="M43" s="21"/>
-      <x:c r="N43" s="23"/>
-      <x:c r="O43" s="30" t="str"/>
-      <x:c r="P43" s="30" t="str">
+      <x:c r="M43" s="30"/>
+      <x:c r="N43" s="30"/>
+      <x:c r="O43" s="31"/>
+      <x:c r="P43" s="30" t="str"/>
+      <x:c r="Q43" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q43" s="30" t="str"/>
-      <x:c r="R43" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S43" s="21" t="str">
+      <x:c r="R43" s="30" t="str"/>
+      <x:c r="S43" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T43" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-14</x:v>
       </x:c>
-      <x:c r="T43" s="21" t="str">
+      <x:c r="U43" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-14-note-1</x:v>
       </x:c>
-      <x:c r="U43" s="24" t="n">
+      <x:c r="V43" s="30" t="str">
+        <x:v>WOLNE przed bramką 18–20 km</x:v>
+      </x:c>
+      <x:c r="W43" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2954,33 +3244,42 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L44" s="21" t="str">
-        <x:v>easy 5:55–6:25/km; MP tylko warunkowo</x:v>
-      </x:c>
-      <x:c r="M44" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 4:58–5:03/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M44" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3 w obu wariantach. Część główna — wariant 18 km: 16 km easy 5:50–6:25/km, RPE 3–4. Część główna — wariant 20 km tylko po spełnieniu bramki: 15 km easy 5:50–6:25/km + 3 km docelowego MP 3:30 4:58–5:03/km, RPE maks. 6. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N44" s="30" t="str">
         <x:v>easy ≤4</x:v>
       </x:c>
-      <x:c r="N44" s="23" t="n">
+      <x:c r="O44" s="31" t="n">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="O44" s="30" t="str">
+      <x:c r="P44" s="30" t="str">
         <x:v>18 km easy. Dodaj do 20 km wyłącznie po spełnieniu warunków; opcjonalnie ostatnie 3 km przy wysiłku maratońskim, nie szybciej.</x:v>
       </x:c>
-      <x:c r="P44" s="30" t="str">
+      <x:c r="Q44" s="30" t="str">
         <x:v>18 km easy bez MP. Przerwij wcześniej przy narastającym bólu lub zmianie kroku.</x:v>
       </x:c>
-      <x:c r="Q44" s="30" t="str">
+      <x:c r="R44" s="30" t="str">
         <x:v>20 km tylko przy bólu 0–2/10, easy RPE ≤4 i braku pogorszenia następnego ranka. W innym przypadku 18 km easy bez bloku docelowego MP.</x:v>
       </x:c>
-      <x:c r="R44" s="30" t="str">
+      <x:c r="S44" s="30" t="str">
         <x:v>Śniadanie 2–3 h przed. 40–60 g węgli/h, płyny i sód według pogody; nic nowego.</x:v>
       </x:c>
-      <x:c r="S44" s="21" t="str">
+      <x:c r="T44" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-15</x:v>
       </x:c>
-      <x:c r="T44" s="21" t="str">
+      <x:c r="U44" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-15-run-1</x:v>
       </x:c>
-      <x:c r="U44" s="24" t="n">
+      <x:c r="V44" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Easy 15km 5:50/km-6:25/km Pace
+- Conditional goal MP 3km 4:58/km-5:03/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W44" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -3017,33 +3316,41 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L45" s="21" t="str">
-        <x:v>6:20–6:50/km</x:v>
-      </x:c>
-      <x:c r="M45" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M45" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 2 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N45" s="30" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="N45" s="23" t="n">
+      <x:c r="O45" s="31" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="O45" s="30" t="str">
+      <x:c r="P45" s="30" t="str">
         <x:v>4 km wyłącznie jeśli rano brak pogorszenia.</x:v>
       </x:c>
-      <x:c r="P45" s="30" t="str">
+      <x:c r="Q45" s="30" t="str">
         <x:v>Pełne wolne.</x:v>
       </x:c>
-      <x:c r="Q45" s="30" t="str">
+      <x:c r="R45" s="30" t="str">
         <x:v>Jeśli rano ból/sztywność większe niż przed longiem — pełne wolne.</x:v>
       </x:c>
-      <x:c r="R45" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S45" s="21" t="str">
+      <x:c r="S45" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T45" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-16</x:v>
       </x:c>
-      <x:c r="T45" s="21" t="str">
+      <x:c r="U45" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-16-run-1</x:v>
       </x:c>
-      <x:c r="U45" s="24" t="n">
+      <x:c r="V45" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Recovery 2km 6:15/km-6:45/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W45" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3076,23 +3383,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L46" s="21"/>
-      <x:c r="M46" s="21"/>
-      <x:c r="N46" s="23"/>
-      <x:c r="O46" s="30" t="str"/>
-      <x:c r="P46" s="30" t="str">
+      <x:c r="M46" s="30"/>
+      <x:c r="N46" s="30"/>
+      <x:c r="O46" s="31"/>
+      <x:c r="P46" s="30" t="str"/>
+      <x:c r="Q46" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q46" s="30" t="str"/>
-      <x:c r="R46" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S46" s="21" t="str">
+      <x:c r="R46" s="30" t="str"/>
+      <x:c r="S46" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T46" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-17</x:v>
       </x:c>
-      <x:c r="T46" s="21" t="str">
+      <x:c r="U46" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-17-note-1</x:v>
       </x:c>
-      <x:c r="U46" s="24" t="n">
+      <x:c r="V46" s="30" t="str">
+        <x:v>Regeneracja</x:v>
+      </x:c>
+      <x:c r="W46" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3127,29 +3438,33 @@
         <x:v>LEKKA</x:v>
       </x:c>
       <x:c r="L47" s="21"/>
-      <x:c r="M47" s="21" t="str">
+      <x:c r="M47" s="30"/>
+      <x:c r="N47" s="30" t="str">
         <x:v>2–4</x:v>
       </x:c>
-      <x:c r="N47" s="23"/>
-      <x:c r="O47" s="30" t="str">
+      <x:c r="O47" s="31"/>
+      <x:c r="P47" s="30" t="str">
         <x:v>Technika: split squat do ławki, wspięcia łydki, hip hinge bez ciężaru, side plank; 1–2 serie, zostaw 4–5 powtórzeń w zapasie.</x:v>
       </x:c>
-      <x:c r="P47" s="30" t="str">
+      <x:c r="Q47" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q47" s="30" t="str">
+      <x:c r="R47" s="30" t="str">
         <x:v>Tylko jeśli po 15.08 nie ma DOMS ani pogorszenia; w innym przypadku mobilność 10 min.</x:v>
       </x:c>
-      <x:c r="R47" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S47" s="21" t="str">
+      <x:c r="S47" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T47" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-17</x:v>
       </x:c>
-      <x:c r="T47" s="21" t="str">
+      <x:c r="U47" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-17-strength-1</x:v>
       </x:c>
-      <x:c r="U47" s="24" t="n">
+      <x:c r="V47" s="30" t="str">
+        <x:v>- Technika i stabilizacja 18m 2-4 RPE</x:v>
+      </x:c>
+      <x:c r="W47" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3186,31 +3501,41 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L48" s="21" t="str">
-        <x:v>odcinki 4:58–5:05/km</x:v>
-      </x:c>
-      <x:c r="M48" s="21" t="str">
-        <x:v>6–7</x:v>
-      </x:c>
-      <x:c r="N48" s="23" t="n">
+        <x:v>6:00–6:30/km albo wolniej • 4:58–5:05/km • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M48" s="30" t="str">
+        <x:v>Rozgrzewka: 1.5 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 3 × 2 km 4:58–5:05/km, RPE 7, na płaskim. Przerwy: 3 min truchtu 6:15–6:45/km, RPE 2–3. Schłodzenie: 1.5 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N48" s="30" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="O48" s="31" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="O48" s="30" t="str">
+      <x:c r="P48" s="30" t="str">
         <x:v>3 × 2 km progowo</x:v>
       </x:c>
-      <x:c r="P48" s="30" t="str">
+      <x:c r="Q48" s="30" t="str">
         <x:v>Zamień na 7–8 km easy, jeśli 15.08 pozostawiło zmęczenie lub ból.</x:v>
       </x:c>
-      <x:c r="Q48" s="30" t="str"/>
-      <x:c r="R48" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S48" s="21" t="str">
+      <x:c r="R48" s="30" t="str"/>
+      <x:c r="S48" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T48" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-18</x:v>
       </x:c>
-      <x:c r="T48" s="21" t="str">
+      <x:c r="U48" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-18-run-1</x:v>
       </x:c>
-      <x:c r="U48" s="24" t="n">
+      <x:c r="V48" s="30" t="str">
+        <x:v>- Warmup 1.5km 6:00/km-6:30/km Pace
+Threshold 3x
+- Threshold 2km 4:58/km-5:05/km Pace
+- Recovery 3m 6:15/km-6:45/km Pace
+- Cooldown 1.5km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W48" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3243,23 +3568,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L49" s="21"/>
-      <x:c r="M49" s="21"/>
-      <x:c r="N49" s="23"/>
-      <x:c r="O49" s="30" t="str"/>
-      <x:c r="P49" s="30" t="str">
+      <x:c r="M49" s="30"/>
+      <x:c r="N49" s="30"/>
+      <x:c r="O49" s="31"/>
+      <x:c r="P49" s="30" t="str"/>
+      <x:c r="Q49" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q49" s="30" t="str"/>
-      <x:c r="R49" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S49" s="21" t="str">
+      <x:c r="R49" s="30" t="str"/>
+      <x:c r="S49" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T49" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-19</x:v>
       </x:c>
-      <x:c r="T49" s="21" t="str">
+      <x:c r="U49" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-19-note-1</x:v>
       </x:c>
-      <x:c r="U49" s="24" t="n">
+      <x:c r="V49" s="30" t="str">
+        <x:v>Pełne wolne</x:v>
+      </x:c>
+      <x:c r="W49" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3296,31 +3625,39 @@
         <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L50" s="21" t="str">
-        <x:v>6:15–6:45/km</x:v>
-      </x:c>
-      <x:c r="M50" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M50" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N50" s="30" t="str">
         <x:v>2–3</x:v>
       </x:c>
-      <x:c r="N50" s="23"/>
-      <x:c r="O50" s="30" t="str">
+      <x:c r="O50" s="31"/>
+      <x:c r="P50" s="30" t="str">
         <x:v>5 km bardzo swobodnie, bez dokładania kilometrów.</x:v>
       </x:c>
-      <x:c r="P50" s="30" t="str">
+      <x:c r="Q50" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q50" s="30" t="str">
-        <x:v>Dostępne dopiero od 10.08; wybierz albo ten bieg, albo rower Z2, albo wolne.</x:v>
-      </x:c>
       <x:c r="R50" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S50" s="21" t="str">
+        <x:v>Dostępne dopiero od 10.08; wybierz albo ten bieg, albo rower Z2, albo wolne. Wybierz tylko jedną opcję z grupy alt-2026-08-19.</x:v>
+      </x:c>
+      <x:c r="S50" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T50" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-19</x:v>
       </x:c>
-      <x:c r="T50" s="21" t="str">
+      <x:c r="U50" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-19-run-alt</x:v>
       </x:c>
-      <x:c r="U50" s="24" t="n">
+      <x:c r="V50" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Recovery 3km 6:15/km-6:45/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W50" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3354,30 +3691,38 @@
       <x:c r="K51" s="21" t="str">
         <x:v>REGENERACJA</x:v>
       </x:c>
-      <x:c r="L51" s="21"/>
-      <x:c r="M51" s="21" t="str">
-        <x:v>2–3</x:v>
-      </x:c>
-      <x:c r="N51" s="23"/>
-      <x:c r="O51" s="30" t="str">
+      <x:c r="L51" s="21" t="str">
+        <x:v>Z2 • RPE 3</x:v>
+      </x:c>
+      <x:c r="M51" s="30" t="str">
+        <x:v>Rower Z2, RPE 3; bez tempa biegowego. Wybierz tylko jedną opcję ALT.</x:v>
+      </x:c>
+      <x:c r="N51" s="30" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O51" s="31"/>
+      <x:c r="P51" s="30" t="str">
         <x:v>45 min spokojnego Z2, kadencja 85–95; bez sweet spotu.</x:v>
       </x:c>
-      <x:c r="P51" s="30" t="str">
+      <x:c r="Q51" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q51" s="30" t="str">
-        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem.</x:v>
-      </x:c>
       <x:c r="R51" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S51" s="21" t="str">
+        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem. Wybierz tylko jedną opcję z grupy alt-2026-08-19.</x:v>
+      </x:c>
+      <x:c r="S51" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T51" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-19</x:v>
       </x:c>
-      <x:c r="T51" s="21" t="str">
+      <x:c r="U51" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-19-ride-alt</x:v>
       </x:c>
-      <x:c r="U51" s="24" t="n">
+      <x:c r="V51" s="30" t="str">
+        <x:v>- Easy spin 45m 55-70% 85-95rpm</x:v>
+      </x:c>
+      <x:c r="W51" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3414,31 +3759,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L52" s="21" t="str">
-        <x:v>5:50–6:20/km</x:v>
-      </x:c>
-      <x:c r="M52" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:45–6:15/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M52" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Średnio-długi easy: 9 km 5:45–6:15/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N52" s="30" t="str">
         <x:v>3–4</x:v>
       </x:c>
-      <x:c r="N52" s="23" t="n">
+      <x:c r="O52" s="31" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O52" s="30" t="str">
+      <x:c r="P52" s="30" t="str">
         <x:v>11 km easy, bez finiszu.</x:v>
       </x:c>
-      <x:c r="P52" s="30" t="str">
+      <x:c r="Q52" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q52" s="30" t="str"/>
-      <x:c r="R52" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S52" s="21" t="str">
+      <x:c r="R52" s="30" t="str"/>
+      <x:c r="S52" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T52" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-20</x:v>
       </x:c>
-      <x:c r="T52" s="21" t="str">
+      <x:c r="U52" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-20-run-1</x:v>
       </x:c>
-      <x:c r="U52" s="24" t="n">
+      <x:c r="V52" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Średnio-długi easy 9km 5:45/km-6:15/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W52" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3471,23 +3824,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L53" s="21"/>
-      <x:c r="M53" s="21"/>
-      <x:c r="N53" s="23"/>
-      <x:c r="O53" s="30" t="str"/>
-      <x:c r="P53" s="30" t="str">
+      <x:c r="M53" s="30"/>
+      <x:c r="N53" s="30"/>
+      <x:c r="O53" s="31"/>
+      <x:c r="P53" s="30" t="str"/>
+      <x:c r="Q53" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q53" s="30" t="str"/>
-      <x:c r="R53" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S53" s="21" t="str">
+      <x:c r="R53" s="30" t="str"/>
+      <x:c r="S53" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T53" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-21</x:v>
       </x:c>
-      <x:c r="T53" s="21" t="str">
+      <x:c r="U53" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-21-note-1</x:v>
       </x:c>
-      <x:c r="U53" s="24" t="n">
+      <x:c r="V53" s="30" t="str">
+        <x:v>WOLNE przed bramką 22–24 km</x:v>
+      </x:c>
+      <x:c r="W53" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3524,33 +3881,42 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L54" s="21" t="str">
-        <x:v>easy 5:55–6:30/km; blok 5:15–5:25/km warunkowo</x:v>
-      </x:c>
-      <x:c r="M54" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 5:15–5:25/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M54" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3 w każdym wariancie. Część główna — wariant 22 km easy: 20 km easy 5:50–6:25/km, RPE 3–4. Część główna — wariant 22 km z blokiem: 17 km easy 5:50–6:25/km + 3 km aktualnego wysiłku maratońskiego 5:15–5:25/km, RPE 5–6. Część główna — wariant 24 km po zaliczeniu 15.08: 19 km easy 5:50–6:25/km + 3 km aktualnego wysiłku maratońskiego 5:15–5:25/km. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N54" s="30" t="str">
         <x:v>3–5</x:v>
       </x:c>
-      <x:c r="N54" s="23" t="n">
+      <x:c r="O54" s="31" t="n">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="O54" s="30" t="str">
+      <x:c r="P54" s="30" t="str">
         <x:v>22 km easy. 24 km tylko po zaliczeniu 15.08. Jeśli bramka 15.08 niezaliczona: 22 km easy albo jeden blok 3 km przy aktualnym wysiłku maratońskim.</x:v>
       </x:c>
-      <x:c r="P54" s="30" t="str">
+      <x:c r="Q54" s="30" t="str">
         <x:v>22 km easy albo 19 km easy + jeden blok 3 km aktualnego wysiłku maratońskiego; bez docelowego MP.</x:v>
       </x:c>
-      <x:c r="Q54" s="30" t="str">
+      <x:c r="R54" s="30" t="str">
         <x:v>24 km tylko po zaliczeniu 15.08: ból 0–2/10, easy RPE ≤4, brak pogorszenia następnego ranka. Bez zaliczenia: maks. 22 km.</x:v>
       </x:c>
-      <x:c r="R54" s="30" t="str">
+      <x:c r="S54" s="30" t="str">
         <x:v>Śniadanie 2–3 h przed. 40–60 g węgli/h, płyny i sód według pogody; nic nowego.</x:v>
       </x:c>
-      <x:c r="S54" s="21" t="str">
+      <x:c r="T54" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-22</x:v>
       </x:c>
-      <x:c r="T54" s="21" t="str">
+      <x:c r="U54" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-22-run-1</x:v>
       </x:c>
-      <x:c r="U54" s="24" t="n">
+      <x:c r="V54" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Long easy 19km 5:50/km-6:25/km Pace
+- Conditional current marathon effort 3km 5:15/km-5:25/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W54" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -3587,31 +3953,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L55" s="21" t="str">
-        <x:v>6:20–6:50/km</x:v>
-      </x:c>
-      <x:c r="M55" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M55" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N55" s="30" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="N55" s="23" t="n">
+      <x:c r="O55" s="31" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="O55" s="30" t="str">
+      <x:c r="P55" s="30" t="str">
         <x:v>5 km wyłącznie jeśli brak pogorszenia.</x:v>
       </x:c>
-      <x:c r="P55" s="30" t="str">
+      <x:c r="Q55" s="30" t="str">
         <x:v>Pełne wolne.</x:v>
       </x:c>
-      <x:c r="Q55" s="30" t="str"/>
-      <x:c r="R55" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S55" s="21" t="str">
+      <x:c r="R55" s="30" t="str"/>
+      <x:c r="S55" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T55" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-23</x:v>
       </x:c>
-      <x:c r="T55" s="21" t="str">
+      <x:c r="U55" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-23-run-1</x:v>
       </x:c>
-      <x:c r="U55" s="24" t="n">
+      <x:c r="V55" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Recovery 3km 6:15/km-6:45/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W55" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3644,23 +4018,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L56" s="21"/>
-      <x:c r="M56" s="21"/>
-      <x:c r="N56" s="23"/>
-      <x:c r="O56" s="30" t="str"/>
-      <x:c r="P56" s="30" t="str">
+      <x:c r="M56" s="30"/>
+      <x:c r="N56" s="30"/>
+      <x:c r="O56" s="31"/>
+      <x:c r="P56" s="30" t="str"/>
+      <x:c r="Q56" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q56" s="30" t="str"/>
-      <x:c r="R56" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S56" s="21" t="str">
+      <x:c r="R56" s="30" t="str"/>
+      <x:c r="S56" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T56" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-24</x:v>
       </x:c>
-      <x:c r="T56" s="21" t="str">
+      <x:c r="U56" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-24-note-1</x:v>
       </x:c>
-      <x:c r="U56" s="24" t="n">
+      <x:c r="V56" s="30" t="str">
+        <x:v>Regeneracja</x:v>
+      </x:c>
+      <x:c r="W56" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3695,29 +4073,33 @@
         <x:v>LEKKA</x:v>
       </x:c>
       <x:c r="L57" s="21"/>
-      <x:c r="M57" s="21" t="str">
+      <x:c r="M57" s="30"/>
+      <x:c r="N57" s="30" t="str">
         <x:v>2–4</x:v>
       </x:c>
-      <x:c r="N57" s="23"/>
-      <x:c r="O57" s="30" t="str">
+      <x:c r="O57" s="31"/>
+      <x:c r="P57" s="30" t="str">
         <x:v>Technika: split squat do ławki, wspięcia łydki, hip hinge bez ciężaru, side plank; 1–2 serie, zostaw 4–5 powtórzeń w zapasie.</x:v>
       </x:c>
-      <x:c r="P57" s="30" t="str">
+      <x:c r="Q57" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q57" s="30" t="str">
+      <x:c r="R57" s="30" t="str">
         <x:v>Pomiń przy DOMS lub pogorszeniu po 22.08.</x:v>
       </x:c>
-      <x:c r="R57" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S57" s="21" t="str">
+      <x:c r="S57" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T57" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-24</x:v>
       </x:c>
-      <x:c r="T57" s="21" t="str">
+      <x:c r="U57" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-24-strength-1</x:v>
       </x:c>
-      <x:c r="U57" s="24" t="n">
+      <x:c r="V57" s="30" t="str">
+        <x:v>- Technika i stabilizacja 18m 2-4 RPE</x:v>
+      </x:c>
+      <x:c r="W57" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3754,33 +4136,41 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L58" s="21" t="str">
-        <x:v>blok 5:15–5:25/km; 4:58/km tylko po obu bramkach</x:v>
-      </x:c>
-      <x:c r="M58" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:15–5:25/km • 4:58–5:03/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M58" s="30" t="str">
+        <x:v>Rozgrzewka: 2 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 6 km aktualnego wysiłku maratońskiego 5:15–5:25/km, RPE 5–6. Docelowe MP 3:30 4:58–5:03/km, RPE maks. 6, wyłącznie po zaliczeniu obu bramek. Przerwy: nie dotyczy. Schłodzenie: 2 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N58" s="30" t="str">
         <x:v>5–6</x:v>
       </x:c>
-      <x:c r="N58" s="23" t="n">
+      <x:c r="O58" s="31" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="O58" s="30" t="str">
+      <x:c r="P58" s="30" t="str">
         <x:v>6 km przy aktualnym wysiłku maratońskim</x:v>
       </x:c>
-      <x:c r="P58" s="30" t="str">
+      <x:c r="Q58" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q58" s="30" t="str">
+      <x:c r="R58" s="30" t="str">
         <x:v>Docelowe MP 4:58/km wolno testować tylko po zaliczeniu bramek 15.08 i 22.08; bez ścigania.</x:v>
       </x:c>
-      <x:c r="R58" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S58" s="21" t="str">
+      <x:c r="S58" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T58" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-25</x:v>
       </x:c>
-      <x:c r="T58" s="21" t="str">
+      <x:c r="U58" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-25-run-1</x:v>
       </x:c>
-      <x:c r="U58" s="24" t="n">
+      <x:c r="V58" s="30" t="str">
+        <x:v>- Warmup 2km 6:00/km-6:30/km Pace
+- Current marathon effort 6km 5:15/km-5:25/km Pace
+- Cooldown 2km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W58" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3813,23 +4203,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L59" s="21"/>
-      <x:c r="M59" s="21"/>
-      <x:c r="N59" s="23"/>
-      <x:c r="O59" s="30" t="str"/>
-      <x:c r="P59" s="30" t="str">
+      <x:c r="M59" s="30"/>
+      <x:c r="N59" s="30"/>
+      <x:c r="O59" s="31"/>
+      <x:c r="P59" s="30" t="str"/>
+      <x:c r="Q59" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q59" s="30" t="str"/>
-      <x:c r="R59" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S59" s="21" t="str">
+      <x:c r="R59" s="30" t="str"/>
+      <x:c r="S59" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T59" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-26</x:v>
       </x:c>
-      <x:c r="T59" s="21" t="str">
+      <x:c r="U59" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-26-note-1</x:v>
       </x:c>
-      <x:c r="U59" s="24" t="n">
+      <x:c r="V59" s="30" t="str">
+        <x:v>Pełne wolne</x:v>
+      </x:c>
+      <x:c r="W59" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3866,31 +4260,39 @@
         <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L60" s="21" t="str">
-        <x:v>6:15–6:45/km</x:v>
-      </x:c>
-      <x:c r="M60" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M60" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N60" s="30" t="str">
         <x:v>2–3</x:v>
       </x:c>
-      <x:c r="N60" s="23"/>
-      <x:c r="O60" s="30" t="str">
+      <x:c r="O60" s="31"/>
+      <x:c r="P60" s="30" t="str">
         <x:v>5 km bardzo swobodnie, bez dokładania kilometrów.</x:v>
       </x:c>
-      <x:c r="P60" s="30" t="str">
+      <x:c r="Q60" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q60" s="30" t="str">
-        <x:v>Dostępne dopiero od 10.08; wybierz albo ten bieg, albo rower Z2, albo wolne.</x:v>
-      </x:c>
       <x:c r="R60" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S60" s="21" t="str">
+        <x:v>Dostępne dopiero od 10.08; wybierz albo ten bieg, albo rower Z2, albo wolne. Wybierz tylko jedną opcję z grupy alt-2026-08-26.</x:v>
+      </x:c>
+      <x:c r="S60" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T60" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-26</x:v>
       </x:c>
-      <x:c r="T60" s="21" t="str">
+      <x:c r="U60" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-26-run-alt</x:v>
       </x:c>
-      <x:c r="U60" s="24" t="n">
+      <x:c r="V60" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Recovery 3km 6:15/km-6:45/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W60" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3924,30 +4326,38 @@
       <x:c r="K61" s="21" t="str">
         <x:v>REGENERACJA</x:v>
       </x:c>
-      <x:c r="L61" s="21"/>
-      <x:c r="M61" s="21" t="str">
-        <x:v>2–3</x:v>
-      </x:c>
-      <x:c r="N61" s="23"/>
-      <x:c r="O61" s="30" t="str">
+      <x:c r="L61" s="21" t="str">
+        <x:v>Z2 • RPE 3</x:v>
+      </x:c>
+      <x:c r="M61" s="30" t="str">
+        <x:v>Rower Z2, RPE 3; bez tempa biegowego. Wybierz tylko jedną opcję ALT.</x:v>
+      </x:c>
+      <x:c r="N61" s="30" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O61" s="31"/>
+      <x:c r="P61" s="30" t="str">
         <x:v>40 min spokojnego Z2, kadencja 85–95; bez sweet spotu.</x:v>
       </x:c>
-      <x:c r="P61" s="30" t="str">
+      <x:c r="Q61" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q61" s="30" t="str">
-        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem.</x:v>
-      </x:c>
       <x:c r="R61" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S61" s="21" t="str">
+        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem. Wybierz tylko jedną opcję z grupy alt-2026-08-26.</x:v>
+      </x:c>
+      <x:c r="S61" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T61" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-26</x:v>
       </x:c>
-      <x:c r="T61" s="21" t="str">
+      <x:c r="U61" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-26-ride-alt</x:v>
       </x:c>
-      <x:c r="U61" s="24" t="n">
+      <x:c r="V61" s="30" t="str">
+        <x:v>- Easy spin 40m 55-70% 85-95rpm</x:v>
+      </x:c>
+      <x:c r="W61" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -3984,33 +4394,44 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L62" s="21" t="str">
-        <x:v>5:50–6:20/km</x:v>
-      </x:c>
-      <x:c r="M62" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:45–6:15/km • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+      </x:c>
+      <x:c r="M62" s="30" t="str">
+        <x:v>Rozgrzewka: 2 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 7 km średnio-długiego easy 5:45–6:15/km, RPE 3–4 + 6 × 10 s hill sprint techniczny, nachylenie 4–6%, RPE 8, bez targetu tempa. Przerwy: 2 min pełnego marszu/truchtu w dół, target otwarty. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Podbieg wykonywany na wysiłek — nie kontroluj tempa chwilowego. Garmin bez alarmu tempa na hill sprintach.</x:v>
+      </x:c>
+      <x:c r="N62" s="30" t="str">
         <x:v>3–4</x:v>
       </x:c>
-      <x:c r="N62" s="23" t="n">
+      <x:c r="O62" s="31" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="O62" s="30" t="str">
+      <x:c r="P62" s="30" t="str">
         <x:v>6 × 10 s sprężyście pod górę, nie maksymalnie</x:v>
       </x:c>
-      <x:c r="P62" s="30" t="str">
+      <x:c r="Q62" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q62" s="30" t="str">
+      <x:c r="R62" s="30" t="str">
         <x:v>Bez celu tempa na podbiegu; hill sprints nie są osobnym ciężkim bodźcem.</x:v>
       </x:c>
-      <x:c r="R62" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S62" s="21" t="str">
+      <x:c r="S62" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T62" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-27</x:v>
       </x:c>
-      <x:c r="T62" s="21" t="str">
+      <x:c r="U62" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-27-run-1</x:v>
       </x:c>
-      <x:c r="U62" s="24" t="n">
+      <x:c r="V62" s="30" t="str">
+        <x:v>- Warmup 2km 6:00/km-6:30/km Pace
+- Medium long easy 7km 5:45/km-6:15/km Pace
+Hill sprints 6x
+- Uphill fast relaxed 10s 8 RPE
+- Full walk-jog recovery 2m open
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W62" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4043,23 +4464,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L63" s="21"/>
-      <x:c r="M63" s="21"/>
-      <x:c r="N63" s="23"/>
-      <x:c r="O63" s="30" t="str"/>
-      <x:c r="P63" s="30" t="str">
+      <x:c r="M63" s="30"/>
+      <x:c r="N63" s="30"/>
+      <x:c r="O63" s="31"/>
+      <x:c r="P63" s="30" t="str"/>
+      <x:c r="Q63" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q63" s="30" t="str"/>
-      <x:c r="R63" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S63" s="21" t="str">
+      <x:c r="R63" s="30" t="str"/>
+      <x:c r="S63" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T63" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-28</x:v>
       </x:c>
-      <x:c r="T63" s="21" t="str">
+      <x:c r="U63" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-28-note-1</x:v>
       </x:c>
-      <x:c r="U63" s="24" t="n">
+      <x:c r="V63" s="30" t="str">
+        <x:v>WOLNE przed long runem</x:v>
+      </x:c>
+      <x:c r="W63" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4096,31 +4521,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L64" s="21" t="str">
-        <x:v>5:55–6:30/km wg terenu</x:v>
-      </x:c>
-      <x:c r="M64" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M64" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 14 km easy 5:50–6:25/km na płaskich fragmentach; na podbiegach według wysiłku, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N64" s="30" t="str">
         <x:v>3–5</x:v>
       </x:c>
-      <x:c r="N64" s="23" t="n">
+      <x:c r="O64" s="31" t="n">
         <x:v>240</x:v>
       </x:c>
-      <x:c r="O64" s="30" t="str">
+      <x:c r="P64" s="30" t="str">
         <x:v>16 km easy po pofałdowanej trasie; bez szybkiego finiszu.</x:v>
       </x:c>
-      <x:c r="P64" s="30" t="str">
+      <x:c r="Q64" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q64" s="30" t="str"/>
-      <x:c r="R64" s="30" t="str">
+      <x:c r="R64" s="30" t="str"/>
+      <x:c r="S64" s="30" t="str">
         <x:v>Śniadanie 2–3 h przed. 40–60 g węgli/h, płyny i sód według pogody; nic nowego.</x:v>
       </x:c>
-      <x:c r="S64" s="21" t="str">
+      <x:c r="T64" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-29</x:v>
       </x:c>
-      <x:c r="T64" s="21" t="str">
+      <x:c r="U64" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-29-run-1</x:v>
       </x:c>
-      <x:c r="U64" s="24" t="n">
+      <x:c r="V64" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Long easy 14km 5:50/km-6:25/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W64" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -4157,31 +4590,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L65" s="21" t="str">
-        <x:v>6:15–6:45/km</x:v>
-      </x:c>
-      <x:c r="M65" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M65" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N65" s="30" t="str">
         <x:v>2–3</x:v>
       </x:c>
-      <x:c r="N65" s="23" t="n">
+      <x:c r="O65" s="31" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="O65" s="30" t="str">
+      <x:c r="P65" s="30" t="str">
         <x:v>5 km bardzo lekko.</x:v>
       </x:c>
-      <x:c r="P65" s="30" t="str">
+      <x:c r="Q65" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q65" s="30" t="str"/>
-      <x:c r="R65" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S65" s="21" t="str">
+      <x:c r="R65" s="30" t="str"/>
+      <x:c r="S65" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T65" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-30</x:v>
       </x:c>
-      <x:c r="T65" s="21" t="str">
+      <x:c r="U65" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-30-run-1</x:v>
       </x:c>
-      <x:c r="U65" s="24" t="n">
+      <x:c r="V65" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Recovery 3km 6:15/km-6:45/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W65" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4214,23 +4655,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L66" s="21"/>
-      <x:c r="M66" s="21"/>
-      <x:c r="N66" s="23"/>
-      <x:c r="O66" s="30" t="str"/>
-      <x:c r="P66" s="30" t="str">
+      <x:c r="M66" s="30"/>
+      <x:c r="N66" s="30"/>
+      <x:c r="O66" s="31"/>
+      <x:c r="P66" s="30" t="str"/>
+      <x:c r="Q66" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q66" s="30" t="str"/>
-      <x:c r="R66" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S66" s="21" t="str">
+      <x:c r="R66" s="30" t="str"/>
+      <x:c r="S66" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T66" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-31</x:v>
       </x:c>
-      <x:c r="T66" s="21" t="str">
+      <x:c r="U66" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-31-note-1</x:v>
       </x:c>
-      <x:c r="U66" s="24" t="n">
+      <x:c r="V66" s="30" t="str">
+        <x:v>Regeneracja</x:v>
+      </x:c>
+      <x:c r="W66" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4265,29 +4710,33 @@
         <x:v>LEKKA</x:v>
       </x:c>
       <x:c r="L67" s="21"/>
-      <x:c r="M67" s="21" t="str">
+      <x:c r="M67" s="30"/>
+      <x:c r="N67" s="30" t="str">
         <x:v>2–4</x:v>
       </x:c>
-      <x:c r="N67" s="23"/>
-      <x:c r="O67" s="30" t="str">
+      <x:c r="O67" s="31"/>
+      <x:c r="P67" s="30" t="str">
         <x:v>Mobilność bioder/łydek, dead bug, side plank; bez obciążeń i bez DOMS.</x:v>
       </x:c>
-      <x:c r="P67" s="30" t="str">
+      <x:c r="Q67" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q67" s="30" t="str">
+      <x:c r="R67" s="30" t="str">
         <x:v>Bez DOMS i bez pracy do upadku. Przerwij przy bólu &gt;2/10.</x:v>
       </x:c>
-      <x:c r="R67" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S67" s="21" t="str">
+      <x:c r="S67" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T67" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-31</x:v>
       </x:c>
-      <x:c r="T67" s="21" t="str">
+      <x:c r="U67" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-08-31-strength-1</x:v>
       </x:c>
-      <x:c r="U67" s="24" t="n">
+      <x:c r="V67" s="30" t="str">
+        <x:v>- Mobility and activation 12m 2 RPE</x:v>
+      </x:c>
+      <x:c r="W67" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4324,33 +4773,43 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L68" s="21" t="str">
-        <x:v>wariant A 4:58–5:02/km; B 5:16–5:20/km; C 5:24–5:34/km</x:v>
-      </x:c>
-      <x:c r="M68" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:15–5:25/km • 4:58–5:03/km • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M68" s="30" t="str">
+        <x:v>Rozgrzewka: 2 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 3 × 2 km — wariant A 4:58–5:03/km, RPE maks. 6 wyłącznie po zaliczeniu bramek; wariant B 5:16–5:20/km; wariant C 5:24–5:34/km. Przerwy: 500 m truchtu 6:15–6:45/km, RPE 2–3. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Wszystkie targety dotyczą płaskiego terenu.</x:v>
+      </x:c>
+      <x:c r="N68" s="30" t="str">
         <x:v>5–6</x:v>
       </x:c>
-      <x:c r="N68" s="23" t="n">
+      <x:c r="O68" s="31" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="O68" s="30" t="str">
+      <x:c r="P68" s="30" t="str">
         <x:v>3 × 2 km w tempie odpowiadającym aktualnie zaliczonej strategii</x:v>
       </x:c>
-      <x:c r="P68" s="30" t="str">
+      <x:c r="Q68" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q68" s="30" t="str">
+      <x:c r="R68" s="30" t="str">
         <x:v>Nie wymuszaj 4:58/km. Zapisz RPE, ból i reakcję następnego ranka do decyzji 02.09.</x:v>
       </x:c>
-      <x:c r="R68" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S68" s="21" t="str">
+      <x:c r="S68" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T68" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-01</x:v>
       </x:c>
-      <x:c r="T68" s="21" t="str">
+      <x:c r="U68" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-01-run-1</x:v>
       </x:c>
-      <x:c r="U68" s="24" t="n">
+      <x:c r="V68" s="30" t="str">
+        <x:v>- Warmup 2km 6:00/km-6:30/km Pace
+Race pace calibration 3x
+- Controlled marathon pace 2km 5:15/km-5:25/km Pace
+- Recovery 500m 6:15/km-6:45/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W68" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4383,27 +4842,31 @@
         <x:v>DECYZJA</x:v>
       </x:c>
       <x:c r="L69" s="21"/>
-      <x:c r="M69" s="21"/>
-      <x:c r="N69" s="23"/>
-      <x:c r="O69" s="30" t="str">
+      <x:c r="M69" s="30"/>
+      <x:c r="N69" s="30"/>
+      <x:c r="O69" s="31"/>
+      <x:c r="P69" s="30" t="str">
         <x:v>Wybierz strategię na podstawie treningów 15.08, 22.08 i 01.09.</x:v>
       </x:c>
-      <x:c r="P69" s="30" t="str">
+      <x:c r="Q69" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q69" s="30" t="str">
+      <x:c r="R69" s="30" t="str">
         <x:v>Plan A pozostaje wyłącznie po zaliczeniu wszystkich trzech bramek bez bólu, nadmiernego RPE ani pogorszenia następnego ranka.</x:v>
       </x:c>
-      <x:c r="R69" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S69" s="21" t="str">
+      <x:c r="S69" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T69" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-02</x:v>
       </x:c>
-      <x:c r="T69" s="21" t="str">
+      <x:c r="U69" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-02-decision-1</x:v>
       </x:c>
-      <x:c r="U69" s="24" t="n">
+      <x:c r="V69" s="30" t="str">
+        <x:v>Plan A 3:30 | Plan B 3:42–3:45 | Plan C 3:48–3:55</x:v>
+      </x:c>
+      <x:c r="W69" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4437,30 +4900,38 @@
       <x:c r="K70" s="21" t="str">
         <x:v>REGENERACJA</x:v>
       </x:c>
-      <x:c r="L70" s="21"/>
-      <x:c r="M70" s="21" t="str">
-        <x:v>2–3</x:v>
-      </x:c>
-      <x:c r="N70" s="23"/>
-      <x:c r="O70" s="30" t="str">
+      <x:c r="L70" s="21" t="str">
+        <x:v>Z2 • RPE 3</x:v>
+      </x:c>
+      <x:c r="M70" s="30" t="str">
+        <x:v>Rower Z2, RPE 3; bez tempa biegowego. Wybierz tylko jedną opcję ALT.</x:v>
+      </x:c>
+      <x:c r="N70" s="30" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O70" s="31"/>
+      <x:c r="P70" s="30" t="str">
         <x:v>30 min spokojnego Z2, kadencja 85–95; bez sweet spotu.</x:v>
       </x:c>
-      <x:c r="P70" s="30" t="str">
+      <x:c r="Q70" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q70" s="30" t="str">
-        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem.</x:v>
-      </x:c>
       <x:c r="R70" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S70" s="21" t="str">
+        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem. Wybierz tylko jedną opcję z grupy alt-2026-09-02.</x:v>
+      </x:c>
+      <x:c r="S70" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T70" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-02</x:v>
       </x:c>
-      <x:c r="T70" s="21" t="str">
+      <x:c r="U70" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-02-ride-alt</x:v>
       </x:c>
-      <x:c r="U70" s="24" t="n">
+      <x:c r="V70" s="30" t="str">
+        <x:v>- Easy spin 30m 55-70% 85-95rpm</x:v>
+      </x:c>
+      <x:c r="W70" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4497,31 +4968,42 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L71" s="21" t="str">
-        <x:v>5:55–6:25/km</x:v>
-      </x:c>
-      <x:c r="M71" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+      </x:c>
+      <x:c r="M71" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 6 km easy 5:50–6:25/km, RPE 3–4 + 4 × 15 s rytmu technicznego, RPE 7–8, bez targetu tempa. Przerwy: 90 s pełnego truchtu lub marszu, target otwarty. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Rytmy wykonuj luźno i technicznie; Garmin bez alarmu tempa. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N71" s="30" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="N71" s="23" t="n">
+      <x:c r="O71" s="31" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="O71" s="30" t="str">
+      <x:c r="P71" s="30" t="str">
         <x:v>4 × 15 s rytmu</x:v>
       </x:c>
-      <x:c r="P71" s="30" t="str">
+      <x:c r="Q71" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q71" s="30" t="str"/>
-      <x:c r="R71" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S71" s="21" t="str">
+      <x:c r="R71" s="30" t="str"/>
+      <x:c r="S71" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T71" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-03</x:v>
       </x:c>
-      <x:c r="T71" s="21" t="str">
+      <x:c r="U71" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-03-run-1</x:v>
       </x:c>
-      <x:c r="U71" s="24" t="n">
+      <x:c r="V71" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Easy 6km 5:50/km-6:25/km Pace
+Strides 4x
+- Fast relaxed 15s 7-8 RPE
+- Full recovery 90s open
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W71" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4554,23 +5036,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L72" s="21"/>
-      <x:c r="M72" s="21"/>
-      <x:c r="N72" s="23"/>
-      <x:c r="O72" s="30" t="str"/>
-      <x:c r="P72" s="30" t="str">
+      <x:c r="M72" s="30"/>
+      <x:c r="N72" s="30"/>
+      <x:c r="O72" s="31"/>
+      <x:c r="P72" s="30" t="str"/>
+      <x:c r="Q72" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q72" s="30" t="str"/>
-      <x:c r="R72" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S72" s="21" t="str">
+      <x:c r="R72" s="30" t="str"/>
+      <x:c r="S72" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T72" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-04</x:v>
       </x:c>
-      <x:c r="T72" s="21" t="str">
+      <x:c r="U72" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-04-note-1</x:v>
       </x:c>
-      <x:c r="U72" s="24" t="n">
+      <x:c r="V72" s="30" t="str">
+        <x:v>WOLNE przed krótkim longiem</x:v>
+      </x:c>
+      <x:c r="W72" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4607,31 +5093,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L73" s="21" t="str">
-        <x:v>5:55–6:25/km</x:v>
-      </x:c>
-      <x:c r="M73" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M73" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 6 km easy 5:50–6:25/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N73" s="30" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="N73" s="23" t="n">
+      <x:c r="O73" s="31" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="O73" s="30" t="str">
+      <x:c r="P73" s="30" t="str">
         <x:v>8 km easy, zakończ z niedosytem.</x:v>
       </x:c>
-      <x:c r="P73" s="30" t="str">
+      <x:c r="Q73" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q73" s="30" t="str"/>
-      <x:c r="R73" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S73" s="21" t="str">
+      <x:c r="R73" s="30" t="str"/>
+      <x:c r="S73" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T73" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-05</x:v>
       </x:c>
-      <x:c r="T73" s="21" t="str">
+      <x:c r="U73" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-05-run-1</x:v>
       </x:c>
-      <x:c r="U73" s="24" t="n">
+      <x:c r="V73" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Long easy 6km 5:50/km-6:25/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W73" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -4668,31 +5162,39 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L74" s="21" t="str">
-        <x:v>6:20–6:50/km</x:v>
-      </x:c>
-      <x:c r="M74" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+      </x:c>
+      <x:c r="M74" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 2 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N74" s="30" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="N74" s="23" t="n">
+      <x:c r="O74" s="31" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="O74" s="30" t="str">
+      <x:c r="P74" s="30" t="str">
         <x:v>4 km bardzo lekko.</x:v>
       </x:c>
-      <x:c r="P74" s="30" t="str">
+      <x:c r="Q74" s="30" t="str">
         <x:v>Pełne wolne.</x:v>
       </x:c>
-      <x:c r="Q74" s="30" t="str"/>
-      <x:c r="R74" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S74" s="21" t="str">
+      <x:c r="R74" s="30" t="str"/>
+      <x:c r="S74" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T74" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-06</x:v>
       </x:c>
-      <x:c r="T74" s="21" t="str">
+      <x:c r="U74" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-06-run-1</x:v>
       </x:c>
-      <x:c r="U74" s="24" t="n">
+      <x:c r="V74" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Recovery 2km 6:15/km-6:45/km Pace
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W74" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4725,23 +5227,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L75" s="21"/>
-      <x:c r="M75" s="21"/>
-      <x:c r="N75" s="23"/>
-      <x:c r="O75" s="30" t="str"/>
-      <x:c r="P75" s="30" t="str">
+      <x:c r="M75" s="30"/>
+      <x:c r="N75" s="30"/>
+      <x:c r="O75" s="31"/>
+      <x:c r="P75" s="30" t="str"/>
+      <x:c r="Q75" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q75" s="30" t="str"/>
-      <x:c r="R75" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S75" s="21" t="str">
+      <x:c r="R75" s="30" t="str"/>
+      <x:c r="S75" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T75" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-07</x:v>
       </x:c>
-      <x:c r="T75" s="21" t="str">
+      <x:c r="U75" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-07-note-1</x:v>
       </x:c>
-      <x:c r="U75" s="24" t="n">
+      <x:c r="V75" s="30" t="str">
+        <x:v>WOLNE — początek tygodnia startowego</x:v>
+      </x:c>
+      <x:c r="W75" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4778,31 +5284,42 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L76" s="21" t="str">
-        <x:v>5:55–6:25/km</x:v>
-      </x:c>
-      <x:c r="M76" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+      </x:c>
+      <x:c r="M76" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 3 km easy 5:50–6:25/km, RPE 3–4 + 4 × 15 s rytmu technicznego, RPE 7–8, bez targetu tempa. Przerwy: 90 s pełnego truchtu lub marszu, target otwarty. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Rytmy wykonuj luźno i technicznie; Garmin bez alarmu tempa. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N76" s="30" t="str">
         <x:v>2–3</x:v>
       </x:c>
-      <x:c r="N76" s="23" t="n">
+      <x:c r="O76" s="31" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="O76" s="30" t="str">
+      <x:c r="P76" s="30" t="str">
         <x:v>4 × 15 s rytmu</x:v>
       </x:c>
-      <x:c r="P76" s="30" t="str">
+      <x:c r="Q76" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q76" s="30" t="str"/>
-      <x:c r="R76" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S76" s="21" t="str">
+      <x:c r="R76" s="30" t="str"/>
+      <x:c r="S76" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T76" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-08</x:v>
       </x:c>
-      <x:c r="T76" s="21" t="str">
+      <x:c r="U76" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-08-run-1</x:v>
       </x:c>
-      <x:c r="U76" s="24" t="n">
+      <x:c r="V76" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Easy 3km 5:50/km-6:25/km Pace
+Strides 4x
+- Fast relaxed 15s 7-8 RPE
+- Full recovery 90s open
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W76" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4835,23 +5352,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L77" s="21"/>
-      <x:c r="M77" s="21"/>
-      <x:c r="N77" s="23"/>
-      <x:c r="O77" s="30" t="str"/>
-      <x:c r="P77" s="30" t="str">
+      <x:c r="M77" s="30"/>
+      <x:c r="N77" s="30"/>
+      <x:c r="O77" s="31"/>
+      <x:c r="P77" s="30" t="str"/>
+      <x:c r="Q77" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q77" s="30" t="str"/>
-      <x:c r="R77" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S77" s="21" t="str">
+      <x:c r="R77" s="30" t="str"/>
+      <x:c r="S77" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T77" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-09</x:v>
       </x:c>
-      <x:c r="T77" s="21" t="str">
+      <x:c r="U77" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-09-note-1</x:v>
       </x:c>
-      <x:c r="U77" s="24" t="n">
+      <x:c r="V77" s="30" t="str">
+        <x:v>Pełne wolne</x:v>
+      </x:c>
+      <x:c r="W77" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4885,30 +5406,38 @@
       <x:c r="K78" s="21" t="str">
         <x:v>REGENERACJA</x:v>
       </x:c>
-      <x:c r="L78" s="21"/>
-      <x:c r="M78" s="21" t="str">
-        <x:v>2–3</x:v>
-      </x:c>
-      <x:c r="N78" s="23"/>
-      <x:c r="O78" s="30" t="str">
+      <x:c r="L78" s="21" t="str">
+        <x:v>Z2 • RPE 3</x:v>
+      </x:c>
+      <x:c r="M78" s="30" t="str">
+        <x:v>Rower Z2, RPE 3; bez tempa biegowego. Wybierz tylko jedną opcję ALT.</x:v>
+      </x:c>
+      <x:c r="N78" s="30" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="O78" s="31"/>
+      <x:c r="P78" s="30" t="str">
         <x:v>25 min spokojnego Z2, kadencja 85–95; bez sweet spotu.</x:v>
       </x:c>
-      <x:c r="P78" s="30" t="str">
+      <x:c r="Q78" s="30" t="str">
         <x:v>Przy zmęczeniu wybierz pełny odpoczynek.</x:v>
       </x:c>
-      <x:c r="Q78" s="30" t="str">
-        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem.</x:v>
-      </x:c>
       <x:c r="R78" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S78" s="21" t="str">
+        <x:v>Wykonaj tylko przy świeżych nogach; pełne wolne jest równorzędnym wyborem. Wybierz tylko jedną opcję z grupy alt-2026-09-09.</x:v>
+      </x:c>
+      <x:c r="S78" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T78" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-09</x:v>
       </x:c>
-      <x:c r="T78" s="21" t="str">
+      <x:c r="U78" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-09-ride-alt</x:v>
       </x:c>
-      <x:c r="U78" s="24" t="n">
+      <x:c r="V78" s="30" t="str">
+        <x:v>- Easy spin 25m 55-70% 85-95rpm</x:v>
+      </x:c>
+      <x:c r="W78" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4945,31 +5474,42 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L79" s="21" t="str">
-        <x:v>6:00–6:30/km</x:v>
-      </x:c>
-      <x:c r="M79" s="21" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+      </x:c>
+      <x:c r="M79" s="30" t="str">
+        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 2 km easy 5:50–6:25/km, RPE 3–4 + 3 × 10 s rytmu technicznego, RPE 7–8, bez targetu tempa. Przerwy: 90 s pełnego truchtu lub marszu, target otwarty. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Rytmy wykonuj luźno i technicznie; Garmin bez alarmu tempa. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+      </x:c>
+      <x:c r="N79" s="30" t="str">
         <x:v>2–3</x:v>
       </x:c>
-      <x:c r="N79" s="23" t="n">
+      <x:c r="O79" s="31" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="O79" s="30" t="str">
+      <x:c r="P79" s="30" t="str">
         <x:v>4 km easy + 3 × 10 s luźnego rytmu, jeśli nogi chcą.</x:v>
       </x:c>
-      <x:c r="P79" s="30" t="str">
+      <x:c r="Q79" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
-      <x:c r="Q79" s="30" t="str"/>
-      <x:c r="R79" s="30" t="str">
-        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
-      </x:c>
-      <x:c r="S79" s="21" t="str">
+      <x:c r="R79" s="30" t="str"/>
+      <x:c r="S79" s="30" t="str">
+        <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
+      </x:c>
+      <x:c r="T79" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-10</x:v>
       </x:c>
-      <x:c r="T79" s="21" t="str">
+      <x:c r="U79" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-10-run-1</x:v>
       </x:c>
-      <x:c r="U79" s="24" t="n">
+      <x:c r="V79" s="30" t="str">
+        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
+- Easy 2km 5:50/km-6:25/km Pace
+Strides 3x
+- Fast relaxed 10s 7-8 RPE
+- Full recovery 90s open
+- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+      </x:c>
+      <x:c r="W79" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -5002,23 +5542,27 @@
         <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="L80" s="21"/>
-      <x:c r="M80" s="21"/>
-      <x:c r="N80" s="23"/>
-      <x:c r="O80" s="30" t="str"/>
-      <x:c r="P80" s="30" t="str">
+      <x:c r="M80" s="30"/>
+      <x:c r="N80" s="30"/>
+      <x:c r="O80" s="31"/>
+      <x:c r="P80" s="30" t="str"/>
+      <x:c r="Q80" s="30" t="str">
         <x:v>Ogranicz chodzenie, przygotuj sprzęt i sen.</x:v>
       </x:c>
-      <x:c r="Q80" s="30" t="str"/>
-      <x:c r="R80" s="30" t="str">
+      <x:c r="R80" s="30" t="str"/>
+      <x:c r="S80" s="30" t="str">
         <x:v>Sprawdzone węglowodany, płyny i sód; bez nowych produktów.</x:v>
       </x:c>
-      <x:c r="S80" s="21" t="str">
+      <x:c r="T80" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-11</x:v>
       </x:c>
-      <x:c r="T80" s="21" t="str">
+      <x:c r="U80" s="21" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-11-note-1</x:v>
       </x:c>
-      <x:c r="U80" s="24" t="n">
+      <x:c r="V80" s="30" t="str">
+        <x:v>WOLNE / logistyka</x:v>
+      </x:c>
+      <x:c r="W80" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -5057,38 +5601,46 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L81" s="26" t="str">
-        <x:v>A 4:58/km | B 5:16–5:20/km | C 5:24–5:34/km</x:v>
-      </x:c>
-      <x:c r="M81" s="26" t="str">
+        <x:v>6:00–6:30/km albo wolniej • 4:58–5:03/km</x:v>
+      </x:c>
+      <x:c r="M81" s="32" t="str">
+        <x:v>Rozgrzewka: 10–15 min bardzo lekko, 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: Plan A 3:30 — 4:58–5:03/km, RPE początkowo 5–6, tylko po wszystkich bramkach; Plan B 5:16–5:20/km; Plan C 5:24–5:34/km. Przerwy: brak; punkty żywieniowe pokonuj według sytuacji. Schłodzenie: 10–15 min marszu lub truchtu, target otwarty, RPE 1–2. Tempo dotyczy płaskich fragmentów; na podbiegach utrzymuj wysiłek.</x:v>
+      </x:c>
+      <x:c r="N81" s="32" t="str">
         <x:v>start 5–6, progres wg stanu</x:v>
       </x:c>
-      <x:c r="N81" s="28" t="n">
+      <x:c r="O81" s="33" t="n">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="O81" s="31" t="str">
+      <x:c r="P81" s="32" t="str">
         <x:v>Strategia A 3:30 tylko po wszystkich bramkach. B 3:42–3:45. C 3:48–3:55. Pierwsze 5 km spokojnie, wysiłek równy na podbiegach.</x:v>
       </x:c>
-      <x:c r="P81" s="31" t="str">
+      <x:c r="Q81" s="32" t="str">
         <x:v>Przejdź z A do B/C przy narastającym bólu, RPE ponad plan albo pogorszeniu techniki; zdrowie ma pierwszeństwo.</x:v>
       </x:c>
-      <x:c r="Q81" s="31" t="str">
+      <x:c r="R81" s="32" t="str">
         <x:v>Plan A 3:30 tylko po zaliczeniu bramek 15.08, 22.08 i 01.09 oraz decyzji 02.09. W przeciwnym razie B 3:42–3:45 lub C 3:48–3:55.</x:v>
       </x:c>
-      <x:c r="R81" s="31" t="str">
+      <x:c r="S81" s="32" t="str">
         <x:v>60–75 g węgli/h, płyny i sód przećwiczone na longach; pierwszy żel wcześnie, nic nowego.</x:v>
       </x:c>
-      <x:c r="S81" s="26" t="str">
+      <x:c r="T81" s="26" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-12</x:v>
       </x:c>
-      <x:c r="T81" s="26" t="str">
+      <x:c r="U81" s="26" t="str">
         <x:v>cc-v2-oslo-2026-2026-09-12-run-1</x:v>
       </x:c>
-      <x:c r="U81" s="29" t="n">
+      <x:c r="V81" s="32" t="str">
+        <x:v>- Race controlled start 5km 5:00/km-5:05/km Pace
+- Race strategy block 32.195km 5:15/km-5:25/km Pace
+- Finish by feel 5km 5-8 RPE</x:v>
+      </x:c>
+      <x:c r="W81" s="29" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:U81">
+  <x:conditionalFormatting sqref="A2:W81">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="OPCJONALNE / ALT"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="BRAMKA"/>
   </x:conditionalFormatting>
@@ -5111,48 +5663,48 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="33" t="str">
+      <x:c r="A1" s="35" t="str">
         <x:v>OSLO 2026 — tygodnie, kilometraż i bramki</x:v>
       </x:c>
-      <x:c r="B1" s="33"/>
-      <x:c r="C1" s="33"/>
-      <x:c r="D1" s="33"/>
-      <x:c r="E1" s="33"/>
-      <x:c r="F1" s="33"/>
-      <x:c r="G1" s="33"/>
-      <x:c r="H1" s="33"/>
+      <x:c r="B1" s="35"/>
+      <x:c r="C1" s="35"/>
+      <x:c r="D1" s="35"/>
+      <x:c r="E1" s="35"/>
+      <x:c r="F1" s="35"/>
+      <x:c r="G1" s="35"/>
+      <x:c r="H1" s="35"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="36" t="str">
+      <x:c r="A3" s="38" t="str">
         <x:v>Tydzień od</x:v>
       </x:c>
-      <x:c r="B3" s="36" t="str">
+      <x:c r="B3" s="38" t="str">
         <x:v>Do</x:v>
       </x:c>
-      <x:c r="C3" s="36" t="str">
+      <x:c r="C3" s="38" t="str">
         <x:v>Biegi obowiązkowe</x:v>
       </x:c>
-      <x:c r="D3" s="36" t="str">
+      <x:c r="D3" s="38" t="str">
         <x:v>Km min</x:v>
       </x:c>
-      <x:c r="E3" s="36" t="str">
+      <x:c r="E3" s="38" t="str">
         <x:v>Km max</x:v>
       </x:c>
-      <x:c r="F3" s="36" t="str">
+      <x:c r="F3" s="38" t="str">
         <x:v>Long min</x:v>
       </x:c>
-      <x:c r="G3" s="36" t="str">
+      <x:c r="G3" s="38" t="str">
         <x:v>Long max</x:v>
       </x:c>
-      <x:c r="H3" s="36" t="str">
+      <x:c r="H3" s="38" t="str">
         <x:v>Kontrola</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="37" t="n">
+      <x:c r="A4" s="39" t="n">
         <x:v>46216.5</x:v>
       </x:c>
-      <x:c r="B4" s="37" t="n">
+      <x:c r="B4" s="39" t="n">
         <x:v>46222.5</x:v>
       </x:c>
       <x:c r="C4" s="12" t="n">
@@ -5168,22 +5720,22 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="F4" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A4,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B4,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A4,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B4,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G4" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A4,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B4,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A4,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B4,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="H4" s="38" t="str">
+      <x:c r="H4" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="37" t="n">
+      <x:c r="A5" s="39" t="n">
         <x:v>46223.5</x:v>
       </x:c>
-      <x:c r="B5" s="37" t="n">
+      <x:c r="B5" s="39" t="n">
         <x:v>46229.5</x:v>
       </x:c>
       <x:c r="C5" s="12" t="n">
@@ -5199,22 +5751,22 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F5" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A5,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B5,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A5,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B5,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G5" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A5,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B5,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A5,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B5,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="H5" s="38" t="str">
+      <x:c r="H5" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="37" t="n">
+      <x:c r="A6" s="39" t="n">
         <x:v>46230.5</x:v>
       </x:c>
-      <x:c r="B6" s="37" t="n">
+      <x:c r="B6" s="39" t="n">
         <x:v>46236.5</x:v>
       </x:c>
       <x:c r="C6" s="12" t="n">
@@ -5230,22 +5782,22 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F6" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A6,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B6,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A6,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B6,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="G6" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A6,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B6,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A6,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B6,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>14</x:v>
       </x:c>
-      <x:c r="H6" s="38" t="str">
+      <x:c r="H6" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="37" t="n">
+      <x:c r="A7" s="39" t="n">
         <x:v>46237.5</x:v>
       </x:c>
-      <x:c r="B7" s="37" t="n">
+      <x:c r="B7" s="39" t="n">
         <x:v>46243.5</x:v>
       </x:c>
       <x:c r="C7" s="12" t="n">
@@ -5261,22 +5813,22 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="F7" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A7,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B7,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A7,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B7,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="G7" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A7,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B7,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A7,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B7,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="H7" s="38" t="str">
+      <x:c r="H7" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="37" t="n">
+      <x:c r="A8" s="39" t="n">
         <x:v>46244.5</x:v>
       </x:c>
-      <x:c r="B8" s="37" t="n">
+      <x:c r="B8" s="39" t="n">
         <x:v>46250.5</x:v>
       </x:c>
       <x:c r="C8" s="12" t="n">
@@ -5292,22 +5844,22 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="F8" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A8,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B8,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A8,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B8,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="G8" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A8,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B8,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A8,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B8,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="H8" s="38" t="str">
+      <x:c r="H8" s="40" t="str">
         <x:v>15.08: ból 0–2, RPE ≤4, brak pogorszenia</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="37" t="n">
+      <x:c r="A9" s="39" t="n">
         <x:v>46251.5</x:v>
       </x:c>
-      <x:c r="B9" s="37" t="n">
+      <x:c r="B9" s="39" t="n">
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="C9" s="12" t="n">
@@ -5323,22 +5875,22 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="F9" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A9,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B9,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A9,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B9,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>22</x:v>
       </x:c>
       <x:c r="G9" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A9,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B9,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A9,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B9,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>24</x:v>
       </x:c>
-      <x:c r="H9" s="38" t="str">
+      <x:c r="H9" s="40" t="str">
         <x:v>22.08 zależne od 15.08</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="37" t="n">
+      <x:c r="A10" s="39" t="n">
         <x:v>46258.5</x:v>
       </x:c>
-      <x:c r="B10" s="37" t="n">
+      <x:c r="B10" s="39" t="n">
         <x:v>46264.5</x:v>
       </x:c>
       <x:c r="C10" s="12" t="n">
@@ -5354,22 +5906,22 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="F10" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A10,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B10,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A10,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B10,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>16</x:v>
       </x:c>
       <x:c r="G10" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A10,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B10,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A10,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B10,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>16</x:v>
       </x:c>
-      <x:c r="H10" s="38" t="str">
+      <x:c r="H10" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="37" t="n">
+      <x:c r="A11" s="39" t="n">
         <x:v>46265.5</x:v>
       </x:c>
-      <x:c r="B11" s="37" t="n">
+      <x:c r="B11" s="39" t="n">
         <x:v>46271.5</x:v>
       </x:c>
       <x:c r="C11" s="12" t="n">
@@ -5385,22 +5937,22 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="F11" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A11,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B11,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A11,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B11,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="G11" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A11,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B11,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A11,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B11,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="H11" s="38" t="str">
+      <x:c r="H11" s="40" t="str">
         <x:v>01.09 test; 02.09 decyzja A/B/C</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="37" t="n">
+      <x:c r="A12" s="39" t="n">
         <x:v>46272.5</x:v>
       </x:c>
-      <x:c r="B12" s="37" t="n">
+      <x:c r="B12" s="39" t="n">
         <x:v>46278.5</x:v>
       </x:c>
       <x:c r="C12" s="12" t="n">
@@ -5416,14 +5968,14 @@
         <x:v>51.195</x:v>
       </x:c>
       <x:c r="F12" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A12,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B12,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$H$2:$H$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A12,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B12,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G12" s="12" t="n">
-        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A12,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B12,'FAZA 1 - OSLO V2'!$U$2:$U$81,1)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H12" s="38" t="str">
+        <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A12,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B12,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H12" s="40" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
@@ -5446,24 +5998,24 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="33" t="str">
+      <x:c r="A1" s="35" t="str">
         <x:v>STRATEGIA STARTOWA — decyzja 02.09.2026</x:v>
       </x:c>
-      <x:c r="B1" s="33"/>
-      <x:c r="C1" s="33"/>
-      <x:c r="D1" s="33"/>
+      <x:c r="B1" s="35"/>
+      <x:c r="C1" s="35"/>
+      <x:c r="D1" s="35"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="36" t="str">
+      <x:c r="A3" s="38" t="str">
         <x:v>Wariant</x:v>
       </x:c>
-      <x:c r="B3" s="36" t="str">
+      <x:c r="B3" s="38" t="str">
         <x:v>Cel</x:v>
       </x:c>
-      <x:c r="C3" s="36" t="str">
+      <x:c r="C3" s="38" t="str">
         <x:v>Tempo</x:v>
       </x:c>
-      <x:c r="D3" s="36" t="str">
+      <x:c r="D3" s="38" t="str">
         <x:v>Warunek</x:v>
       </x:c>
     </x:row>
@@ -5510,12 +6062,12 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="41" t="str">
+      <x:c r="A8" s="43" t="str">
         <x:v>Plan A 3:30 pozostaje wyłącznie po zaliczeniu wszystkich bramek: 15.08, 22.08 i 01.09. Ostateczna decyzja: 02.09.</x:v>
       </x:c>
-      <x:c r="B8" s="41"/>
-      <x:c r="C8" s="41"/>
-      <x:c r="D8" s="41"/>
+      <x:c r="B8" s="43"/>
+      <x:c r="C8" s="43"/>
+      <x:c r="D8" s="43"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
fix: recalibrate Oslo V2 paces from 40:08
</commit_message>
<xml_diff>
--- a/source_plan_v2.xlsx
+++ b/source_plan_v2.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAZA 1 - OSLO V2" sheetId="1" r:id="Rce6f739af7a5444c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TYGODNIE I BRAMKI" sheetId="2" r:id="R0aa656e5b50f4164"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STRATEGIA STARTOWA" sheetId="3" r:id="R0b51aa4b9f9443c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAZA 1 - OSLO V2" sheetId="1" r:id="R0b13e69ed383463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TYGODNIE I BRAMKI" sheetId="2" r:id="R0b06c961b0c240c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STRATEGIA STARTOWA" sheetId="3" r:id="R3eefde276ceb413e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -722,10 +722,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L4" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+        <x:v>5:30–6:05/km • 5:10–5:45/km • 5:35–6:15/km • odcinki wysiłkowo</x:v>
       </x:c>
       <x:c r="M4" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 5 km easy 5:50–6:25/km, RPE 3–4 + 6 × 20 s rytmu technicznego, RPE 7–8, bez targetu tempa. Przerwy: 90 s pełnego truchtu lub marszu, target otwarty. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Rytmy wykonuj luźno i technicznie; Garmin bez alarmu tempa. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna: 5 km easy 5:10–5:45/km, RPE 3–4 + 6 × 20 s rytmu technicznego, RPE 7–8, bez targetu tempa. Przerwy: 90 s pełnego truchtu lub marszu, target otwarty. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Rytmy wykonuj luźno i technicznie; Garmin bez alarmu tempa. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N4" s="30" t="str">
         <x:v>3–4</x:v>
@@ -750,12 +750,12 @@
         <x:v>cc-v2-oslo-2026-2026-07-16-run-1</x:v>
       </x:c>
       <x:c r="V4" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Easy 5km 5:50/km-6:25/km Pace
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Easy 5km 5:10/km-5:45/km Pace
 Strides 6x
 - Fast relaxed 20s 7-8 RPE
 - Full recovery 90s open
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W4" s="24" t="n">
         <x:v>0</x:v>
@@ -908,10 +908,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L7" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:15–5:50/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M7" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 10 km easy 5:50–6:25/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna: 10 km easy 5:15–5:50/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N7" s="30" t="str">
         <x:v>3–4</x:v>
@@ -938,9 +938,9 @@
         <x:v>cc-v2-oslo-2026-2026-07-18-run-1</x:v>
       </x:c>
       <x:c r="V7" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Long easy 10km 5:50/km-6:25/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Long easy 10km 5:15/km-5:50/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W7" s="24" t="n">
         <x:v>1</x:v>
@@ -979,10 +979,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L8" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M8" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Recovery: 3 km 5:40–6:20/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem. Przy zmęczeniu nie przyspieszaj: pozostań w zakresie, a RPE ma pierwszeństwo.</x:v>
       </x:c>
       <x:c r="N8" s="30" t="str">
         <x:v>2–3</x:v>
@@ -1007,9 +1007,9 @@
         <x:v>cc-v2-oslo-2026-2026-07-19-run-1</x:v>
       </x:c>
       <x:c r="V8" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Recovery 3km 6:15/km-6:45/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Recovery 3km 5:40/km-6:20/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W8" s="24" t="n">
         <x:v>0</x:v>
@@ -1162,10 +1162,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L11" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 4:58–5:05/km • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 4:12–4:20/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M11" s="30" t="str">
-        <x:v>Rozgrzewka: 2 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 3 × 1 km 4:58–5:05/km, RPE 7, na płaskim. Przerwy: 2 min truchtu 6:15–6:45/km, RPE 2–3. Schłodzenie: 2 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 2 km 5:30–6:05/km, RPE 2–3. Część główna: 3 × 1 km 4:12–4:20/km, RPE 7, na płaskim. Przerwy: 2 min truchtu 5:40–6:20/km, RPE 2–3. Schłodzenie: 2 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N11" s="30" t="str">
         <x:v>7</x:v>
@@ -1190,11 +1190,11 @@
         <x:v>cc-v2-oslo-2026-2026-07-21-run-1</x:v>
       </x:c>
       <x:c r="V11" s="30" t="str">
-        <x:v>- Warmup 2km 6:00/km-6:30/km Pace
+        <x:v>- Warmup 2km 5:30/km-6:05/km Pace
 Threshold 3x
-- Threshold 1km 4:58/km-5:05/km Pace
-- Recovery 2m 6:15/km-6:45/km Pace
-- Cooldown 2km 6:10/km-6:40/km Pace</x:v>
+- Threshold 1km 4:12/km-4:20/km Pace
+- Recovery 2m 5:40/km-6:20/km Pace
+- Cooldown 2km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W11" s="24" t="n">
         <x:v>0</x:v>
@@ -1351,10 +1351,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L14" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:45–6:15/km • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+        <x:v>5:30–6:05/km • 5:05–5:35/km • 5:35–6:15/km • odcinki wysiłkowo</x:v>
       </x:c>
       <x:c r="M14" s="30" t="str">
-        <x:v>Rozgrzewka: 2 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 7 km średnio-długiego easy 5:45–6:15/km, RPE 3–4 + 6 × 8 s hill sprint techniczny, nachylenie 4–6%, RPE 8, bez targetu tempa. Przerwy: 2 min pełnego marszu/truchtu w dół, target otwarty. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Podbieg wykonywany na wysiłek — nie kontroluj tempa chwilowego. Garmin bez alarmu tempa na hill sprintach.</x:v>
+        <x:v>Rozgrzewka: 2 km 5:30–6:05/km, RPE 2–3. Część główna: 7 km średnio-długiego easy 5:05–5:35/km, RPE 3–4 + 6 × 8 s hill sprint techniczny, nachylenie 4–6%, RPE 8, bez targetu tempa. Przerwy: 2 min pełnego marszu/truchtu w dół, target otwarty. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Podbieg wykonywany na wysiłek — nie kontroluj tempa chwilowego. Garmin bez alarmu tempa na hill sprintach.</x:v>
       </x:c>
       <x:c r="N14" s="30" t="str">
         <x:v>3–4</x:v>
@@ -1381,12 +1381,12 @@
         <x:v>cc-v2-oslo-2026-2026-07-23-run-1</x:v>
       </x:c>
       <x:c r="V14" s="30" t="str">
-        <x:v>- Warmup 2km 6:00/km-6:30/km Pace
-- Medium long easy 7km 5:45/km-6:15/km Pace
+        <x:v>- Warmup 2km 5:30/km-6:05/km Pace
+- Medium long easy 7km 5:05/km-5:35/km Pace
 Hill sprints 6x
 - Uphill fast relaxed 8s 8 RPE
 - Full walk-jog recovery 2m open
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W14" s="24" t="n">
         <x:v>0</x:v>
@@ -1478,10 +1478,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L16" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:15–5:50/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M16" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 10 km easy 5:50–6:25/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna: 10 km easy 5:15–5:50/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N16" s="30" t="str">
         <x:v>3–4</x:v>
@@ -1506,9 +1506,9 @@
         <x:v>cc-v2-oslo-2026-2026-07-25-run-1</x:v>
       </x:c>
       <x:c r="V16" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Long easy 10km 5:50/km-6:25/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Long easy 10km 5:15/km-5:50/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W16" s="24" t="n">
         <x:v>1</x:v>
@@ -1547,10 +1547,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L17" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M17" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Recovery: 3 km 5:40–6:20/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem. Przy zmęczeniu nie przyspieszaj: pozostań w zakresie, a RPE ma pierwszeństwo.</x:v>
       </x:c>
       <x:c r="N17" s="30" t="str">
         <x:v>2–3</x:v>
@@ -1575,9 +1575,9 @@
         <x:v>cc-v2-oslo-2026-2026-07-26-run-1</x:v>
       </x:c>
       <x:c r="V17" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Recovery 3km 6:15/km-6:45/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Recovery 3km 5:40/km-6:20/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W17" s="24" t="n">
         <x:v>0</x:v>
@@ -1730,10 +1730,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L20" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+        <x:v>5:30–6:05/km • 5:35–6:15/km • odcinki wysiłkowo</x:v>
       </x:c>
       <x:c r="M20" s="30" t="str">
-        <x:v>Rozgrzewka: 2.5 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 6 × 60 s pod górę, nachylenie 4–7%, RPE 7; bez targetu tempa. Przerwy: pełny trucht w dół 2.5 min, target otwarty, RPE 2–3. Schłodzenie: 2 km 6:10–6:40/km, RPE 2–3. Podbieg wykonywany na wysiłek — nie kontroluj tempa chwilowego.</x:v>
+        <x:v>Rozgrzewka: 2.5 km 5:30–6:05/km, RPE 2–3. Część główna: 6 × 60 s pod górę, nachylenie 4–7%, RPE 7; bez targetu tempa. Przerwy: pełny trucht w dół 2.5 min, target otwarty, RPE 2–3. Schłodzenie: 2 km 5:35–6:15/km, RPE 2–3. Podbieg wykonywany na wysiłek — nie kontroluj tempa chwilowego.</x:v>
       </x:c>
       <x:c r="N20" s="30" t="str">
         <x:v>7 na podbiegach</x:v>
@@ -1760,11 +1760,11 @@
         <x:v>cc-v2-oslo-2026-2026-07-28-run-1</x:v>
       </x:c>
       <x:c r="V20" s="30" t="str">
-        <x:v>- Warmup 2.5km 6:00/km-6:30/km Pace
+        <x:v>- Warmup 2.5km 5:30/km-6:05/km Pace
 Uphill effort 6x
 - Uphill 60s 7 RPE
 - Full jog-down recovery 150s open
-- Cooldown 2km 6:10/km-6:40/km Pace</x:v>
+- Cooldown 2km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W20" s="24" t="n">
         <x:v>0</x:v>
@@ -1921,10 +1921,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L23" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:45–6:15/km • 5:20–5:35/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:05–5:35/km • 4:40–4:55/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M23" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 6 km średnio-długiego easy 5:45–6:15/km, RPE 3–4 + 3 km steady 5:20–5:35/km, RPE 5–6. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna: 6 km średnio-długiego easy 5:05–5:35/km, RPE 3–4 + 3 km steady 4:40–4:55/km, RPE 5–6. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N23" s="30" t="str">
         <x:v>3–5</x:v>
@@ -1949,10 +1949,10 @@
         <x:v>cc-v2-oslo-2026-2026-07-30-run-1</x:v>
       </x:c>
       <x:c r="V23" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Medium long easy 6km 5:45/km-6:15/km Pace
-- Steady 3km 5:20/km-5:35/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Medium long easy 6km 5:05/km-5:35/km Pace
+- Steady 3km 4:40/km-4:55/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W23" s="24" t="n">
         <x:v>0</x:v>
@@ -2044,10 +2044,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L25" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:15–5:50/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M25" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 12 km easy 5:50–6:25/km na płaskich fragmentach; na podbiegach według wysiłku, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna: 12 km easy 5:15–5:50/km na płaskich fragmentach; na podbiegach według wysiłku, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N25" s="30" t="str">
         <x:v>3–5</x:v>
@@ -2074,9 +2074,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-01-run-1</x:v>
       </x:c>
       <x:c r="V25" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Long easy 12km 5:50/km-6:25/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Long easy 12km 5:15/km-5:50/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W25" s="24" t="n">
         <x:v>1</x:v>
@@ -2115,10 +2115,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L26" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M26" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Recovery: 3 km 5:40–6:20/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem. Przy zmęczeniu nie przyspieszaj: pozostań w zakresie, a RPE ma pierwszeństwo.</x:v>
       </x:c>
       <x:c r="N26" s="30" t="str">
         <x:v>2–3</x:v>
@@ -2143,9 +2143,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-02-run-1</x:v>
       </x:c>
       <x:c r="V26" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Recovery 3km 6:15/km-6:45/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Recovery 3km 5:40/km-6:20/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W26" s="24" t="n">
         <x:v>0</x:v>
@@ -2298,10 +2298,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L29" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 4:58–5:05/km • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 4:12–4:20/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M29" s="30" t="str">
-        <x:v>Rozgrzewka: 2 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 4 × 1 km 4:58–5:05/km, RPE 7, na płaskim. Przerwy: 2 min truchtu 6:15–6:45/km, RPE 2–3. Schłodzenie: 2 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 2 km 5:30–6:05/km, RPE 2–3. Część główna: 4 × 1 km 4:12–4:20/km, RPE 7, na płaskim. Przerwy: 2 min truchtu 5:40–6:20/km, RPE 2–3. Schłodzenie: 2 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N29" s="30" t="str">
         <x:v>7</x:v>
@@ -2326,11 +2326,11 @@
         <x:v>cc-v2-oslo-2026-2026-08-04-run-1</x:v>
       </x:c>
       <x:c r="V29" s="30" t="str">
-        <x:v>- Warmup 2km 6:00/km-6:30/km Pace
+        <x:v>- Warmup 2km 5:30/km-6:05/km Pace
 Threshold 4x
-- Threshold 1km 4:58/km-5:05/km Pace
-- Recovery 2m 6:15/km-6:45/km Pace
-- Cooldown 2km 6:10/km-6:40/km Pace</x:v>
+- Threshold 1km 4:12/km-4:20/km Pace
+- Recovery 2m 5:40/km-6:20/km Pace
+- Cooldown 2km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W29" s="24" t="n">
         <x:v>0</x:v>
@@ -2487,10 +2487,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L32" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:45–6:15/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:05–5:35/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M32" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Średnio-długi easy: 8 km 5:45–6:15/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Średnio-długi easy: 8 km 5:05–5:35/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N32" s="30" t="str">
         <x:v>3–4</x:v>
@@ -2515,9 +2515,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-06-run-1</x:v>
       </x:c>
       <x:c r="V32" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Średnio-długi easy 8km 5:45/km-6:15/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Średnio-długi easy 8km 5:05/km-5:35/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W32" s="24" t="n">
         <x:v>0</x:v>
@@ -2609,10 +2609,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L34" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:15–5:50/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M34" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 10 km easy 5:50–6:25/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna: 10 km easy 5:15–5:50/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N34" s="30" t="str">
         <x:v>3–4</x:v>
@@ -2637,9 +2637,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-08-run-1</x:v>
       </x:c>
       <x:c r="V34" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Long easy 10km 5:50/km-6:25/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Long easy 10km 5:15/km-5:50/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W34" s="24" t="n">
         <x:v>1</x:v>
@@ -2678,10 +2678,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L35" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M35" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Recovery: 3 km 5:40–6:20/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem. Przy zmęczeniu nie przyspieszaj: pozostań w zakresie, a RPE ma pierwszeństwo.</x:v>
       </x:c>
       <x:c r="N35" s="30" t="str">
         <x:v>2–3</x:v>
@@ -2706,9 +2706,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-09-run-1</x:v>
       </x:c>
       <x:c r="V35" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Recovery 3km 6:15/km-6:45/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Recovery 3km 5:40/km-6:20/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W35" s="24" t="n">
         <x:v>0</x:v>
@@ -2861,10 +2861,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L38" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+        <x:v>5:30–6:05/km • 5:35–6:15/km • odcinki wysiłkowo</x:v>
       </x:c>
       <x:c r="M38" s="30" t="str">
-        <x:v>Rozgrzewka: 2.5 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 4 × 3 min pod górę, nachylenie 4–7%, RPE 7; bez targetu tempa. Przerwy: pełny trucht w dół 3 min, target otwarty, RPE 2–3. Schłodzenie: 2 km 6:10–6:40/km, RPE 2–3. Podbieg wykonywany na wysiłek — nie kontroluj tempa chwilowego.</x:v>
+        <x:v>Rozgrzewka: 2.5 km 5:30–6:05/km, RPE 2–3. Część główna: 4 × 3 min pod górę, nachylenie 4–7%, RPE 7; bez targetu tempa. Przerwy: pełny trucht w dół 3 min, target otwarty, RPE 2–3. Schłodzenie: 2 km 5:35–6:15/km, RPE 2–3. Podbieg wykonywany na wysiłek — nie kontroluj tempa chwilowego.</x:v>
       </x:c>
       <x:c r="N38" s="30" t="str">
         <x:v>7</x:v>
@@ -2891,11 +2891,11 @@
         <x:v>cc-v2-oslo-2026-2026-08-11-run-1</x:v>
       </x:c>
       <x:c r="V38" s="30" t="str">
-        <x:v>- Warmup 2.5km 6:00/km-6:30/km Pace
+        <x:v>- Warmup 2.5km 5:30/km-6:05/km Pace
 Uphill effort 4x
 - Uphill 180s 7 RPE
 - Full jog-down recovery 180s open
-- Cooldown 2km 6:10/km-6:40/km Pace</x:v>
+- Cooldown 2km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W38" s="24" t="n">
         <x:v>0</x:v>
@@ -2987,10 +2987,10 @@
         <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L40" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M40" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Recovery: 3 km 5:40–6:20/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem. Przy zmęczeniu nie przyspieszaj: pozostań w zakresie, a RPE ma pierwszeństwo.</x:v>
       </x:c>
       <x:c r="N40" s="30" t="str">
         <x:v>2–3</x:v>
@@ -3015,9 +3015,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-12-run-alt</x:v>
       </x:c>
       <x:c r="V40" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Recovery 3km 6:15/km-6:45/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Recovery 3km 5:40/km-6:20/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W40" s="24" t="n">
         <x:v>0</x:v>
@@ -3121,10 +3121,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L42" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:45–6:15/km • 5:20–5:35/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:05–5:35/km • 4:40–4:55/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M42" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 6 km średnio-długiego easy 5:45–6:15/km, RPE 3–4 + 3 km steady 5:20–5:35/km, RPE 5–6. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna: 6 km średnio-długiego easy 5:05–5:35/km, RPE 3–4 + 3 km steady 4:40–4:55/km, RPE 5–6. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N42" s="30" t="str">
         <x:v>3–5</x:v>
@@ -3149,10 +3149,10 @@
         <x:v>cc-v2-oslo-2026-2026-08-13-run-1</x:v>
       </x:c>
       <x:c r="V42" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Medium long easy 6km 5:45/km-6:15/km Pace
-- Steady 3km 5:20/km-5:35/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Medium long easy 6km 5:05/km-5:35/km Pace
+- Steady 3km 4:40/km-4:55/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W42" s="24" t="n">
         <x:v>0</x:v>
@@ -3244,10 +3244,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L44" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 4:58–5:03/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:15–5:50/km • 4:55–5:02/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M44" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3 w obu wariantach. Część główna — wariant 18 km: 16 km easy 5:50–6:25/km, RPE 3–4. Część główna — wariant 20 km tylko po spełnieniu bramki: 15 km easy 5:50–6:25/km + 3 km docelowego MP 3:30 4:58–5:03/km, RPE maks. 6. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3 w obu wariantach. Część główna — wariant 18 km: 16 km long easy 5:15–5:50/km, RPE 3–4. Część główna — wariant 20 km tylko po spełnieniu bramki: 15 km long easy 5:15–5:50/km + 3 km docelowego MP 3:30 4:55–5:02/km, RPE maks. 6. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N44" s="30" t="str">
         <x:v>easy ≤4</x:v>
@@ -3274,10 +3274,10 @@
         <x:v>cc-v2-oslo-2026-2026-08-15-run-1</x:v>
       </x:c>
       <x:c r="V44" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Easy 15km 5:50/km-6:25/km Pace
-- Conditional goal MP 3km 4:58/km-5:03/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Long easy 15km 5:15/km-5:50/km Pace
+- Conditional goal MP 3km 4:55/km-5:02/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W44" s="24" t="n">
         <x:v>1</x:v>
@@ -3316,10 +3316,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L45" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M45" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 2 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Recovery: 2 km 5:40–6:20/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem. Przy zmęczeniu nie przyspieszaj: pozostań w zakresie, a RPE ma pierwszeństwo.</x:v>
       </x:c>
       <x:c r="N45" s="30" t="str">
         <x:v>2</x:v>
@@ -3346,9 +3346,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-16-run-1</x:v>
       </x:c>
       <x:c r="V45" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Recovery 2km 6:15/km-6:45/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Recovery 2km 5:40/km-6:20/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W45" s="24" t="n">
         <x:v>0</x:v>
@@ -3501,10 +3501,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L48" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 4:58–5:05/km • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 4:12–4:20/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M48" s="30" t="str">
-        <x:v>Rozgrzewka: 1.5 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 3 × 2 km 4:58–5:05/km, RPE 7, na płaskim. Przerwy: 3 min truchtu 6:15–6:45/km, RPE 2–3. Schłodzenie: 1.5 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1.5 km 5:30–6:05/km, RPE 2–3. Część główna: 3 × 2 km 4:12–4:20/km, RPE 7, na płaskim. Przerwy: 3 min truchtu 5:40–6:20/km, RPE 2–3. Schłodzenie: 1.5 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N48" s="30" t="str">
         <x:v>7</x:v>
@@ -3529,11 +3529,11 @@
         <x:v>cc-v2-oslo-2026-2026-08-18-run-1</x:v>
       </x:c>
       <x:c r="V48" s="30" t="str">
-        <x:v>- Warmup 1.5km 6:00/km-6:30/km Pace
+        <x:v>- Warmup 1.5km 5:30/km-6:05/km Pace
 Threshold 3x
-- Threshold 2km 4:58/km-5:05/km Pace
-- Recovery 3m 6:15/km-6:45/km Pace
-- Cooldown 1.5km 6:10/km-6:40/km Pace</x:v>
+- Threshold 2km 4:12/km-4:20/km Pace
+- Recovery 3m 5:40/km-6:20/km Pace
+- Cooldown 1.5km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W48" s="24" t="n">
         <x:v>0</x:v>
@@ -3625,10 +3625,10 @@
         <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L50" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M50" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Recovery: 3 km 5:40–6:20/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem. Przy zmęczeniu nie przyspieszaj: pozostań w zakresie, a RPE ma pierwszeństwo.</x:v>
       </x:c>
       <x:c r="N50" s="30" t="str">
         <x:v>2–3</x:v>
@@ -3653,9 +3653,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-19-run-alt</x:v>
       </x:c>
       <x:c r="V50" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Recovery 3km 6:15/km-6:45/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Recovery 3km 5:40/km-6:20/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W50" s="24" t="n">
         <x:v>0</x:v>
@@ -3759,10 +3759,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L52" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:45–6:15/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:05–5:35/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M52" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Średnio-długi easy: 9 km 5:45–6:15/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Średnio-długi easy: 9 km 5:05–5:35/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N52" s="30" t="str">
         <x:v>3–4</x:v>
@@ -3787,9 +3787,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-20-run-1</x:v>
       </x:c>
       <x:c r="V52" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Średnio-długi easy 9km 5:45/km-6:15/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Średnio-długi easy 9km 5:05/km-5:35/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W52" s="24" t="n">
         <x:v>0</x:v>
@@ -3881,10 +3881,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L54" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 5:15–5:25/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:15–5:50/km • 4:40–4:55/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M54" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3 w każdym wariancie. Część główna — wariant 22 km easy: 20 km easy 5:50–6:25/km, RPE 3–4. Część główna — wariant 22 km z blokiem: 17 km easy 5:50–6:25/km + 3 km aktualnego wysiłku maratońskiego 5:15–5:25/km, RPE 5–6. Część główna — wariant 24 km po zaliczeniu 15.08: 19 km easy 5:50–6:25/km + 3 km aktualnego wysiłku maratońskiego 5:15–5:25/km. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3 w każdym wariancie. Część główna — wariant 22 km easy: 20 km long easy 5:15–5:50/km, RPE 3–4. Część główna — wariant 22 km z blokiem: 17 km long easy 5:15–5:50/km + 3 km steady 4:40–4:55/km, RPE 5–6. Część główna — wariant 24 km po zaliczeniu 15.08: 19 km long easy 5:15–5:50/km + 3 km steady 4:40–4:55/km, RPE 5–6. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N54" s="30" t="str">
         <x:v>3–5</x:v>
@@ -3893,10 +3893,10 @@
         <x:v>300</x:v>
       </x:c>
       <x:c r="P54" s="30" t="str">
-        <x:v>22 km easy. 24 km tylko po zaliczeniu 15.08. Jeśli bramka 15.08 niezaliczona: 22 km easy albo jeden blok 3 km przy aktualnym wysiłku maratońskim.</x:v>
+        <x:v>22 km long easy. 24 km tylko po zaliczeniu 15.08. Opcjonalny blok 3 km steady, bez zwiększania dystansu.</x:v>
       </x:c>
       <x:c r="Q54" s="30" t="str">
-        <x:v>22 km easy albo 19 km easy + jeden blok 3 km aktualnego wysiłku maratońskiego; bez docelowego MP.</x:v>
+        <x:v>22 km long easy albo 19 km long easy + jeden blok 3 km steady; bez docelowego MP.</x:v>
       </x:c>
       <x:c r="R54" s="30" t="str">
         <x:v>24 km tylko po zaliczeniu 15.08: ból 0–2/10, easy RPE ≤4, brak pogorszenia następnego ranka. Bez zaliczenia: maks. 22 km.</x:v>
@@ -3911,10 +3911,10 @@
         <x:v>cc-v2-oslo-2026-2026-08-22-run-1</x:v>
       </x:c>
       <x:c r="V54" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Long easy 19km 5:50/km-6:25/km Pace
-- Conditional current marathon effort 3km 5:15/km-5:25/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Long easy 19km 5:15/km-5:50/km Pace
+- Conditional steady 3km 4:40/km-4:55/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W54" s="24" t="n">
         <x:v>1</x:v>
@@ -3953,10 +3953,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L55" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M55" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Recovery: 3 km 5:40–6:20/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem. Przy zmęczeniu nie przyspieszaj: pozostań w zakresie, a RPE ma pierwszeństwo.</x:v>
       </x:c>
       <x:c r="N55" s="30" t="str">
         <x:v>2</x:v>
@@ -3981,9 +3981,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-23-run-1</x:v>
       </x:c>
       <x:c r="V55" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Recovery 3km 6:15/km-6:45/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Recovery 3km 5:40/km-6:20/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W55" s="24" t="n">
         <x:v>0</x:v>
@@ -4120,7 +4120,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F58" s="21" t="str">
-        <x:v>Aktualny wysiłek maratoński 6 km</x:v>
+        <x:v>Steady 6 km / warunkowo goal MP</x:v>
       </x:c>
       <x:c r="G58" s="21" t="str">
         <x:v>MARATHON_EFFORT</x:v>
@@ -4136,10 +4136,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L58" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:15–5:25/km • 4:58–5:03/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 4:40–4:55/km • 4:55–5:02/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M58" s="30" t="str">
-        <x:v>Rozgrzewka: 2 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 6 km aktualnego wysiłku maratońskiego 5:15–5:25/km, RPE 5–6. Docelowe MP 3:30 4:58–5:03/km, RPE maks. 6, wyłącznie po zaliczeniu obu bramek. Przerwy: nie dotyczy. Schłodzenie: 2 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 2 km 5:30–6:05/km, RPE 2–3. Część główna: 6 km steady 4:40–4:55/km, RPE 5–6. Wariant warunkowy po zaliczeniu obu bramek: 6 km docelowego MP 3:30 4:55–5:02/km, RPE maks. 6, zamiast steady. Przerwy: nie dotyczy. Schłodzenie: 2 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N58" s="30" t="str">
         <x:v>5–6</x:v>
@@ -4148,13 +4148,13 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="P58" s="30" t="str">
-        <x:v>6 km przy aktualnym wysiłku maratońskim</x:v>
+        <x:v>6 km steady; po zaliczeniu bramek opcjonalnie 6 km goal MP zamiast steady</x:v>
       </x:c>
       <x:c r="Q58" s="30" t="str">
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
       <x:c r="R58" s="30" t="str">
-        <x:v>Docelowe MP 4:58/km wolno testować tylko po zaliczeniu bramek 15.08 i 22.08; bez ścigania.</x:v>
+        <x:v>Goal MP 4:55–5:02/km wolno wykonać tylko po zaliczeniu bramek 15.08 i 22.08; ból 0–2/10, RPE maks. 6 i bez pogorszenia następnego ranka.</x:v>
       </x:c>
       <x:c r="S58" s="30" t="str">
         <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
@@ -4166,9 +4166,10 @@
         <x:v>cc-v2-oslo-2026-2026-08-25-run-1</x:v>
       </x:c>
       <x:c r="V58" s="30" t="str">
-        <x:v>- Warmup 2km 6:00/km-6:30/km Pace
-- Current marathon effort 6km 5:15/km-5:25/km Pace
-- Cooldown 2km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 2km 5:30/km-6:05/km Pace
+- Steady 6km 4:40/km-4:55/km Pace
+- Conditional goal MP instead 6km 4:55/km-5:02/km Pace
+- Cooldown 2km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W58" s="24" t="n">
         <x:v>0</x:v>
@@ -4260,10 +4261,10 @@
         <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L60" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M60" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Recovery: 3 km 5:40–6:20/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem. Przy zmęczeniu nie przyspieszaj: pozostań w zakresie, a RPE ma pierwszeństwo.</x:v>
       </x:c>
       <x:c r="N60" s="30" t="str">
         <x:v>2–3</x:v>
@@ -4288,9 +4289,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-26-run-alt</x:v>
       </x:c>
       <x:c r="V60" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Recovery 3km 6:15/km-6:45/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Recovery 3km 5:40/km-6:20/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W60" s="24" t="n">
         <x:v>0</x:v>
@@ -4394,10 +4395,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L62" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:45–6:15/km • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+        <x:v>5:30–6:05/km • 5:05–5:35/km • 5:35–6:15/km • odcinki wysiłkowo</x:v>
       </x:c>
       <x:c r="M62" s="30" t="str">
-        <x:v>Rozgrzewka: 2 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 7 km średnio-długiego easy 5:45–6:15/km, RPE 3–4 + 6 × 10 s hill sprint techniczny, nachylenie 4–6%, RPE 8, bez targetu tempa. Przerwy: 2 min pełnego marszu/truchtu w dół, target otwarty. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Podbieg wykonywany na wysiłek — nie kontroluj tempa chwilowego. Garmin bez alarmu tempa na hill sprintach.</x:v>
+        <x:v>Rozgrzewka: 2 km 5:30–6:05/km, RPE 2–3. Część główna: 7 km średnio-długiego easy 5:05–5:35/km, RPE 3–4 + 6 × 10 s hill sprint techniczny, nachylenie 4–6%, RPE 8, bez targetu tempa. Przerwy: 2 min pełnego marszu/truchtu w dół, target otwarty. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Podbieg wykonywany na wysiłek — nie kontroluj tempa chwilowego. Garmin bez alarmu tempa na hill sprintach.</x:v>
       </x:c>
       <x:c r="N62" s="30" t="str">
         <x:v>3–4</x:v>
@@ -4424,12 +4425,12 @@
         <x:v>cc-v2-oslo-2026-2026-08-27-run-1</x:v>
       </x:c>
       <x:c r="V62" s="30" t="str">
-        <x:v>- Warmup 2km 6:00/km-6:30/km Pace
-- Medium long easy 7km 5:45/km-6:15/km Pace
+        <x:v>- Warmup 2km 5:30/km-6:05/km Pace
+- Medium long easy 7km 5:05/km-5:35/km Pace
 Hill sprints 6x
 - Uphill fast relaxed 10s 8 RPE
 - Full walk-jog recovery 2m open
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W62" s="24" t="n">
         <x:v>0</x:v>
@@ -4521,10 +4522,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L64" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:15–5:50/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M64" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 14 km easy 5:50–6:25/km na płaskich fragmentach; na podbiegach według wysiłku, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna: 14 km easy 5:15–5:50/km na płaskich fragmentach; na podbiegach według wysiłku, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N64" s="30" t="str">
         <x:v>3–5</x:v>
@@ -4549,9 +4550,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-29-run-1</x:v>
       </x:c>
       <x:c r="V64" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Long easy 14km 5:50/km-6:25/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Long easy 14km 5:15/km-5:50/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W64" s="24" t="n">
         <x:v>1</x:v>
@@ -4590,10 +4591,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L65" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M65" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 3 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Recovery: 3 km 5:40–6:20/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem. Przy zmęczeniu nie przyspieszaj: pozostań w zakresie, a RPE ma pierwszeństwo.</x:v>
       </x:c>
       <x:c r="N65" s="30" t="str">
         <x:v>2–3</x:v>
@@ -4618,9 +4619,9 @@
         <x:v>cc-v2-oslo-2026-2026-08-30-run-1</x:v>
       </x:c>
       <x:c r="V65" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Recovery 3km 6:15/km-6:45/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Recovery 3km 5:40/km-6:20/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W65" s="24" t="n">
         <x:v>0</x:v>
@@ -4773,10 +4774,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L68" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:15–5:25/km • 4:58–5:03/km • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 4:55–5:02/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M68" s="30" t="str">
-        <x:v>Rozgrzewka: 2 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 3 × 2 km — wariant A 4:58–5:03/km, RPE maks. 6 wyłącznie po zaliczeniu bramek; wariant B 5:16–5:20/km; wariant C 5:24–5:34/km. Przerwy: 500 m truchtu 6:15–6:45/km, RPE 2–3. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Wszystkie targety dotyczą płaskiego terenu.</x:v>
+        <x:v>Rozgrzewka: 2 km 5:30–6:05/km, RPE 2–3. Część główna: 3 × 2 km — wariant A 4:55–5:02/km, RPE maks. 6 wyłącznie po zaliczeniu bramek; wariant B 5:16–5:20/km; wariant C 5:24–5:34/km. Przerwy: 500 m truchtu 5:40–6:20/km, RPE 2–3. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Wszystkie targety dotyczą płaskiego terenu.</x:v>
       </x:c>
       <x:c r="N68" s="30" t="str">
         <x:v>5–6</x:v>
@@ -4791,7 +4792,7 @@
         <x:v>Ból ≥3/10, narastanie bólu lub zmiana kroku: przerwij bieg i zastąp go odpoczynkiem lub lekkim rowerem.</x:v>
       </x:c>
       <x:c r="R68" s="30" t="str">
-        <x:v>Nie wymuszaj 4:58/km. Zapisz RPE, ból i reakcję następnego ranka do decyzji 02.09.</x:v>
+        <x:v>Goal MP 4:55–5:02/km wykonuj wyłącznie po zaliczeniu wcześniejszych bramek. Zapisz RPE, ból i reakcję następnego ranka do decyzji 02.09; przy niespełnieniu warunków wybierz Plan B.</x:v>
       </x:c>
       <x:c r="S68" s="30" t="str">
         <x:v>Normalny posiłek i nawodnienie; po treningu białko oraz węglowodany.</x:v>
@@ -4803,11 +4804,11 @@
         <x:v>cc-v2-oslo-2026-2026-09-01-run-1</x:v>
       </x:c>
       <x:c r="V68" s="30" t="str">
-        <x:v>- Warmup 2km 6:00/km-6:30/km Pace
-Race pace calibration 3x
-- Controlled marathon pace 2km 5:15/km-5:25/km Pace
-- Recovery 500m 6:15/km-6:45/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 2km 5:30/km-6:05/km Pace
+Conditional goal MP calibration 3x
+- Goal MP 2km 4:55/km-5:02/km Pace
+- Recovery 500m 5:40/km-6:20/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W68" s="24" t="n">
         <x:v>0</x:v>
@@ -4968,10 +4969,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L71" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+        <x:v>5:30–6:05/km • 5:10–5:45/km • 5:35–6:15/km • odcinki wysiłkowo</x:v>
       </x:c>
       <x:c r="M71" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 6 km easy 5:50–6:25/km, RPE 3–4 + 4 × 15 s rytmu technicznego, RPE 7–8, bez targetu tempa. Przerwy: 90 s pełnego truchtu lub marszu, target otwarty. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Rytmy wykonuj luźno i technicznie; Garmin bez alarmu tempa. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna: 6 km easy 5:10–5:45/km, RPE 3–4 + 4 × 15 s rytmu technicznego, RPE 7–8, bez targetu tempa. Przerwy: 90 s pełnego truchtu lub marszu, target otwarty. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Rytmy wykonuj luźno i technicznie; Garmin bez alarmu tempa. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N71" s="30" t="str">
         <x:v>3</x:v>
@@ -4996,12 +4997,12 @@
         <x:v>cc-v2-oslo-2026-2026-09-03-run-1</x:v>
       </x:c>
       <x:c r="V71" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Easy 6km 5:50/km-6:25/km Pace
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Easy 6km 5:10/km-5:45/km Pace
 Strides 4x
 - Fast relaxed 15s 7-8 RPE
 - Full recovery 90s open
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W71" s="24" t="n">
         <x:v>0</x:v>
@@ -5093,10 +5094,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L73" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:15–5:50/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M73" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 6 km easy 5:50–6:25/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna: 6 km easy 5:15–5:50/km, RPE 3–4. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N73" s="30" t="str">
         <x:v>3</x:v>
@@ -5121,9 +5122,9 @@
         <x:v>cc-v2-oslo-2026-2026-09-05-run-1</x:v>
       </x:c>
       <x:c r="V73" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Long easy 6km 5:50/km-6:25/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Long easy 6km 5:15/km-5:50/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W73" s="24" t="n">
         <x:v>1</x:v>
@@ -5162,10 +5163,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L74" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 6:15–6:45/km • 6:10–6:40/km</x:v>
+        <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
       </x:c>
       <x:c r="M74" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna — Recovery: 2 km 6:15–6:45/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna — Recovery: 2 km 5:40–6:20/km, RPE 2–3. Przerwy: nie dotyczy. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem. Przy zmęczeniu nie przyspieszaj: pozostań w zakresie, a RPE ma pierwszeństwo.</x:v>
       </x:c>
       <x:c r="N74" s="30" t="str">
         <x:v>2</x:v>
@@ -5190,9 +5191,9 @@
         <x:v>cc-v2-oslo-2026-2026-09-06-run-1</x:v>
       </x:c>
       <x:c r="V74" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Recovery 2km 6:15/km-6:45/km Pace
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Recovery 2km 5:40/km-6:20/km Pace
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W74" s="24" t="n">
         <x:v>0</x:v>
@@ -5284,10 +5285,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L76" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+        <x:v>5:30–6:05/km • 5:10–5:45/km • 5:35–6:15/km • odcinki wysiłkowo</x:v>
       </x:c>
       <x:c r="M76" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 3 km easy 5:50–6:25/km, RPE 3–4 + 4 × 15 s rytmu technicznego, RPE 7–8, bez targetu tempa. Przerwy: 90 s pełnego truchtu lub marszu, target otwarty. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Rytmy wykonuj luźno i technicznie; Garmin bez alarmu tempa. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna: 3 km easy 5:10–5:45/km, RPE 3–4 + 4 × 15 s rytmu technicznego, RPE 7–8, bez targetu tempa. Przerwy: 90 s pełnego truchtu lub marszu, target otwarty. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Rytmy wykonuj luźno i technicznie; Garmin bez alarmu tempa. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N76" s="30" t="str">
         <x:v>2–3</x:v>
@@ -5312,12 +5313,12 @@
         <x:v>cc-v2-oslo-2026-2026-09-08-run-1</x:v>
       </x:c>
       <x:c r="V76" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Easy 3km 5:50/km-6:25/km Pace
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Easy 3km 5:10/km-5:45/km Pace
 Strides 4x
 - Fast relaxed 15s 7-8 RPE
 - Full recovery 90s open
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W76" s="24" t="n">
         <x:v>0</x:v>
@@ -5474,10 +5475,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L79" s="21" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 5:50–6:25/km • 6:10–6:40/km • odcinki wysiłkowo</x:v>
+        <x:v>5:30–6:05/km • 5:10–5:45/km • 5:35–6:15/km • odcinki wysiłkowo</x:v>
       </x:c>
       <x:c r="M79" s="30" t="str">
-        <x:v>Rozgrzewka: 1 km 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: 2 km easy 5:50–6:25/km, RPE 3–4 + 3 × 10 s rytmu technicznego, RPE 7–8, bez targetu tempa. Przerwy: 90 s pełnego truchtu lub marszu, target otwarty. Schłodzenie: 1 km 6:10–6:40/km, RPE 2–3. Rytmy wykonuj luźno i technicznie; Garmin bez alarmu tempa. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu; na podbiegach utrzymuj wskazane RPE.</x:v>
+        <x:v>Rozgrzewka: 1 km 5:30–6:05/km, RPE 2–3. Część główna: 2 km easy 5:10–5:45/km, RPE 3–4 + 3 × 10 s rytmu technicznego, RPE 7–8, bez targetu tempa. Przerwy: 90 s pełnego truchtu lub marszu, target otwarty. Schłodzenie: 1 km 5:35–6:15/km, RPE 2–3. Rytmy wykonuj luźno i technicznie; Garmin bez alarmu tempa. Zakresy tempa dotyczą płaskiego lub łagodnie pofałdowanego terenu. Na pagórkach, w upale i przy wietrze RPE ma pierwszeństwo przed tempem.</x:v>
       </x:c>
       <x:c r="N79" s="30" t="str">
         <x:v>2–3</x:v>
@@ -5502,12 +5503,12 @@
         <x:v>cc-v2-oslo-2026-2026-09-10-run-1</x:v>
       </x:c>
       <x:c r="V79" s="30" t="str">
-        <x:v>- Warmup 1km 6:00/km-6:30/km Pace
-- Easy 2km 5:50/km-6:25/km Pace
+        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+- Easy 2km 5:10/km-5:45/km Pace
 Strides 3x
 - Fast relaxed 10s 7-8 RPE
 - Full recovery 90s open
-- Cooldown 1km 6:10/km-6:40/km Pace</x:v>
+- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W79" s="24" t="n">
         <x:v>0</x:v>
@@ -5601,10 +5602,10 @@
         <x:v>ŁATWY</x:v>
       </x:c>
       <x:c r="L81" s="26" t="str">
-        <x:v>6:00–6:30/km albo wolniej • 4:58–5:03/km</x:v>
+        <x:v>5:30–6:05/km • 4:55–5:02/km</x:v>
       </x:c>
       <x:c r="M81" s="32" t="str">
-        <x:v>Rozgrzewka: 10–15 min bardzo lekko, 6:00–6:30/km albo wolniej, RPE 2–3. Część główna: Plan A 3:30 — 4:58–5:03/km, RPE początkowo 5–6, tylko po wszystkich bramkach; Plan B 5:16–5:20/km; Plan C 5:24–5:34/km. Przerwy: brak; punkty żywieniowe pokonuj według sytuacji. Schłodzenie: 10–15 min marszu lub truchtu, target otwarty, RPE 1–2. Tempo dotyczy płaskich fragmentów; na podbiegach utrzymuj wysiłek.</x:v>
+        <x:v>Rozgrzewka: 10–15 min bardzo lekko, 5:30–6:05/km, RPE 2–3. Część główna: Plan A 3:30 — 4:55–5:02/km, RPE początkowo 5–6, tylko po wszystkich bramkach; Plan B 5:16–5:20/km; Plan C 5:24–5:34/km. Przerwy: brak; punkty żywieniowe pokonuj według sytuacji. Schłodzenie: 10–15 min marszu lub truchtu, target otwarty, RPE 1–2. Tempo dotyczy płaskich fragmentów; na podbiegach utrzymuj wysiłek.</x:v>
       </x:c>
       <x:c r="N81" s="32" t="str">
         <x:v>start 5–6, progres wg stanu</x:v>
@@ -5631,8 +5632,8 @@
         <x:v>cc-v2-oslo-2026-2026-09-12-run-1</x:v>
       </x:c>
       <x:c r="V81" s="32" t="str">
-        <x:v>- Race controlled start 5km 5:00/km-5:05/km Pace
-- Race strategy block 32.195km 5:15/km-5:25/km Pace
+        <x:v>- Race controlled start 5km 4:58/km-5:02/km Pace
+- Race strategy block 32.195km 4:55/km-5:02/km Pace
 - Finish by feel 5km 5-8 RPE</x:v>
       </x:c>
       <x:c r="W81" s="29" t="n">
@@ -6027,7 +6028,7 @@
         <x:v>3:30</x:v>
       </x:c>
       <x:c r="C4" s="11" t="str">
-        <x:v>4:58/km</x:v>
+        <x:v>4:55–5:02/km</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
         <x:v>Wyłącznie po zaliczeniu bramek 15.08, 22.08 i 01.09; decyzja 02.09.</x:v>

</xml_diff>

<commit_message>
fix: align Oslo V2 workout intensity metadata
</commit_message>
<xml_diff>
--- a/source_plan_v2.xlsx
+++ b/source_plan_v2.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAZA 1 - OSLO V2" sheetId="1" r:id="R0b13e69ed383463d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TYGODNIE I BRAMKI" sheetId="2" r:id="R0b06c961b0c240c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STRATEGIA STARTOWA" sheetId="3" r:id="R3eefde276ceb413e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAZA 1 - OSLO V2" sheetId="1" r:id="R-sheet1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TYGODNIE I BRAMKI" sheetId="2" r:id="R-sheet2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STRATEGIA STARTOWA" sheetId="3" r:id="R-sheet3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -976,7 +976,7 @@
       </x:c>
       <x:c r="J8" s="22"/>
       <x:c r="K8" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L8" s="21" t="str">
         <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
@@ -1159,7 +1159,7 @@
       </x:c>
       <x:c r="J11" s="22"/>
       <x:c r="K11" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>PROGOWY</x:v>
       </x:c>
       <x:c r="L11" s="21" t="str">
         <x:v>5:30–6:05/km • 4:12–4:20/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
@@ -1348,7 +1348,7 @@
       </x:c>
       <x:c r="J14" s="22"/>
       <x:c r="K14" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>SIŁA BIEGOWA</x:v>
       </x:c>
       <x:c r="L14" s="21" t="str">
         <x:v>5:30–6:05/km • 5:05–5:35/km • 5:35–6:15/km • odcinki wysiłkowo</x:v>
@@ -1544,7 +1544,7 @@
       </x:c>
       <x:c r="J17" s="22"/>
       <x:c r="K17" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L17" s="21" t="str">
         <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
@@ -1727,7 +1727,7 @@
       </x:c>
       <x:c r="J20" s="22"/>
       <x:c r="K20" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>PODBIEGI</x:v>
       </x:c>
       <x:c r="L20" s="21" t="str">
         <x:v>5:30–6:05/km • 5:35–6:15/km • odcinki wysiłkowo</x:v>
@@ -1918,7 +1918,7 @@
       </x:c>
       <x:c r="J23" s="22"/>
       <x:c r="K23" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>UMIARKOWANY</x:v>
       </x:c>
       <x:c r="L23" s="21" t="str">
         <x:v>5:30–6:05/km • 5:05–5:35/km • 4:40–4:55/km • 5:35–6:15/km</x:v>
@@ -2112,7 +2112,7 @@
       </x:c>
       <x:c r="J26" s="22"/>
       <x:c r="K26" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L26" s="21" t="str">
         <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
@@ -2295,7 +2295,7 @@
       </x:c>
       <x:c r="J29" s="22"/>
       <x:c r="K29" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>PROGOWY</x:v>
       </x:c>
       <x:c r="L29" s="21" t="str">
         <x:v>5:30–6:05/km • 4:12–4:20/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
@@ -2675,7 +2675,7 @@
       </x:c>
       <x:c r="J35" s="22"/>
       <x:c r="K35" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L35" s="21" t="str">
         <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
@@ -2858,7 +2858,7 @@
       </x:c>
       <x:c r="J38" s="22"/>
       <x:c r="K38" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>PODBIEGI</x:v>
       </x:c>
       <x:c r="L38" s="21" t="str">
         <x:v>5:30–6:05/km • 5:35–6:15/km • odcinki wysiłkowo</x:v>
@@ -3118,7 +3118,7 @@
       </x:c>
       <x:c r="J42" s="22"/>
       <x:c r="K42" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>UMIARKOWANY</x:v>
       </x:c>
       <x:c r="L42" s="21" t="str">
         <x:v>5:30–6:05/km • 5:05–5:35/km • 4:40–4:55/km • 5:35–6:15/km</x:v>
@@ -3241,7 +3241,7 @@
       </x:c>
       <x:c r="J44" s="22"/>
       <x:c r="K44" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>MARATOŃSKI</x:v>
       </x:c>
       <x:c r="L44" s="21" t="str">
         <x:v>5:30–6:05/km • 5:15–5:50/km • 4:55–5:02/km • 5:35–6:15/km</x:v>
@@ -3313,7 +3313,7 @@
       </x:c>
       <x:c r="J45" s="22"/>
       <x:c r="K45" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L45" s="21" t="str">
         <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
@@ -3498,7 +3498,7 @@
       </x:c>
       <x:c r="J48" s="22"/>
       <x:c r="K48" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>PROGOWY</x:v>
       </x:c>
       <x:c r="L48" s="21" t="str">
         <x:v>5:30–6:05/km • 4:12–4:20/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
@@ -3878,7 +3878,7 @@
       </x:c>
       <x:c r="J54" s="22"/>
       <x:c r="K54" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>UMIARKOWANY</x:v>
       </x:c>
       <x:c r="L54" s="21" t="str">
         <x:v>5:30–6:05/km • 5:15–5:50/km • 4:40–4:55/km • 5:35–6:15/km</x:v>
@@ -3950,7 +3950,7 @@
       </x:c>
       <x:c r="J55" s="22"/>
       <x:c r="K55" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L55" s="21" t="str">
         <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
@@ -4133,7 +4133,7 @@
       </x:c>
       <x:c r="J58" s="22"/>
       <x:c r="K58" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>MARATOŃSKI</x:v>
       </x:c>
       <x:c r="L58" s="21" t="str">
         <x:v>5:30–6:05/km • 4:40–4:55/km • 4:55–5:02/km • 5:35–6:15/km</x:v>
@@ -4392,7 +4392,7 @@
       </x:c>
       <x:c r="J62" s="22"/>
       <x:c r="K62" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>SIŁA BIEGOWA</x:v>
       </x:c>
       <x:c r="L62" s="21" t="str">
         <x:v>5:30–6:05/km • 5:05–5:35/km • 5:35–6:15/km • odcinki wysiłkowo</x:v>
@@ -4588,7 +4588,7 @@
       </x:c>
       <x:c r="J65" s="22"/>
       <x:c r="K65" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L65" s="21" t="str">
         <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
@@ -4771,7 +4771,7 @@
       </x:c>
       <x:c r="J68" s="22"/>
       <x:c r="K68" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>MARATOŃSKI</x:v>
       </x:c>
       <x:c r="L68" s="21" t="str">
         <x:v>5:30–6:05/km • 4:55–5:02/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
@@ -5160,7 +5160,7 @@
       </x:c>
       <x:c r="J74" s="22"/>
       <x:c r="K74" s="21" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>REGENERACJA</x:v>
       </x:c>
       <x:c r="L74" s="21" t="str">
         <x:v>5:30–6:05/km • 5:40–6:20/km • 5:35–6:15/km</x:v>
@@ -5599,7 +5599,7 @@
         <x:v>210</x:v>
       </x:c>
       <x:c r="K81" s="26" t="str">
-        <x:v>ŁATWY</x:v>
+        <x:v>MARATOŃSKI</x:v>
       </x:c>
       <x:c r="L81" s="26" t="str">
         <x:v>5:30–6:05/km • 4:55–5:02/km</x:v>

</xml_diff>

<commit_message>
fix: simplify workout descriptions
</commit_message>
<xml_diff>
--- a/source_plan_v2.xlsx
+++ b/source_plan_v2.xlsx
@@ -163,7 +163,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="44">
+  <x:cellXfs count="46">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -232,6 +232,12 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="202" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -498,6 +504,7 @@
     <x:col min="21" max="21" width="38" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="55" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="10" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="55" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -567,8 +574,11 @@
       <x:c r="V1" s="8" t="str">
         <x:v>Structured workout</x:v>
       </x:c>
-      <x:c r="W1" s="9" t="str">
+      <x:c r="W1" s="8" t="str">
         <x:v>Long</x:v>
+      </x:c>
+      <x:c r="X1" s="9" t="str">
+        <x:v>compactDescription</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -588,7 +598,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F2" s="21" t="str">
-        <x:v>WOLNE (alternatywa dla roweru)</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G2" s="21" t="str">
         <x:v>REST</x:v>
@@ -618,10 +628,19 @@
         <x:v>cc-v2-oslo-2026-2026-07-15-note-1</x:v>
       </x:c>
       <x:c r="V2" s="30" t="str">
-        <x:v>Pełne wolne</x:v>
-      </x:c>
-      <x:c r="W2" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 40 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
+      </x:c>
+      <x:c r="W2" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X2" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 40 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -641,7 +660,7 @@
         <x:v>Ride</x:v>
       </x:c>
       <x:c r="F3" s="21" t="str">
-        <x:v>ALT: rower Z2 albo pełne wolne</x:v>
+        <x:v>Rower Z2 — 40 min</x:v>
       </x:c>
       <x:c r="G3" s="21" t="str">
         <x:v>ENDURANCE</x:v>
@@ -683,10 +702,16 @@
         <x:v>cc-v2-oslo-2026-2026-07-15-ride-alt</x:v>
       </x:c>
       <x:c r="V3" s="30" t="str">
-        <x:v>- Easy spin 40m 55-70% 85-95rpm</x:v>
-      </x:c>
-      <x:c r="W3" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rower Z2 40m 3 RPE</x:v>
+      </x:c>
+      <x:c r="W3" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X3" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 40 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -706,7 +731,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F4" s="21" t="str">
-        <x:v>Easy + rytmy</x:v>
+        <x:v>Easy 7 km + rytmy</x:v>
       </x:c>
       <x:c r="G4" s="21" t="str">
         <x:v>EASY_STRIDES</x:v>
@@ -750,15 +775,21 @@
         <x:v>cc-v2-oslo-2026-2026-07-16-run-1</x:v>
       </x:c>
       <x:c r="V4" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Easy 5km 5:10/km-5:45/km Pace
-Strides 6x
-- Fast relaxed 20s 7-8 RPE
-- Full recovery 90s open
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W4" s="24" t="n">
-        <x:v>0</x:v>
+Rytm 6x
+- Rytm 20s 7–8 RPE
+- Trucht 90s open
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W4" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X4" s="34" t="str">
+        <x:v>Easy 7 km + rytmy
+Easy 5 km @ 5:10–5:45/km, RPE 3–4
+6 × Rytm 20 s, RPE 7–8
+Przerwa: 90 s easy</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -778,7 +809,7 @@
         <x:v>Strength</x:v>
       </x:c>
       <x:c r="F5" s="21" t="str">
-        <x:v>Siła techniczna — nauka ruchu</x:v>
+        <x:v>Siła — 12 min</x:v>
       </x:c>
       <x:c r="G5" s="21" t="str">
         <x:v>STRENGTH</x:v>
@@ -816,10 +847,23 @@
         <x:v>cc-v2-oslo-2026-2026-07-16-strength-1</x:v>
       </x:c>
       <x:c r="V5" s="30" t="str">
-        <x:v>- Technika i stabilizacja 12m 2-4 RPE</x:v>
-      </x:c>
-      <x:c r="W5" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Siła — 12 min
+- Split squat 1–2 serie
+- Wspięcia łydki 1–2 serie
+- Hip hinge 1–2 serie
+- Side plank 1–2 serie
+- RPE: 2–4</x:v>
+      </x:c>
+      <x:c r="W5" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X5" s="34" t="str">
+        <x:v>Siła — 12 min
+Split squat 1–2 serie
+Wspięcia łydki 1–2 serie
+Hip hinge 1–2 serie
+Side plank 1–2 serie
+RPE: 2–4</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -839,7 +883,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F6" s="21" t="str">
-        <x:v>WOLNE przed long runem</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G6" s="21" t="str">
         <x:v>REST</x:v>
@@ -869,10 +913,13 @@
         <x:v>cc-v2-oslo-2026-2026-07-17-note-1</x:v>
       </x:c>
       <x:c r="V6" s="30" t="str">
-        <x:v>WOLNE przed long runem</x:v>
-      </x:c>
-      <x:c r="W6" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W6" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X6" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -892,7 +939,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F7" s="21" t="str">
-        <x:v>Long easy 12 km</x:v>
+        <x:v>Long 12 km</x:v>
       </x:c>
       <x:c r="G7" s="21" t="str">
         <x:v>LONG_RUN</x:v>
@@ -938,12 +985,16 @@
         <x:v>cc-v2-oslo-2026-2026-07-18-run-1</x:v>
       </x:c>
       <x:c r="V7" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Long easy 10km 5:15/km-5:50/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W7" s="24" t="n">
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W7" s="21" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="X7" s="34" t="str">
+        <x:v>Long 12 km
+Long easy 10 km @ 5:15–5:50/km, RPE 3–4</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -963,7 +1014,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F8" s="21" t="str">
-        <x:v>Recovery run</x:v>
+        <x:v>Recovery 5 km</x:v>
       </x:c>
       <x:c r="G8" s="21" t="str">
         <x:v>RECOVERY</x:v>
@@ -1007,12 +1058,17 @@
         <x:v>cc-v2-oslo-2026-2026-07-19-run-1</x:v>
       </x:c>
       <x:c r="V8" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Recovery 3km 5:40/km-6:20/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W8" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W8" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X8" s="34" t="str">
+        <x:v>Recovery 5 km
+Tempo: 5:40–6:20/km
+RPE: 2–3</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1032,7 +1088,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F9" s="21" t="str">
-        <x:v>Regeneracja + opcjonalna siła techniczna</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G9" s="21" t="str">
         <x:v>REST</x:v>
@@ -1062,10 +1118,13 @@
         <x:v>cc-v2-oslo-2026-2026-07-20-note-1</x:v>
       </x:c>
       <x:c r="V9" s="30" t="str">
-        <x:v>Regeneracja</x:v>
-      </x:c>
-      <x:c r="W9" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W9" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X9" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1085,7 +1144,7 @@
         <x:v>Strength</x:v>
       </x:c>
       <x:c r="F10" s="21" t="str">
-        <x:v>Siła techniczna — minimalna objętość</x:v>
+        <x:v>Siła — 15 min</x:v>
       </x:c>
       <x:c r="G10" s="21" t="str">
         <x:v>STRENGTH</x:v>
@@ -1123,10 +1182,23 @@
         <x:v>cc-v2-oslo-2026-2026-07-20-strength-1</x:v>
       </x:c>
       <x:c r="V10" s="30" t="str">
-        <x:v>- Technika i stabilizacja 15m 2-4 RPE</x:v>
-      </x:c>
-      <x:c r="W10" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Siła — 15 min
+- Split squat 1–2 serie
+- Wspięcia łydki 1–2 serie
+- Hip hinge 1–2 serie
+- Side plank 1–2 serie
+- RPE: 2–4</x:v>
+      </x:c>
+      <x:c r="W10" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X10" s="34" t="str">
+        <x:v>Siła — 15 min
+Split squat 1–2 serie
+Wspięcia łydki 1–2 serie
+Hip hinge 1–2 serie
+Side plank 1–2 serie
+RPE: 2–4</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1146,7 +1218,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F11" s="21" t="str">
-        <x:v>Próg kontrolowany 3 × 1 km</x:v>
+        <x:v>Threshold 8 km</x:v>
       </x:c>
       <x:c r="G11" s="21" t="str">
         <x:v>THRESHOLD</x:v>
@@ -1190,14 +1262,23 @@
         <x:v>cc-v2-oslo-2026-2026-07-21-run-1</x:v>
       </x:c>
       <x:c r="V11" s="30" t="str">
-        <x:v>- Warmup 2km 5:30/km-6:05/km Pace
-Threshold 3x
-- Threshold 1km 4:12/km-4:20/km Pace
-- Recovery 2m 5:40/km-6:20/km Pace
-- Cooldown 2km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W11" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rozgrzewka 2km 5:30/km-6:05/km Pace
+Próg 3x
+- Próg 1km 4:12/km-4:20/km Pace
+- Trucht 2m 5:40/km-6:20/km Pace
+- Schłodzenie 2km 5:35/km-6:15/km Pace
+Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
+      </x:c>
+      <x:c r="W11" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X11" s="34" t="str">
+        <x:v>Threshold 8 km
+WU: 2 km @ 5:30–6:05/km
+3 × Próg 1 km @ 4:12–4:20/km, RPE 7
+Przerwa: 2 min @ 5:40–6:20/km
+CD: 2 km @ 5:35–6:15/km
+Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1217,7 +1298,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F12" s="21" t="str">
-        <x:v>WOLNE (alternatywa dla roweru)</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G12" s="21" t="str">
         <x:v>REST</x:v>
@@ -1247,10 +1328,19 @@
         <x:v>cc-v2-oslo-2026-2026-07-22-note-1</x:v>
       </x:c>
       <x:c r="V12" s="30" t="str">
-        <x:v>Pełne wolne</x:v>
-      </x:c>
-      <x:c r="W12" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 45 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
+      </x:c>
+      <x:c r="W12" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X12" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 45 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1270,7 +1360,7 @@
         <x:v>Ride</x:v>
       </x:c>
       <x:c r="F13" s="21" t="str">
-        <x:v>ALT: rower Z2 albo pełne wolne</x:v>
+        <x:v>Rower Z2 — 45 min</x:v>
       </x:c>
       <x:c r="G13" s="21" t="str">
         <x:v>ENDURANCE</x:v>
@@ -1312,10 +1402,16 @@
         <x:v>cc-v2-oslo-2026-2026-07-22-ride-alt</x:v>
       </x:c>
       <x:c r="V13" s="30" t="str">
-        <x:v>- Easy spin 45m 55-70% 85-95rpm</x:v>
-      </x:c>
-      <x:c r="W13" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rower Z2 45m 3 RPE</x:v>
+      </x:c>
+      <x:c r="W13" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X13" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 45 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1335,7 +1431,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F14" s="21" t="str">
-        <x:v>Średnio-długi easy + hill sprints</x:v>
+        <x:v>Easy 10 km + hill sprints</x:v>
       </x:c>
       <x:c r="G14" s="21" t="str">
         <x:v>MEDIUM_LONG</x:v>
@@ -1381,15 +1477,22 @@
         <x:v>cc-v2-oslo-2026-2026-07-23-run-1</x:v>
       </x:c>
       <x:c r="V14" s="30" t="str">
-        <x:v>- Warmup 2km 5:30/km-6:05/km Pace
-- Medium long easy 7km 5:05/km-5:35/km Pace
-Hill sprints 6x
-- Uphill fast relaxed 8s 8 RPE
-- Full walk-jog recovery 2m open
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W14" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rozgrzewka 2km 5:30/km-6:05/km Pace
+- Easy 7km 5:05/km-5:35/km Pace
+Podbieg 6x
+- Podbieg 8s 8 RPE
+- Powrót 120s open
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W14" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X14" s="34" t="str">
+        <x:v>Easy 10 km + hill sprints
+Easy 7 km @ 5:05–5:35/km, RPE 3–4
+6 × Podbieg 8 s, nachylenie 4–6%, RPE 8
+Powrót: 120 s trucht w dół
+Bez targetu tempa pod górę.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1409,7 +1512,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F15" s="21" t="str">
-        <x:v>WOLNE przed long runem</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G15" s="21" t="str">
         <x:v>REST</x:v>
@@ -1439,10 +1542,13 @@
         <x:v>cc-v2-oslo-2026-2026-07-24-note-1</x:v>
       </x:c>
       <x:c r="V15" s="30" t="str">
-        <x:v>WOLNE przed long runem</x:v>
-      </x:c>
-      <x:c r="W15" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W15" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X15" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1462,7 +1568,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F16" s="21" t="str">
-        <x:v>Long easy 12 km</x:v>
+        <x:v>Long 12 km</x:v>
       </x:c>
       <x:c r="G16" s="21" t="str">
         <x:v>LONG_RUN</x:v>
@@ -1506,12 +1612,16 @@
         <x:v>cc-v2-oslo-2026-2026-07-25-run-1</x:v>
       </x:c>
       <x:c r="V16" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Long easy 10km 5:15/km-5:50/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W16" s="24" t="n">
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W16" s="21" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="X16" s="34" t="str">
+        <x:v>Long 12 km
+Long easy 10 km @ 5:15–5:50/km, RPE 3–4</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1531,7 +1641,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F17" s="21" t="str">
-        <x:v>Recovery run</x:v>
+        <x:v>Recovery 5 km</x:v>
       </x:c>
       <x:c r="G17" s="21" t="str">
         <x:v>RECOVERY</x:v>
@@ -1575,12 +1685,17 @@
         <x:v>cc-v2-oslo-2026-2026-07-26-run-1</x:v>
       </x:c>
       <x:c r="V17" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Recovery 3km 5:40/km-6:20/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W17" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W17" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X17" s="34" t="str">
+        <x:v>Recovery 5 km
+Tempo: 5:40–6:20/km
+RPE: 2–3</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1600,7 +1715,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F18" s="21" t="str">
-        <x:v>Regeneracja + opcjonalna siła techniczna</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G18" s="21" t="str">
         <x:v>REST</x:v>
@@ -1630,10 +1745,13 @@
         <x:v>cc-v2-oslo-2026-2026-07-27-note-1</x:v>
       </x:c>
       <x:c r="V18" s="30" t="str">
-        <x:v>Regeneracja</x:v>
-      </x:c>
-      <x:c r="W18" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W18" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X18" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1653,7 +1771,7 @@
         <x:v>Strength</x:v>
       </x:c>
       <x:c r="F19" s="21" t="str">
-        <x:v>Siła techniczna — kontrola ekscentryczna</x:v>
+        <x:v>Siła — 18 min</x:v>
       </x:c>
       <x:c r="G19" s="21" t="str">
         <x:v>STRENGTH</x:v>
@@ -1691,10 +1809,23 @@
         <x:v>cc-v2-oslo-2026-2026-07-27-strength-1</x:v>
       </x:c>
       <x:c r="V19" s="30" t="str">
-        <x:v>- Technika i stabilizacja 18m 2-4 RPE</x:v>
-      </x:c>
-      <x:c r="W19" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Siła — 18 min
+- Split squat 1–2 serie
+- Wspięcia łydki 1–2 serie
+- Hip hinge 1–2 serie
+- Side plank 1–2 serie
+- RPE: 2–4</x:v>
+      </x:c>
+      <x:c r="W19" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X19" s="34" t="str">
+        <x:v>Siła — 18 min
+Split squat 1–2 serie
+Wspięcia łydki 1–2 serie
+Hip hinge 1–2 serie
+Side plank 1–2 serie
+RPE: 2–4</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1714,7 +1845,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F20" s="21" t="str">
-        <x:v>Długie podbiegi 6 × 60 s</x:v>
+        <x:v>Podbiegi 9 km</x:v>
       </x:c>
       <x:c r="G20" s="21" t="str">
         <x:v>HILLS</x:v>
@@ -1760,14 +1891,22 @@
         <x:v>cc-v2-oslo-2026-2026-07-28-run-1</x:v>
       </x:c>
       <x:c r="V20" s="30" t="str">
-        <x:v>- Warmup 2.5km 5:30/km-6:05/km Pace
-Uphill effort 6x
-- Uphill 60s 7 RPE
-- Full jog-down recovery 150s open
-- Cooldown 2km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W20" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rozgrzewka 2.5km 5:30/km-6:05/km Pace
+Podbieg 6x
+- Podbieg 60s 7 RPE
+- Powrót 150s open
+- Schłodzenie 2km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W20" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X20" s="34" t="str">
+        <x:v>Podbiegi 9 km
+WU: 2,5 km @ 5:30–6:05/km
+6 × Podbieg 60 s, nachylenie 4–7%, RPE 7
+Powrót: 150 s trucht w dół
+CD: 2 km @ 5:35–6:15/km
+Bez targetu tempa pod górę.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1787,7 +1926,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F21" s="21" t="str">
-        <x:v>WOLNE (alternatywa dla roweru)</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G21" s="21" t="str">
         <x:v>REST</x:v>
@@ -1817,10 +1956,19 @@
         <x:v>cc-v2-oslo-2026-2026-07-29-note-1</x:v>
       </x:c>
       <x:c r="V21" s="30" t="str">
-        <x:v>Pełne wolne</x:v>
-      </x:c>
-      <x:c r="W21" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 45 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
+      </x:c>
+      <x:c r="W21" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X21" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 45 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1840,7 +1988,7 @@
         <x:v>Ride</x:v>
       </x:c>
       <x:c r="F22" s="21" t="str">
-        <x:v>ALT: rower Z2 albo pełne wolne</x:v>
+        <x:v>Rower Z2 — 45 min</x:v>
       </x:c>
       <x:c r="G22" s="21" t="str">
         <x:v>ENDURANCE</x:v>
@@ -1882,10 +2030,16 @@
         <x:v>cc-v2-oslo-2026-2026-07-29-ride-alt</x:v>
       </x:c>
       <x:c r="V22" s="30" t="str">
-        <x:v>- Easy spin 45m 55-70% 85-95rpm</x:v>
-      </x:c>
-      <x:c r="W22" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rower Z2 45m 3 RPE</x:v>
+      </x:c>
+      <x:c r="W22" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X22" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 45 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1905,7 +2059,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F23" s="21" t="str">
-        <x:v>Średnio-długi easy/steady</x:v>
+        <x:v>Średnio-długi 11 km</x:v>
       </x:c>
       <x:c r="G23" s="21" t="str">
         <x:v>MEDIUM_LONG</x:v>
@@ -1949,13 +2103,20 @@
         <x:v>cc-v2-oslo-2026-2026-07-30-run-1</x:v>
       </x:c>
       <x:c r="V23" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
-- Medium long easy 6km 5:05/km-5:35/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
+- Easy 6km 5:05/km-5:35/km Pace
 - Steady 3km 4:40/km-4:55/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W23" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W23" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X23" s="34" t="str">
+        <x:v>Średnio-długi 11 km
+WU: 1 km @ 5:30–6:05/km
+Easy 6 km @ 5:05–5:35/km, RPE 3–4
+Steady 3 km @ 4:40–4:55/km, RPE 5–6
+CD: 1 km @ 5:35–6:15/km</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1975,7 +2136,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F24" s="21" t="str">
-        <x:v>WOLNE przed long runem</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G24" s="21" t="str">
         <x:v>REST</x:v>
@@ -2005,10 +2166,13 @@
         <x:v>cc-v2-oslo-2026-2026-07-31-note-1</x:v>
       </x:c>
       <x:c r="V24" s="30" t="str">
-        <x:v>WOLNE przed long runem</x:v>
-      </x:c>
-      <x:c r="W24" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W24" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X24" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2028,7 +2192,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F25" s="21" t="str">
-        <x:v>Long pofałdowany 14 km</x:v>
+        <x:v>Long 14 km</x:v>
       </x:c>
       <x:c r="G25" s="21" t="str">
         <x:v>LONG_RUN_HILLY</x:v>
@@ -2074,12 +2238,16 @@
         <x:v>cc-v2-oslo-2026-2026-08-01-run-1</x:v>
       </x:c>
       <x:c r="V25" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Long easy 12km 5:15/km-5:50/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W25" s="24" t="n">
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W25" s="21" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="X25" s="34" t="str">
+        <x:v>Long 14 km
+Long easy 12 km @ 5:15–5:50/km, RPE 3–4</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2099,7 +2267,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F26" s="21" t="str">
-        <x:v>Recovery run</x:v>
+        <x:v>Recovery 5 km</x:v>
       </x:c>
       <x:c r="G26" s="21" t="str">
         <x:v>RECOVERY</x:v>
@@ -2143,12 +2311,17 @@
         <x:v>cc-v2-oslo-2026-2026-08-02-run-1</x:v>
       </x:c>
       <x:c r="V26" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Recovery 3km 5:40/km-6:20/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W26" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W26" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X26" s="34" t="str">
+        <x:v>Recovery 5 km
+Tempo: 5:40–6:20/km
+RPE: 2–3</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2168,7 +2341,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F27" s="21" t="str">
-        <x:v>Regeneracja + opcjonalna siła techniczna</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G27" s="21" t="str">
         <x:v>REST</x:v>
@@ -2198,10 +2371,13 @@
         <x:v>cc-v2-oslo-2026-2026-08-03-note-1</x:v>
       </x:c>
       <x:c r="V27" s="30" t="str">
-        <x:v>Regeneracja</x:v>
-      </x:c>
-      <x:c r="W27" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W27" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X27" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -2221,7 +2397,7 @@
         <x:v>Strength</x:v>
       </x:c>
       <x:c r="F28" s="21" t="str">
-        <x:v>Siła techniczna — bez DOMS</x:v>
+        <x:v>Siła — 20 min</x:v>
       </x:c>
       <x:c r="G28" s="21" t="str">
         <x:v>STRENGTH</x:v>
@@ -2259,10 +2435,23 @@
         <x:v>cc-v2-oslo-2026-2026-08-03-strength-1</x:v>
       </x:c>
       <x:c r="V28" s="30" t="str">
-        <x:v>- Technika i stabilizacja 20m 2-4 RPE</x:v>
-      </x:c>
-      <x:c r="W28" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Siła — 20 min
+- Split squat 1–2 serie
+- Wspięcia łydki 1–2 serie
+- Hip hinge 1–2 serie
+- Side plank 1–2 serie
+- RPE: 2–4</x:v>
+      </x:c>
+      <x:c r="W28" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X28" s="34" t="str">
+        <x:v>Siła — 20 min
+Split squat 1–2 serie
+Wspięcia łydki 1–2 serie
+Hip hinge 1–2 serie
+Side plank 1–2 serie
+RPE: 2–4</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2282,7 +2471,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F29" s="21" t="str">
-        <x:v>Próg 4 × 1 km</x:v>
+        <x:v>Threshold 9 km</x:v>
       </x:c>
       <x:c r="G29" s="21" t="str">
         <x:v>THRESHOLD</x:v>
@@ -2326,14 +2515,23 @@
         <x:v>cc-v2-oslo-2026-2026-08-04-run-1</x:v>
       </x:c>
       <x:c r="V29" s="30" t="str">
-        <x:v>- Warmup 2km 5:30/km-6:05/km Pace
-Threshold 4x
-- Threshold 1km 4:12/km-4:20/km Pace
-- Recovery 2m 5:40/km-6:20/km Pace
-- Cooldown 2km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W29" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rozgrzewka 2km 5:30/km-6:05/km Pace
+Próg 4x
+- Próg 1km 4:12/km-4:20/km Pace
+- Trucht 2m 5:40/km-6:20/km Pace
+- Schłodzenie 2km 5:35/km-6:15/km Pace
+Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
+      </x:c>
+      <x:c r="W29" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X29" s="34" t="str">
+        <x:v>Threshold 9 km
+WU: 2 km @ 5:30–6:05/km
+4 × Próg 1 km @ 4:12–4:20/km, RPE 7
+Przerwa: 2 min @ 5:40–6:20/km
+CD: 2 km @ 5:35–6:15/km
+Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2353,7 +2551,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F30" s="21" t="str">
-        <x:v>WOLNE (alternatywa dla roweru)</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G30" s="21" t="str">
         <x:v>REST</x:v>
@@ -2383,10 +2581,19 @@
         <x:v>cc-v2-oslo-2026-2026-08-05-note-1</x:v>
       </x:c>
       <x:c r="V30" s="30" t="str">
-        <x:v>Pełne wolne</x:v>
-      </x:c>
-      <x:c r="W30" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 40 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
+      </x:c>
+      <x:c r="W30" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X30" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 40 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2406,7 +2613,7 @@
         <x:v>Ride</x:v>
       </x:c>
       <x:c r="F31" s="21" t="str">
-        <x:v>ALT: rower Z2 albo pełne wolne</x:v>
+        <x:v>Rower Z2 — 40 min</x:v>
       </x:c>
       <x:c r="G31" s="21" t="str">
         <x:v>ENDURANCE</x:v>
@@ -2448,10 +2655,16 @@
         <x:v>cc-v2-oslo-2026-2026-08-05-ride-alt</x:v>
       </x:c>
       <x:c r="V31" s="30" t="str">
-        <x:v>- Easy spin 40m 55-70% 85-95rpm</x:v>
-      </x:c>
-      <x:c r="W31" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rower Z2 40m 3 RPE</x:v>
+      </x:c>
+      <x:c r="W31" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X31" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 40 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2471,7 +2684,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F32" s="21" t="str">
-        <x:v>Średnio-długi easy</x:v>
+        <x:v>Średnio-długi 10 km</x:v>
       </x:c>
       <x:c r="G32" s="21" t="str">
         <x:v>MEDIUM_LONG</x:v>
@@ -2515,12 +2728,17 @@
         <x:v>cc-v2-oslo-2026-2026-08-06-run-1</x:v>
       </x:c>
       <x:c r="V32" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
-- Średnio-długi easy 8km 5:05/km-5:35/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W32" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
+- Easy 8km 5:05/km-5:35/km Pace
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W32" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X32" s="34" t="str">
+        <x:v>Średnio-długi 10 km
+Tempo: 5:05–5:35/km
+RPE: 3–4</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -2540,7 +2758,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F33" s="21" t="str">
-        <x:v>WOLNE przed long runem</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G33" s="21" t="str">
         <x:v>REST</x:v>
@@ -2570,10 +2788,13 @@
         <x:v>cc-v2-oslo-2026-2026-08-07-note-1</x:v>
       </x:c>
       <x:c r="V33" s="30" t="str">
-        <x:v>WOLNE przed long runem</x:v>
-      </x:c>
-      <x:c r="W33" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W33" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X33" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -2593,7 +2814,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F34" s="21" t="str">
-        <x:v>Long easy 12 km — cutback</x:v>
+        <x:v>Long 12 km</x:v>
       </x:c>
       <x:c r="G34" s="21" t="str">
         <x:v>LONG_RUN</x:v>
@@ -2637,12 +2858,16 @@
         <x:v>cc-v2-oslo-2026-2026-08-08-run-1</x:v>
       </x:c>
       <x:c r="V34" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Long easy 10km 5:15/km-5:50/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W34" s="24" t="n">
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W34" s="21" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="X34" s="34" t="str">
+        <x:v>Long 12 km
+Long easy 10 km @ 5:15–5:50/km, RPE 3–4</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -2662,7 +2887,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F35" s="21" t="str">
-        <x:v>Recovery run</x:v>
+        <x:v>Recovery 5 km</x:v>
       </x:c>
       <x:c r="G35" s="21" t="str">
         <x:v>RECOVERY</x:v>
@@ -2706,12 +2931,17 @@
         <x:v>cc-v2-oslo-2026-2026-08-09-run-1</x:v>
       </x:c>
       <x:c r="V35" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Recovery 3km 5:40/km-6:20/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W35" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W35" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X35" s="34" t="str">
+        <x:v>Recovery 5 km
+Tempo: 5:40–6:20/km
+RPE: 2–3</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2731,7 +2961,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F36" s="21" t="str">
-        <x:v>Regeneracja + opcjonalna siła lekka</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G36" s="21" t="str">
         <x:v>REST</x:v>
@@ -2761,10 +2991,13 @@
         <x:v>cc-v2-oslo-2026-2026-08-10-note-1</x:v>
       </x:c>
       <x:c r="V36" s="30" t="str">
-        <x:v>Regeneracja</x:v>
-      </x:c>
-      <x:c r="W36" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W36" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X36" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -2784,7 +3017,7 @@
         <x:v>Strength</x:v>
       </x:c>
       <x:c r="F37" s="21" t="str">
-        <x:v>Siła podtrzymująca — lekka</x:v>
+        <x:v>Siła — 20 min</x:v>
       </x:c>
       <x:c r="G37" s="21" t="str">
         <x:v>STRENGTH</x:v>
@@ -2822,10 +3055,23 @@
         <x:v>cc-v2-oslo-2026-2026-08-10-strength-1</x:v>
       </x:c>
       <x:c r="V37" s="30" t="str">
-        <x:v>- Technika i stabilizacja 20m 2-4 RPE</x:v>
-      </x:c>
-      <x:c r="W37" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Siła — 20 min
+- Split squat 1–2 serie
+- Wspięcia łydki 1–2 serie
+- Hip hinge 1–2 serie
+- Side plank 1–2 serie
+- RPE: 2–4</x:v>
+      </x:c>
+      <x:c r="W37" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X37" s="34" t="str">
+        <x:v>Siła — 20 min
+Split squat 1–2 serie
+Wspięcia łydki 1–2 serie
+Hip hinge 1–2 serie
+Side plank 1–2 serie
+RPE: 2–4</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -2845,7 +3091,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F38" s="21" t="str">
-        <x:v>Długie podbiegi 4 × 3 min</x:v>
+        <x:v>Podbiegi 10 km</x:v>
       </x:c>
       <x:c r="G38" s="21" t="str">
         <x:v>HILLS</x:v>
@@ -2891,14 +3137,22 @@
         <x:v>cc-v2-oslo-2026-2026-08-11-run-1</x:v>
       </x:c>
       <x:c r="V38" s="30" t="str">
-        <x:v>- Warmup 2.5km 5:30/km-6:05/km Pace
-Uphill effort 4x
-- Uphill 180s 7 RPE
-- Full jog-down recovery 180s open
-- Cooldown 2km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W38" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rozgrzewka 2.5km 5:30/km-6:05/km Pace
+Podbieg 4x
+- Podbieg 180s 7 RPE
+- Powrót 180s open
+- Schłodzenie 2km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W38" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X38" s="34" t="str">
+        <x:v>Podbiegi 10 km
+WU: 2,5 km @ 5:30–6:05/km
+4 × Podbieg 180 s, nachylenie 4–7%, RPE 7
+Powrót: 180 s trucht w dół
+CD: 2 km @ 5:35–6:15/km
+Bez targetu tempa pod górę.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2918,7 +3172,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F39" s="21" t="str">
-        <x:v>WOLNE (alternatywa ALT)</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G39" s="21" t="str">
         <x:v>REST</x:v>
@@ -2948,10 +3202,21 @@
         <x:v>cc-v2-oslo-2026-2026-08-12-note-1</x:v>
       </x:c>
       <x:c r="V39" s="30" t="str">
-        <x:v>Pełne wolne</x:v>
-      </x:c>
-      <x:c r="W39" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>Wybierz jedną opcję:
+A: Recovery 5 km @ 5:40–6:20/km
+B: Rower Z2 45 min, RPE 3
+C: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
+      </x:c>
+      <x:c r="W39" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X39" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Recovery 5 km @ 5:40–6:20/km
+B: Rower Z2 45 min, RPE 3
+C: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2971,7 +3236,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F40" s="21" t="str">
-        <x:v>ALT: recovery run</x:v>
+        <x:v>Recovery 5 km</x:v>
       </x:c>
       <x:c r="G40" s="21" t="str">
         <x:v>RECOVERY</x:v>
@@ -3015,12 +3280,19 @@
         <x:v>cc-v2-oslo-2026-2026-08-12-run-alt</x:v>
       </x:c>
       <x:c r="V40" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Recovery 3km 5:40/km-6:20/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W40" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W40" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X40" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Recovery 5 km @ 5:40–6:20/km
+B: Rower Z2 45 min, RPE 3
+C: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -3040,7 +3312,7 @@
         <x:v>Ride</x:v>
       </x:c>
       <x:c r="F41" s="21" t="str">
-        <x:v>ALT: rower Z2 albo pełne wolne</x:v>
+        <x:v>Rower Z2 — 45 min</x:v>
       </x:c>
       <x:c r="G41" s="21" t="str">
         <x:v>ENDURANCE</x:v>
@@ -3082,10 +3354,17 @@
         <x:v>cc-v2-oslo-2026-2026-08-12-ride-alt</x:v>
       </x:c>
       <x:c r="V41" s="30" t="str">
-        <x:v>- Easy spin 45m 55-70% 85-95rpm</x:v>
-      </x:c>
-      <x:c r="W41" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rower Z2 45m 3 RPE</x:v>
+      </x:c>
+      <x:c r="W41" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X41" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Recovery 5 km @ 5:40–6:20/km
+B: Rower Z2 45 min, RPE 3
+C: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -3105,7 +3384,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F42" s="21" t="str">
-        <x:v>Średnio-długi easy/steady</x:v>
+        <x:v>Średnio-długi 11 km</x:v>
       </x:c>
       <x:c r="G42" s="21" t="str">
         <x:v>MEDIUM_LONG</x:v>
@@ -3149,13 +3428,20 @@
         <x:v>cc-v2-oslo-2026-2026-08-13-run-1</x:v>
       </x:c>
       <x:c r="V42" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
-- Medium long easy 6km 5:05/km-5:35/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
+- Easy 6km 5:05/km-5:35/km Pace
 - Steady 3km 4:40/km-4:55/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W42" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W42" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X42" s="34" t="str">
+        <x:v>Średnio-długi 11 km
+WU: 1 km @ 5:30–6:05/km
+Easy 6 km @ 5:05–5:35/km, RPE 3–4
+Steady 3 km @ 4:40–4:55/km, RPE 5–6
+CD: 1 km @ 5:35–6:15/km</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -3175,7 +3461,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F43" s="21" t="str">
-        <x:v>WOLNE przed bramką 18–20 km</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G43" s="21" t="str">
         <x:v>REST</x:v>
@@ -3205,10 +3491,13 @@
         <x:v>cc-v2-oslo-2026-2026-08-14-note-1</x:v>
       </x:c>
       <x:c r="V43" s="30" t="str">
-        <x:v>WOLNE przed bramką 18–20 km</x:v>
-      </x:c>
-      <x:c r="W43" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W43" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X43" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -3228,7 +3517,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F44" s="21" t="str">
-        <x:v>BRAMKA A: long 18–20 km</x:v>
+        <x:v>Long 18–20 km</x:v>
       </x:c>
       <x:c r="G44" s="21" t="str">
         <x:v>LONG_RUN_GATE</x:v>
@@ -3274,13 +3563,20 @@
         <x:v>cc-v2-oslo-2026-2026-08-15-run-1</x:v>
       </x:c>
       <x:c r="V44" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Long easy 15km 5:15/km-5:50/km Pace
-- Conditional goal MP 3km 4:55/km-5:02/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W44" s="24" t="n">
+- MP 3km 4:55/km-5:02/km Pace
+- Schłodzenie 1km 5:35/km-6:15/km Pace
+Plan B: 18 km easy bez MP.</x:v>
+      </x:c>
+      <x:c r="W44" s="21" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="X44" s="34" t="str">
+        <x:v>Long 18–20 km
+Long easy 15 km @ 5:15–5:50/km, RPE 3–4
+MP 3 km @ 4:55–5:02/km, RPE ≤6
+Plan B: 18 km easy bez MP.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -3300,7 +3596,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F45" s="21" t="str">
-        <x:v>Recovery run</x:v>
+        <x:v>Recovery 4 km</x:v>
       </x:c>
       <x:c r="G45" s="21" t="str">
         <x:v>RECOVERY</x:v>
@@ -3346,12 +3642,17 @@
         <x:v>cc-v2-oslo-2026-2026-08-16-run-1</x:v>
       </x:c>
       <x:c r="V45" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Recovery 2km 5:40/km-6:20/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W45" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W45" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X45" s="34" t="str">
+        <x:v>Recovery 4 km
+Tempo: 5:40–6:20/km
+RPE: 2–3</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -3371,7 +3672,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F46" s="21" t="str">
-        <x:v>Regeneracja + opcjonalna siła lekka</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G46" s="21" t="str">
         <x:v>REST</x:v>
@@ -3401,10 +3702,13 @@
         <x:v>cc-v2-oslo-2026-2026-08-17-note-1</x:v>
       </x:c>
       <x:c r="V46" s="30" t="str">
-        <x:v>Regeneracja</x:v>
-      </x:c>
-      <x:c r="W46" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W46" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X46" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -3424,7 +3728,7 @@
         <x:v>Strength</x:v>
       </x:c>
       <x:c r="F47" s="21" t="str">
-        <x:v>Siła podtrzymująca — bez ekscentrycznego zmęczenia</x:v>
+        <x:v>Siła — 18 min</x:v>
       </x:c>
       <x:c r="G47" s="21" t="str">
         <x:v>STRENGTH</x:v>
@@ -3462,10 +3766,23 @@
         <x:v>cc-v2-oslo-2026-2026-08-17-strength-1</x:v>
       </x:c>
       <x:c r="V47" s="30" t="str">
-        <x:v>- Technika i stabilizacja 18m 2-4 RPE</x:v>
-      </x:c>
-      <x:c r="W47" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Siła — 18 min
+- Split squat 1–2 serie
+- Wspięcia łydki 1–2 serie
+- Hip hinge 1–2 serie
+- Side plank 1–2 serie
+- RPE: 2–4</x:v>
+      </x:c>
+      <x:c r="W47" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X47" s="34" t="str">
+        <x:v>Siła — 18 min
+Split squat 1–2 serie
+Wspięcia łydki 1–2 serie
+Hip hinge 1–2 serie
+Side plank 1–2 serie
+RPE: 2–4</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -3485,7 +3802,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F48" s="21" t="str">
-        <x:v>Próg 3 × 2 km</x:v>
+        <x:v>Threshold 9 km</x:v>
       </x:c>
       <x:c r="G48" s="21" t="str">
         <x:v>THRESHOLD</x:v>
@@ -3529,14 +3846,23 @@
         <x:v>cc-v2-oslo-2026-2026-08-18-run-1</x:v>
       </x:c>
       <x:c r="V48" s="30" t="str">
-        <x:v>- Warmup 1.5km 5:30/km-6:05/km Pace
-Threshold 3x
-- Threshold 2km 4:12/km-4:20/km Pace
-- Recovery 3m 5:40/km-6:20/km Pace
-- Cooldown 1.5km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W48" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rozgrzewka 1.5km 5:30/km-6:05/km Pace
+Próg 3x
+- Próg 2km 4:12/km-4:20/km Pace
+- Trucht 3m 5:40/km-6:20/km Pace
+- Schłodzenie 1.5km 5:35/km-6:15/km Pace
+Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
+      </x:c>
+      <x:c r="W48" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X48" s="34" t="str">
+        <x:v>Threshold 9 km
+WU: 1,5 km @ 5:30–6:05/km
+3 × Próg 2 km @ 4:12–4:20/km, RPE 7
+Przerwa: 3 min @ 5:40–6:20/km
+CD: 1,5 km @ 5:35–6:15/km
+Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -3556,7 +3882,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F49" s="21" t="str">
-        <x:v>WOLNE (alternatywa ALT)</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G49" s="21" t="str">
         <x:v>REST</x:v>
@@ -3586,10 +3912,21 @@
         <x:v>cc-v2-oslo-2026-2026-08-19-note-1</x:v>
       </x:c>
       <x:c r="V49" s="30" t="str">
-        <x:v>Pełne wolne</x:v>
-      </x:c>
-      <x:c r="W49" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>Wybierz jedną opcję:
+A: Recovery 5 km @ 5:40–6:20/km
+B: Rower Z2 45 min, RPE 3
+C: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
+      </x:c>
+      <x:c r="W49" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X49" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Recovery 5 km @ 5:40–6:20/km
+B: Rower Z2 45 min, RPE 3
+C: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -3609,7 +3946,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F50" s="21" t="str">
-        <x:v>ALT: recovery run</x:v>
+        <x:v>Recovery 5 km</x:v>
       </x:c>
       <x:c r="G50" s="21" t="str">
         <x:v>RECOVERY</x:v>
@@ -3653,12 +3990,19 @@
         <x:v>cc-v2-oslo-2026-2026-08-19-run-alt</x:v>
       </x:c>
       <x:c r="V50" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Recovery 3km 5:40/km-6:20/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W50" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W50" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X50" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Recovery 5 km @ 5:40–6:20/km
+B: Rower Z2 45 min, RPE 3
+C: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -3678,7 +4022,7 @@
         <x:v>Ride</x:v>
       </x:c>
       <x:c r="F51" s="21" t="str">
-        <x:v>ALT: rower Z2 albo pełne wolne</x:v>
+        <x:v>Rower Z2 — 45 min</x:v>
       </x:c>
       <x:c r="G51" s="21" t="str">
         <x:v>ENDURANCE</x:v>
@@ -3720,10 +4064,17 @@
         <x:v>cc-v2-oslo-2026-2026-08-19-ride-alt</x:v>
       </x:c>
       <x:c r="V51" s="30" t="str">
-        <x:v>- Easy spin 45m 55-70% 85-95rpm</x:v>
-      </x:c>
-      <x:c r="W51" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rower Z2 45m 3 RPE</x:v>
+      </x:c>
+      <x:c r="W51" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X51" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Recovery 5 km @ 5:40–6:20/km
+B: Rower Z2 45 min, RPE 3
+C: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -3743,7 +4094,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F52" s="21" t="str">
-        <x:v>Średnio-długi easy</x:v>
+        <x:v>Średnio-długi 11 km</x:v>
       </x:c>
       <x:c r="G52" s="21" t="str">
         <x:v>MEDIUM_LONG</x:v>
@@ -3787,12 +4138,17 @@
         <x:v>cc-v2-oslo-2026-2026-08-20-run-1</x:v>
       </x:c>
       <x:c r="V52" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
-- Średnio-długi easy 9km 5:05/km-5:35/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W52" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
+- Easy 9km 5:05/km-5:35/km Pace
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W52" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X52" s="34" t="str">
+        <x:v>Średnio-długi 11 km
+Tempo: 5:05–5:35/km
+RPE: 3–4</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -3812,7 +4168,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F53" s="21" t="str">
-        <x:v>WOLNE przed bramką 22–24 km</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G53" s="21" t="str">
         <x:v>REST</x:v>
@@ -3842,10 +4198,13 @@
         <x:v>cc-v2-oslo-2026-2026-08-21-note-1</x:v>
       </x:c>
       <x:c r="V53" s="30" t="str">
-        <x:v>WOLNE przed bramką 22–24 km</x:v>
-      </x:c>
-      <x:c r="W53" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W53" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X53" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -3865,7 +4224,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F54" s="21" t="str">
-        <x:v>BRAMKA A: long 22–24 km</x:v>
+        <x:v>Long 22–24 km</x:v>
       </x:c>
       <x:c r="G54" s="21" t="str">
         <x:v>LONG_RUN_GATE</x:v>
@@ -3911,13 +4270,20 @@
         <x:v>cc-v2-oslo-2026-2026-08-22-run-1</x:v>
       </x:c>
       <x:c r="V54" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Long easy 19km 5:15/km-5:50/km Pace
-- Conditional steady 3km 4:40/km-4:55/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W54" s="24" t="n">
+- Steady 3km 4:40/km-4:55/km Pace
+- Schłodzenie 1km 5:35/km-6:15/km Pace
+Plan B: Wybierz dolny dystans bez bloku jakościowego.</x:v>
+      </x:c>
+      <x:c r="W54" s="21" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="X54" s="34" t="str">
+        <x:v>Long 22–24 km
+Long easy 19 km @ 5:15–5:50/km, RPE 3–4
+Steady 3 km @ 4:40–4:55/km, RPE 5–6
+Plan B: Wybierz dolny dystans bez bloku jakościowego.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -3937,7 +4303,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F55" s="21" t="str">
-        <x:v>Recovery run</x:v>
+        <x:v>Recovery 5 km</x:v>
       </x:c>
       <x:c r="G55" s="21" t="str">
         <x:v>RECOVERY</x:v>
@@ -3981,12 +4347,17 @@
         <x:v>cc-v2-oslo-2026-2026-08-23-run-1</x:v>
       </x:c>
       <x:c r="V55" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Recovery 3km 5:40/km-6:20/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W55" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W55" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X55" s="34" t="str">
+        <x:v>Recovery 5 km
+Tempo: 5:40–6:20/km
+RPE: 2–3</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -4006,7 +4377,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F56" s="21" t="str">
-        <x:v>Regeneracja + opcjonalna siła lekka</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G56" s="21" t="str">
         <x:v>REST</x:v>
@@ -4036,10 +4407,13 @@
         <x:v>cc-v2-oslo-2026-2026-08-24-note-1</x:v>
       </x:c>
       <x:c r="V56" s="30" t="str">
-        <x:v>Regeneracja</x:v>
-      </x:c>
-      <x:c r="W56" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W56" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X56" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -4059,7 +4433,7 @@
         <x:v>Strength</x:v>
       </x:c>
       <x:c r="F57" s="21" t="str">
-        <x:v>Siła podtrzymująca — lekka</x:v>
+        <x:v>Siła — 18 min</x:v>
       </x:c>
       <x:c r="G57" s="21" t="str">
         <x:v>STRENGTH</x:v>
@@ -4097,10 +4471,23 @@
         <x:v>cc-v2-oslo-2026-2026-08-24-strength-1</x:v>
       </x:c>
       <x:c r="V57" s="30" t="str">
-        <x:v>- Technika i stabilizacja 18m 2-4 RPE</x:v>
-      </x:c>
-      <x:c r="W57" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Siła — 18 min
+- Split squat 1–2 serie
+- Wspięcia łydki 1–2 serie
+- Hip hinge 1–2 serie
+- Side plank 1–2 serie
+- RPE: 2–4</x:v>
+      </x:c>
+      <x:c r="W57" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X57" s="34" t="str">
+        <x:v>Siła — 18 min
+Split squat 1–2 serie
+Wspięcia łydki 1–2 serie
+Hip hinge 1–2 serie
+Side plank 1–2 serie
+RPE: 2–4</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -4166,13 +4553,22 @@
         <x:v>cc-v2-oslo-2026-2026-08-25-run-1</x:v>
       </x:c>
       <x:c r="V58" s="30" t="str">
-        <x:v>- Warmup 2km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 2km 5:30/km-6:05/km Pace
 - Steady 6km 4:40/km-4:55/km Pace
-- Conditional goal MP instead 6km 4:55/km-5:02/km Pace
-- Cooldown 2km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W58" s="24" t="n">
-        <x:v>0</x:v>
+- MP 6km 4:55/km-5:02/km Pace
+- Schłodzenie 2km 5:35/km-6:15/km Pace
+Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
+      </x:c>
+      <x:c r="W58" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X58" s="34" t="str">
+        <x:v>Steady 6 km / warunkowo goal MP
+WU: 2 km @ 5:30–6:05/km
+Steady 6 km @ 4:40–4:55/km, RPE 5–6
+MP 6 km @ 4:55–5:02/km, RPE ≤6
+CD: 2 km @ 5:35–6:15/km
+Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -4192,7 +4588,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F59" s="21" t="str">
-        <x:v>WOLNE (alternatywa ALT)</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G59" s="21" t="str">
         <x:v>REST</x:v>
@@ -4222,10 +4618,21 @@
         <x:v>cc-v2-oslo-2026-2026-08-26-note-1</x:v>
       </x:c>
       <x:c r="V59" s="30" t="str">
-        <x:v>Pełne wolne</x:v>
-      </x:c>
-      <x:c r="W59" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>Wybierz jedną opcję:
+A: Recovery 5 km @ 5:40–6:20/km
+B: Rower Z2 40 min, RPE 3
+C: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
+      </x:c>
+      <x:c r="W59" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X59" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Recovery 5 km @ 5:40–6:20/km
+B: Rower Z2 40 min, RPE 3
+C: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -4245,7 +4652,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F60" s="21" t="str">
-        <x:v>ALT: recovery run</x:v>
+        <x:v>Recovery 5 km</x:v>
       </x:c>
       <x:c r="G60" s="21" t="str">
         <x:v>RECOVERY</x:v>
@@ -4289,12 +4696,19 @@
         <x:v>cc-v2-oslo-2026-2026-08-26-run-alt</x:v>
       </x:c>
       <x:c r="V60" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Recovery 3km 5:40/km-6:20/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W60" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W60" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X60" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Recovery 5 km @ 5:40–6:20/km
+B: Rower Z2 40 min, RPE 3
+C: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -4314,7 +4728,7 @@
         <x:v>Ride</x:v>
       </x:c>
       <x:c r="F61" s="21" t="str">
-        <x:v>ALT: rower Z2 albo pełne wolne</x:v>
+        <x:v>Rower Z2 — 40 min</x:v>
       </x:c>
       <x:c r="G61" s="21" t="str">
         <x:v>ENDURANCE</x:v>
@@ -4356,10 +4770,17 @@
         <x:v>cc-v2-oslo-2026-2026-08-26-ride-alt</x:v>
       </x:c>
       <x:c r="V61" s="30" t="str">
-        <x:v>- Easy spin 40m 55-70% 85-95rpm</x:v>
-      </x:c>
-      <x:c r="W61" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rower Z2 40m 3 RPE</x:v>
+      </x:c>
+      <x:c r="W61" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X61" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Recovery 5 km @ 5:40–6:20/km
+B: Rower Z2 40 min, RPE 3
+C: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -4379,7 +4800,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F62" s="21" t="str">
-        <x:v>Średnio-długi easy + hill sprints</x:v>
+        <x:v>Easy 10 km + hill sprints</x:v>
       </x:c>
       <x:c r="G62" s="21" t="str">
         <x:v>MEDIUM_LONG</x:v>
@@ -4425,15 +4846,22 @@
         <x:v>cc-v2-oslo-2026-2026-08-27-run-1</x:v>
       </x:c>
       <x:c r="V62" s="30" t="str">
-        <x:v>- Warmup 2km 5:30/km-6:05/km Pace
-- Medium long easy 7km 5:05/km-5:35/km Pace
-Hill sprints 6x
-- Uphill fast relaxed 10s 8 RPE
-- Full walk-jog recovery 2m open
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W62" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rozgrzewka 2km 5:30/km-6:05/km Pace
+- Easy 7km 5:05/km-5:35/km Pace
+Podbieg 6x
+- Podbieg 10s 8 RPE
+- Powrót 120s open
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W62" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X62" s="34" t="str">
+        <x:v>Easy 10 km + hill sprints
+Easy 7 km @ 5:05–5:35/km, RPE 3–4
+6 × Podbieg 10 s, nachylenie 4–6%, RPE 8
+Powrót: 120 s trucht w dół
+Bez targetu tempa pod górę.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -4453,7 +4881,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F63" s="21" t="str">
-        <x:v>WOLNE przed long runem</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G63" s="21" t="str">
         <x:v>REST</x:v>
@@ -4483,10 +4911,13 @@
         <x:v>cc-v2-oslo-2026-2026-08-28-note-1</x:v>
       </x:c>
       <x:c r="V63" s="30" t="str">
-        <x:v>WOLNE przed long runem</x:v>
-      </x:c>
-      <x:c r="W63" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W63" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X63" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -4506,7 +4937,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F64" s="21" t="str">
-        <x:v>Long pofałdowany 16 km</x:v>
+        <x:v>Long 16 km</x:v>
       </x:c>
       <x:c r="G64" s="21" t="str">
         <x:v>LONG_RUN_HILLY</x:v>
@@ -4550,12 +4981,16 @@
         <x:v>cc-v2-oslo-2026-2026-08-29-run-1</x:v>
       </x:c>
       <x:c r="V64" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Long easy 14km 5:15/km-5:50/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W64" s="24" t="n">
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W64" s="21" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="X64" s="34" t="str">
+        <x:v>Long 16 km
+Long easy 14 km @ 5:15–5:50/km, RPE 3–4</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -4575,7 +5010,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F65" s="21" t="str">
-        <x:v>Recovery run</x:v>
+        <x:v>Recovery 5 km</x:v>
       </x:c>
       <x:c r="G65" s="21" t="str">
         <x:v>RECOVERY</x:v>
@@ -4619,12 +5054,17 @@
         <x:v>cc-v2-oslo-2026-2026-08-30-run-1</x:v>
       </x:c>
       <x:c r="V65" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Recovery 3km 5:40/km-6:20/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W65" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W65" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X65" s="34" t="str">
+        <x:v>Recovery 5 km
+Tempo: 5:40–6:20/km
+RPE: 2–3</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -4644,7 +5084,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F66" s="21" t="str">
-        <x:v>Regeneracja + opcjonalna aktywacja</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G66" s="21" t="str">
         <x:v>REST</x:v>
@@ -4674,10 +5114,13 @@
         <x:v>cc-v2-oslo-2026-2026-08-31-note-1</x:v>
       </x:c>
       <x:c r="V66" s="30" t="str">
-        <x:v>Regeneracja</x:v>
-      </x:c>
-      <x:c r="W66" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W66" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X66" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -4697,7 +5140,7 @@
         <x:v>Strength</x:v>
       </x:c>
       <x:c r="F67" s="21" t="str">
-        <x:v>Mobilność + aktywacja</x:v>
+        <x:v>Siła — 12 min</x:v>
       </x:c>
       <x:c r="G67" s="21" t="str">
         <x:v>STRENGTH</x:v>
@@ -4735,10 +5178,23 @@
         <x:v>cc-v2-oslo-2026-2026-08-31-strength-1</x:v>
       </x:c>
       <x:c r="V67" s="30" t="str">
-        <x:v>- Mobility and activation 12m 2 RPE</x:v>
-      </x:c>
-      <x:c r="W67" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Siła — 12 min
+- Mobilność bioder
+- Most biodrowy
+- Dead bug
+- Wspięcia łydki
+- RPE: 2–4</x:v>
+      </x:c>
+      <x:c r="W67" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X67" s="34" t="str">
+        <x:v>Siła — 12 min
+Mobilność bioder
+Most biodrowy
+Dead bug
+Wspięcia łydki
+RPE: 2–4</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -4804,14 +5260,23 @@
         <x:v>cc-v2-oslo-2026-2026-09-01-run-1</x:v>
       </x:c>
       <x:c r="V68" s="30" t="str">
-        <x:v>- Warmup 2km 5:30/km-6:05/km Pace
-Conditional goal MP calibration 3x
-- Goal MP 2km 4:55/km-5:02/km Pace
-- Recovery 500m 5:40/km-6:20/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W68" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rozgrzewka 2km 5:30/km-6:05/km Pace
+MP 3x
+- MP 2km 4:55/km-5:02/km Pace
+- Trucht 0.5km 5:40/km-6:20/km Pace
+- Schłodzenie 1km 5:35/km-6:15/km Pace
+Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
+      </x:c>
+      <x:c r="W68" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X68" s="34" t="str">
+        <x:v>BRAMKA A: kalibracja tempa 3 × 2 km
+WU: 2 km @ 5:30–6:05/km
+3 × MP 2 km @ 4:55–5:02/km, RPE ≤6
+Przerwa: 0,5 km @ 5:40–6:20/km
+CD: 1 km @ 5:35–6:15/km
+Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -4865,10 +5330,13 @@
         <x:v>cc-v2-oslo-2026-2026-09-02-decision-1</x:v>
       </x:c>
       <x:c r="V69" s="30" t="str">
-        <x:v>Plan A 3:30 | Plan B 3:42–3:45 | Plan C 3:48–3:55</x:v>
-      </x:c>
-      <x:c r="W69" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>DECYZJA STARTOWA A / B / C</x:v>
+      </x:c>
+      <x:c r="W69" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X69" s="34" t="str">
+        <x:v>DECYZJA STARTOWA A / B / C</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -4888,7 +5356,7 @@
         <x:v>Ride</x:v>
       </x:c>
       <x:c r="F70" s="21" t="str">
-        <x:v>ALT: rower Z2 albo pełne wolne</x:v>
+        <x:v>Rower Z2 — 30 min</x:v>
       </x:c>
       <x:c r="G70" s="21" t="str">
         <x:v>ENDURANCE</x:v>
@@ -4930,10 +5398,15 @@
         <x:v>cc-v2-oslo-2026-2026-09-02-ride-alt</x:v>
       </x:c>
       <x:c r="V70" s="30" t="str">
-        <x:v>- Easy spin 30m 55-70% 85-95rpm</x:v>
-      </x:c>
-      <x:c r="W70" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rower Z2 30m 3 RPE</x:v>
+      </x:c>
+      <x:c r="W70" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X70" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 30 min, RPE 3
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -4953,7 +5426,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F71" s="21" t="str">
-        <x:v>Easy + 4 rytmy</x:v>
+        <x:v>Easy 8 km + rytmy</x:v>
       </x:c>
       <x:c r="G71" s="21" t="str">
         <x:v>EASY_STRIDES</x:v>
@@ -4997,15 +5470,21 @@
         <x:v>cc-v2-oslo-2026-2026-09-03-run-1</x:v>
       </x:c>
       <x:c r="V71" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Easy 6km 5:10/km-5:45/km Pace
-Strides 4x
-- Fast relaxed 15s 7-8 RPE
-- Full recovery 90s open
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W71" s="24" t="n">
-        <x:v>0</x:v>
+Rytm 4x
+- Rytm 15s 7–8 RPE
+- Trucht 90s open
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W71" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X71" s="34" t="str">
+        <x:v>Easy 8 km + rytmy
+Easy 6 km @ 5:10–5:45/km, RPE 3–4
+4 × Rytm 15 s, RPE 7–8
+Przerwa: 90 s easy</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -5025,7 +5504,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F72" s="21" t="str">
-        <x:v>WOLNE przed krótkim longiem</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G72" s="21" t="str">
         <x:v>REST</x:v>
@@ -5055,10 +5534,13 @@
         <x:v>cc-v2-oslo-2026-2026-09-04-note-1</x:v>
       </x:c>
       <x:c r="V72" s="30" t="str">
-        <x:v>WOLNE przed krótkim longiem</x:v>
-      </x:c>
-      <x:c r="W72" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W72" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X72" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -5078,7 +5560,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F73" s="21" t="str">
-        <x:v>Long easy taper 8 km</x:v>
+        <x:v>Long 8 km</x:v>
       </x:c>
       <x:c r="G73" s="21" t="str">
         <x:v>LONG_RUN_TAPER</x:v>
@@ -5122,12 +5604,16 @@
         <x:v>cc-v2-oslo-2026-2026-09-05-run-1</x:v>
       </x:c>
       <x:c r="V73" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Long easy 6km 5:15/km-5:50/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W73" s="24" t="n">
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W73" s="21" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="X73" s="34" t="str">
+        <x:v>Long 8 km
+Long easy 6 km @ 5:15–5:50/km, RPE 3–4</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -5147,7 +5633,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F74" s="21" t="str">
-        <x:v>Recovery run</x:v>
+        <x:v>Recovery 4 km</x:v>
       </x:c>
       <x:c r="G74" s="21" t="str">
         <x:v>RECOVERY</x:v>
@@ -5191,12 +5677,17 @@
         <x:v>cc-v2-oslo-2026-2026-09-06-run-1</x:v>
       </x:c>
       <x:c r="V74" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Recovery 2km 5:40/km-6:20/km Pace
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W74" s="24" t="n">
-        <x:v>0</x:v>
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W74" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X74" s="34" t="str">
+        <x:v>Recovery 4 km
+Tempo: 5:40–6:20/km
+RPE: 2–3</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -5216,7 +5707,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F75" s="21" t="str">
-        <x:v>WOLNE — początek tygodnia startowego</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G75" s="21" t="str">
         <x:v>REST</x:v>
@@ -5246,10 +5737,13 @@
         <x:v>cc-v2-oslo-2026-2026-09-07-note-1</x:v>
       </x:c>
       <x:c r="V75" s="30" t="str">
-        <x:v>WOLNE — początek tygodnia startowego</x:v>
-      </x:c>
-      <x:c r="W75" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W75" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X75" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -5269,7 +5763,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F76" s="21" t="str">
-        <x:v>Rozruch + rytmy</x:v>
+        <x:v>Easy 5 km + rytmy</x:v>
       </x:c>
       <x:c r="G76" s="21" t="str">
         <x:v>TAPER_SHARPEN</x:v>
@@ -5313,15 +5807,21 @@
         <x:v>cc-v2-oslo-2026-2026-09-08-run-1</x:v>
       </x:c>
       <x:c r="V76" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Easy 3km 5:10/km-5:45/km Pace
-Strides 4x
-- Fast relaxed 15s 7-8 RPE
-- Full recovery 90s open
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W76" s="24" t="n">
-        <x:v>0</x:v>
+Rytm 4x
+- Rytm 15s 7–8 RPE
+- Trucht 90s open
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W76" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X76" s="34" t="str">
+        <x:v>Easy 5 km + rytmy
+Easy 3 km @ 5:10–5:45/km, RPE 3–4
+4 × Rytm 15 s, RPE 7–8
+Przerwa: 90 s easy</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -5341,7 +5841,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F77" s="21" t="str">
-        <x:v>WOLNE (alternatywa dla roweru)</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G77" s="21" t="str">
         <x:v>REST</x:v>
@@ -5371,10 +5871,19 @@
         <x:v>cc-v2-oslo-2026-2026-09-09-note-1</x:v>
       </x:c>
       <x:c r="V77" s="30" t="str">
-        <x:v>Pełne wolne</x:v>
-      </x:c>
-      <x:c r="W77" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 25 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
+      </x:c>
+      <x:c r="W77" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X77" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 25 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -5394,7 +5903,7 @@
         <x:v>Ride</x:v>
       </x:c>
       <x:c r="F78" s="21" t="str">
-        <x:v>ALT: rower Z2 albo pełne wolne</x:v>
+        <x:v>Rower Z2 — 25 min</x:v>
       </x:c>
       <x:c r="G78" s="21" t="str">
         <x:v>ENDURANCE</x:v>
@@ -5436,10 +5945,16 @@
         <x:v>cc-v2-oslo-2026-2026-09-09-ride-alt</x:v>
       </x:c>
       <x:c r="V78" s="30" t="str">
-        <x:v>- Easy spin 25m 55-70% 85-95rpm</x:v>
-      </x:c>
-      <x:c r="W78" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rower Z2 25m 3 RPE</x:v>
+      </x:c>
+      <x:c r="W78" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X78" s="34" t="str">
+        <x:v>Wybierz jedną opcję:
+A: Rower Z2 25 min, RPE 3
+B: Pełne wolne
+Nie wykonuj więcej niż jednej.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -5459,7 +5974,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F79" s="21" t="str">
-        <x:v>Krótki rozruch</x:v>
+        <x:v>Easy 4 km</x:v>
       </x:c>
       <x:c r="G79" s="21" t="str">
         <x:v>TAPER_EASY</x:v>
@@ -5503,15 +6018,21 @@
         <x:v>cc-v2-oslo-2026-2026-09-10-run-1</x:v>
       </x:c>
       <x:c r="V79" s="30" t="str">
-        <x:v>- Warmup 1km 5:30/km-6:05/km Pace
+        <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Easy 2km 5:10/km-5:45/km Pace
-Strides 3x
-- Fast relaxed 10s 7-8 RPE
-- Full recovery 90s open
-- Cooldown 1km 5:35/km-6:15/km Pace</x:v>
-      </x:c>
-      <x:c r="W79" s="24" t="n">
-        <x:v>0</x:v>
+Rytm 3x
+- Rytm 10s 7–8 RPE
+- Trucht 90s open
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
+      </x:c>
+      <x:c r="W79" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X79" s="34" t="str">
+        <x:v>Easy 4 km
+Easy 2 km @ 5:10–5:45/km, RPE 3–4
+3 × Rytm 10 s, RPE 7–8
+Przerwa: 90 s easy</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -5531,7 +6052,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="F80" s="21" t="str">
-        <x:v>WOLNE / logistyka</x:v>
+        <x:v>WOLNE</x:v>
       </x:c>
       <x:c r="G80" s="21" t="str">
         <x:v>REST</x:v>
@@ -5561,10 +6082,13 @@
         <x:v>cc-v2-oslo-2026-2026-09-11-note-1</x:v>
       </x:c>
       <x:c r="V80" s="30" t="str">
-        <x:v>WOLNE / logistyka</x:v>
-      </x:c>
-      <x:c r="W80" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>WOLNE</x:v>
+      </x:c>
+      <x:c r="W80" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X80" s="34" t="str">
+        <x:v>WOLNE</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -5584,7 +6108,7 @@
         <x:v>Run</x:v>
       </x:c>
       <x:c r="F81" s="26" t="str">
-        <x:v>START: OSLO MARATHON</x:v>
+        <x:v>Oslo Marathon — 42,195 km</x:v>
       </x:c>
       <x:c r="G81" s="26" t="str">
         <x:v>RACE</x:v>
@@ -5632,16 +6156,22 @@
         <x:v>cc-v2-oslo-2026-2026-09-12-run-1</x:v>
       </x:c>
       <x:c r="V81" s="32" t="str">
-        <x:v>- Race controlled start 5km 4:58/km-5:02/km Pace
-- Race strategy block 32.195km 4:55/km-5:02/km Pace
-- Finish by feel 5km 5-8 RPE</x:v>
-      </x:c>
-      <x:c r="W81" s="29" t="n">
-        <x:v>0</x:v>
+        <x:v>- Rozgrzewka 12m 5:30/km-6:05/km Pace
+- MP 42.195km 4:55/km-5:02/km Pace
+- Schłodzenie 12m open
+Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
+      </x:c>
+      <x:c r="W81" s="26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X81" s="35" t="str">
+        <x:v>Oslo Marathon — 42,195 km
+Tempo: 4:55–5:02/km
+RPE: 5–7</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:W81">
+  <x:conditionalFormatting sqref="A2:X81">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="OPCJONALNE / ALT"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="BRAMKA"/>
   </x:conditionalFormatting>
@@ -5664,48 +6194,48 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="35" t="str">
+      <x:c r="A1" s="37" t="str">
         <x:v>OSLO 2026 — tygodnie, kilometraż i bramki</x:v>
       </x:c>
-      <x:c r="B1" s="35"/>
-      <x:c r="C1" s="35"/>
-      <x:c r="D1" s="35"/>
-      <x:c r="E1" s="35"/>
-      <x:c r="F1" s="35"/>
-      <x:c r="G1" s="35"/>
-      <x:c r="H1" s="35"/>
+      <x:c r="B1" s="37"/>
+      <x:c r="C1" s="37"/>
+      <x:c r="D1" s="37"/>
+      <x:c r="E1" s="37"/>
+      <x:c r="F1" s="37"/>
+      <x:c r="G1" s="37"/>
+      <x:c r="H1" s="37"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="38" t="str">
+      <x:c r="A3" s="40" t="str">
         <x:v>Tydzień od</x:v>
       </x:c>
-      <x:c r="B3" s="38" t="str">
+      <x:c r="B3" s="40" t="str">
         <x:v>Do</x:v>
       </x:c>
-      <x:c r="C3" s="38" t="str">
+      <x:c r="C3" s="40" t="str">
         <x:v>Biegi obowiązkowe</x:v>
       </x:c>
-      <x:c r="D3" s="38" t="str">
+      <x:c r="D3" s="40" t="str">
         <x:v>Km min</x:v>
       </x:c>
-      <x:c r="E3" s="38" t="str">
+      <x:c r="E3" s="40" t="str">
         <x:v>Km max</x:v>
       </x:c>
-      <x:c r="F3" s="38" t="str">
+      <x:c r="F3" s="40" t="str">
         <x:v>Long min</x:v>
       </x:c>
-      <x:c r="G3" s="38" t="str">
+      <x:c r="G3" s="40" t="str">
         <x:v>Long max</x:v>
       </x:c>
-      <x:c r="H3" s="38" t="str">
+      <x:c r="H3" s="40" t="str">
         <x:v>Kontrola</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="39" t="n">
+      <x:c r="A4" s="41" t="n">
         <x:v>46216.5</x:v>
       </x:c>
-      <x:c r="B4" s="39" t="n">
+      <x:c r="B4" s="41" t="n">
         <x:v>46222.5</x:v>
       </x:c>
       <x:c r="C4" s="12" t="n">
@@ -5728,15 +6258,15 @@
         <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A4,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B4,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="H4" s="40" t="str">
+      <x:c r="H4" s="42" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="39" t="n">
+      <x:c r="A5" s="41" t="n">
         <x:v>46223.5</x:v>
       </x:c>
-      <x:c r="B5" s="39" t="n">
+      <x:c r="B5" s="41" t="n">
         <x:v>46229.5</x:v>
       </x:c>
       <x:c r="C5" s="12" t="n">
@@ -5759,15 +6289,15 @@
         <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A5,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B5,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="H5" s="40" t="str">
+      <x:c r="H5" s="42" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="39" t="n">
+      <x:c r="A6" s="41" t="n">
         <x:v>46230.5</x:v>
       </x:c>
-      <x:c r="B6" s="39" t="n">
+      <x:c r="B6" s="41" t="n">
         <x:v>46236.5</x:v>
       </x:c>
       <x:c r="C6" s="12" t="n">
@@ -5790,15 +6320,15 @@
         <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A6,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B6,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>14</x:v>
       </x:c>
-      <x:c r="H6" s="40" t="str">
+      <x:c r="H6" s="42" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="39" t="n">
+      <x:c r="A7" s="41" t="n">
         <x:v>46237.5</x:v>
       </x:c>
-      <x:c r="B7" s="39" t="n">
+      <x:c r="B7" s="41" t="n">
         <x:v>46243.5</x:v>
       </x:c>
       <x:c r="C7" s="12" t="n">
@@ -5821,15 +6351,15 @@
         <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A7,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B7,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="H7" s="40" t="str">
+      <x:c r="H7" s="42" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="39" t="n">
+      <x:c r="A8" s="41" t="n">
         <x:v>46244.5</x:v>
       </x:c>
-      <x:c r="B8" s="39" t="n">
+      <x:c r="B8" s="41" t="n">
         <x:v>46250.5</x:v>
       </x:c>
       <x:c r="C8" s="12" t="n">
@@ -5852,15 +6382,15 @@
         <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A8,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B8,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="H8" s="40" t="str">
+      <x:c r="H8" s="42" t="str">
         <x:v>15.08: ból 0–2, RPE ≤4, brak pogorszenia</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="39" t="n">
+      <x:c r="A9" s="41" t="n">
         <x:v>46251.5</x:v>
       </x:c>
-      <x:c r="B9" s="39" t="n">
+      <x:c r="B9" s="41" t="n">
         <x:v>46257.5</x:v>
       </x:c>
       <x:c r="C9" s="12" t="n">
@@ -5883,15 +6413,15 @@
         <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A9,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B9,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>24</x:v>
       </x:c>
-      <x:c r="H9" s="40" t="str">
+      <x:c r="H9" s="42" t="str">
         <x:v>22.08 zależne od 15.08</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="39" t="n">
+      <x:c r="A10" s="41" t="n">
         <x:v>46258.5</x:v>
       </x:c>
-      <x:c r="B10" s="39" t="n">
+      <x:c r="B10" s="41" t="n">
         <x:v>46264.5</x:v>
       </x:c>
       <x:c r="C10" s="12" t="n">
@@ -5914,15 +6444,15 @@
         <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A10,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B10,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>16</x:v>
       </x:c>
-      <x:c r="H10" s="40" t="str">
+      <x:c r="H10" s="42" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="39" t="n">
+      <x:c r="A11" s="41" t="n">
         <x:v>46265.5</x:v>
       </x:c>
-      <x:c r="B11" s="39" t="n">
+      <x:c r="B11" s="41" t="n">
         <x:v>46271.5</x:v>
       </x:c>
       <x:c r="C11" s="12" t="n">
@@ -5945,15 +6475,15 @@
         <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A11,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B11,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="H11" s="40" t="str">
+      <x:c r="H11" s="42" t="str">
         <x:v>01.09 test; 02.09 decyzja A/B/C</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="39" t="n">
+      <x:c r="A12" s="41" t="n">
         <x:v>46272.5</x:v>
       </x:c>
-      <x:c r="B12" s="39" t="n">
+      <x:c r="B12" s="41" t="n">
         <x:v>46278.5</x:v>
       </x:c>
       <x:c r="C12" s="12" t="n">
@@ -5976,7 +6506,7 @@
         <x:f>SUMIFS('FAZA 1 - OSLO V2'!$I$2:$I$81,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&gt;="&amp;A12,'FAZA 1 - OSLO V2'!$A$2:$A$81,"&lt;="&amp;B12,'FAZA 1 - OSLO V2'!$W$2:$W$81,1)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H12" s="40" t="str">
+      <x:c r="H12" s="42" t="str">
         <x:v>—</x:v>
       </x:c>
     </x:row>
@@ -5999,24 +6529,24 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="35" t="str">
+      <x:c r="A1" s="37" t="str">
         <x:v>STRATEGIA STARTOWA — decyzja 02.09.2026</x:v>
       </x:c>
-      <x:c r="B1" s="35"/>
-      <x:c r="C1" s="35"/>
-      <x:c r="D1" s="35"/>
+      <x:c r="B1" s="37"/>
+      <x:c r="C1" s="37"/>
+      <x:c r="D1" s="37"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="38" t="str">
+      <x:c r="A3" s="40" t="str">
         <x:v>Wariant</x:v>
       </x:c>
-      <x:c r="B3" s="38" t="str">
+      <x:c r="B3" s="40" t="str">
         <x:v>Cel</x:v>
       </x:c>
-      <x:c r="C3" s="38" t="str">
+      <x:c r="C3" s="40" t="str">
         <x:v>Tempo</x:v>
       </x:c>
-      <x:c r="D3" s="38" t="str">
+      <x:c r="D3" s="40" t="str">
         <x:v>Warunek</x:v>
       </x:c>
     </x:row>
@@ -6063,12 +6593,12 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="43" t="str">
+      <x:c r="A8" s="45" t="str">
         <x:v>Plan A 3:30 pozostaje wyłącznie po zaliczeniu wszystkich bramek: 15.08, 22.08 i 01.09. Ostateczna decyzja: 02.09.</x:v>
       </x:c>
-      <x:c r="B8" s="43"/>
-      <x:c r="C8" s="43"/>
-      <x:c r="D8" s="43"/>
+      <x:c r="B8" s="45"/>
+      <x:c r="C8" s="45"/>
+      <x:c r="D8" s="45"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
fix: preserve structured workout semantics
</commit_message>
<xml_diff>
--- a/source_plan_v2.xlsx
+++ b/source_plan_v2.xlsx
@@ -702,7 +702,7 @@
         <x:v>cc-v2-oslo-2026-2026-07-15-ride-alt</x:v>
       </x:c>
       <x:c r="V3" s="30" t="str">
-        <x:v>- Rower Z2 40m 3 RPE</x:v>
+        <x:v>- Rower Z2 40m 55-70% 85-95rpm</x:v>
       </x:c>
       <x:c r="W3" s="21" t="n">
         <x:v>0</x:v>
@@ -778,7 +778,7 @@
         <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Easy 5km 5:10/km-5:45/km Pace
 Rytm 6x
-- Rytm 20s 7–8 RPE
+- Rytm 20s 7-8 RPE
 - Trucht 90s open
 - Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
@@ -847,12 +847,7 @@
         <x:v>cc-v2-oslo-2026-2026-07-16-strength-1</x:v>
       </x:c>
       <x:c r="V5" s="30" t="str">
-        <x:v>- Siła — 12 min
-- Split squat 1–2 serie
-- Wspięcia łydki 1–2 serie
-- Hip hinge 1–2 serie
-- Side plank 1–2 serie
-- RPE: 2–4</x:v>
+        <x:v>- Siła 12m 2-4 RPE</x:v>
       </x:c>
       <x:c r="W5" s="21" t="n">
         <x:v>0</x:v>
@@ -1182,12 +1177,7 @@
         <x:v>cc-v2-oslo-2026-2026-07-20-strength-1</x:v>
       </x:c>
       <x:c r="V10" s="30" t="str">
-        <x:v>- Siła — 15 min
-- Split squat 1–2 serie
-- Wspięcia łydki 1–2 serie
-- Hip hinge 1–2 serie
-- Side plank 1–2 serie
-- RPE: 2–4</x:v>
+        <x:v>- Siła 15m 2-4 RPE</x:v>
       </x:c>
       <x:c r="W10" s="21" t="n">
         <x:v>0</x:v>
@@ -1266,8 +1256,7 @@
 Próg 3x
 - Próg 1km 4:12/km-4:20/km Pace
 - Trucht 2m 5:40/km-6:20/km Pace
-- Schłodzenie 2km 5:35/km-6:15/km Pace
-Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
+- Schłodzenie 2km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W11" s="21" t="n">
         <x:v>0</x:v>
@@ -1402,7 +1391,7 @@
         <x:v>cc-v2-oslo-2026-2026-07-22-ride-alt</x:v>
       </x:c>
       <x:c r="V13" s="30" t="str">
-        <x:v>- Rower Z2 45m 3 RPE</x:v>
+        <x:v>- Rower Z2 45m 55-70% 85-95rpm</x:v>
       </x:c>
       <x:c r="W13" s="21" t="n">
         <x:v>0</x:v>
@@ -1478,10 +1467,10 @@
       </x:c>
       <x:c r="V14" s="30" t="str">
         <x:v>- Rozgrzewka 2km 5:30/km-6:05/km Pace
-- Easy 7km 5:05/km-5:35/km Pace
+- Medium long easy 7km 5:05/km-5:35/km Pace
 Podbieg 6x
 - Podbieg 8s 8 RPE
-- Powrót 120s open
+- Powrót 2m open
 - Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W14" s="21" t="n">
@@ -1809,12 +1798,7 @@
         <x:v>cc-v2-oslo-2026-2026-07-27-strength-1</x:v>
       </x:c>
       <x:c r="V19" s="30" t="str">
-        <x:v>- Siła — 18 min
-- Split squat 1–2 serie
-- Wspięcia łydki 1–2 serie
-- Hip hinge 1–2 serie
-- Side plank 1–2 serie
-- RPE: 2–4</x:v>
+        <x:v>- Siła 18m 2-4 RPE</x:v>
       </x:c>
       <x:c r="W19" s="21" t="n">
         <x:v>0</x:v>
@@ -2030,7 +2014,7 @@
         <x:v>cc-v2-oslo-2026-2026-07-29-ride-alt</x:v>
       </x:c>
       <x:c r="V22" s="30" t="str">
-        <x:v>- Rower Z2 45m 3 RPE</x:v>
+        <x:v>- Rower Z2 45m 55-70% 85-95rpm</x:v>
       </x:c>
       <x:c r="W22" s="21" t="n">
         <x:v>0</x:v>
@@ -2435,12 +2419,7 @@
         <x:v>cc-v2-oslo-2026-2026-08-03-strength-1</x:v>
       </x:c>
       <x:c r="V28" s="30" t="str">
-        <x:v>- Siła — 20 min
-- Split squat 1–2 serie
-- Wspięcia łydki 1–2 serie
-- Hip hinge 1–2 serie
-- Side plank 1–2 serie
-- RPE: 2–4</x:v>
+        <x:v>- Siła 20m 2-4 RPE</x:v>
       </x:c>
       <x:c r="W28" s="21" t="n">
         <x:v>0</x:v>
@@ -2519,8 +2498,7 @@
 Próg 4x
 - Próg 1km 4:12/km-4:20/km Pace
 - Trucht 2m 5:40/km-6:20/km Pace
-- Schłodzenie 2km 5:35/km-6:15/km Pace
-Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
+- Schłodzenie 2km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W29" s="21" t="n">
         <x:v>0</x:v>
@@ -2655,7 +2633,7 @@
         <x:v>cc-v2-oslo-2026-2026-08-05-ride-alt</x:v>
       </x:c>
       <x:c r="V31" s="30" t="str">
-        <x:v>- Rower Z2 40m 3 RPE</x:v>
+        <x:v>- Rower Z2 40m 55-70% 85-95rpm</x:v>
       </x:c>
       <x:c r="W31" s="21" t="n">
         <x:v>0</x:v>
@@ -3055,12 +3033,7 @@
         <x:v>cc-v2-oslo-2026-2026-08-10-strength-1</x:v>
       </x:c>
       <x:c r="V37" s="30" t="str">
-        <x:v>- Siła — 20 min
-- Split squat 1–2 serie
-- Wspięcia łydki 1–2 serie
-- Hip hinge 1–2 serie
-- Side plank 1–2 serie
-- RPE: 2–4</x:v>
+        <x:v>- Siła 20m 2-4 RPE</x:v>
       </x:c>
       <x:c r="W37" s="21" t="n">
         <x:v>0</x:v>
@@ -3354,7 +3327,7 @@
         <x:v>cc-v2-oslo-2026-2026-08-12-ride-alt</x:v>
       </x:c>
       <x:c r="V41" s="30" t="str">
-        <x:v>- Rower Z2 45m 3 RPE</x:v>
+        <x:v>- Rower Z2 45m 55-70% 85-95rpm</x:v>
       </x:c>
       <x:c r="W41" s="21" t="n">
         <x:v>0</x:v>
@@ -3766,12 +3739,7 @@
         <x:v>cc-v2-oslo-2026-2026-08-17-strength-1</x:v>
       </x:c>
       <x:c r="V47" s="30" t="str">
-        <x:v>- Siła — 18 min
-- Split squat 1–2 serie
-- Wspięcia łydki 1–2 serie
-- Hip hinge 1–2 serie
-- Side plank 1–2 serie
-- RPE: 2–4</x:v>
+        <x:v>- Siła 18m 2-4 RPE</x:v>
       </x:c>
       <x:c r="W47" s="21" t="n">
         <x:v>0</x:v>
@@ -3850,8 +3818,7 @@
 Próg 3x
 - Próg 2km 4:12/km-4:20/km Pace
 - Trucht 3m 5:40/km-6:20/km Pace
-- Schłodzenie 1.5km 5:35/km-6:15/km Pace
-Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
+- Schłodzenie 1.5km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W48" s="21" t="n">
         <x:v>0</x:v>
@@ -4064,7 +4031,7 @@
         <x:v>cc-v2-oslo-2026-2026-08-19-ride-alt</x:v>
       </x:c>
       <x:c r="V51" s="30" t="str">
-        <x:v>- Rower Z2 45m 3 RPE</x:v>
+        <x:v>- Rower Z2 45m 55-70% 85-95rpm</x:v>
       </x:c>
       <x:c r="W51" s="21" t="n">
         <x:v>0</x:v>
@@ -4471,12 +4438,7 @@
         <x:v>cc-v2-oslo-2026-2026-08-24-strength-1</x:v>
       </x:c>
       <x:c r="V57" s="30" t="str">
-        <x:v>- Siła — 18 min
-- Split squat 1–2 serie
-- Wspięcia łydki 1–2 serie
-- Hip hinge 1–2 serie
-- Side plank 1–2 serie
-- RPE: 2–4</x:v>
+        <x:v>- Siła 18m 2-4 RPE</x:v>
       </x:c>
       <x:c r="W57" s="21" t="n">
         <x:v>0</x:v>
@@ -4770,7 +4732,7 @@
         <x:v>cc-v2-oslo-2026-2026-08-26-ride-alt</x:v>
       </x:c>
       <x:c r="V61" s="30" t="str">
-        <x:v>- Rower Z2 40m 3 RPE</x:v>
+        <x:v>- Rower Z2 40m 55-70% 85-95rpm</x:v>
       </x:c>
       <x:c r="W61" s="21" t="n">
         <x:v>0</x:v>
@@ -4847,10 +4809,10 @@
       </x:c>
       <x:c r="V62" s="30" t="str">
         <x:v>- Rozgrzewka 2km 5:30/km-6:05/km Pace
-- Easy 7km 5:05/km-5:35/km Pace
+- Medium long easy 7km 5:05/km-5:35/km Pace
 Podbieg 6x
 - Podbieg 10s 8 RPE
-- Powrót 120s open
+- Powrót 2m open
 - Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W62" s="21" t="n">
@@ -5178,12 +5140,7 @@
         <x:v>cc-v2-oslo-2026-2026-08-31-strength-1</x:v>
       </x:c>
       <x:c r="V67" s="30" t="str">
-        <x:v>- Siła — 12 min
-- Mobilność bioder
-- Most biodrowy
-- Dead bug
-- Wspięcia łydki
-- RPE: 2–4</x:v>
+        <x:v>- Siła 12m 2 RPE</x:v>
       </x:c>
       <x:c r="W67" s="21" t="n">
         <x:v>0</x:v>
@@ -5263,9 +5220,8 @@
         <x:v>- Rozgrzewka 2km 5:30/km-6:05/km Pace
 MP 3x
 - MP 2km 4:55/km-5:02/km Pace
-- Trucht 0.5km 5:40/km-6:20/km Pace
-- Schłodzenie 1km 5:35/km-6:15/km Pace
-Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
+- Trucht 500m 5:40/km-6:20/km Pace
+- Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
       <x:c r="W68" s="21" t="n">
         <x:v>0</x:v>
@@ -5398,7 +5354,7 @@
         <x:v>cc-v2-oslo-2026-2026-09-02-ride-alt</x:v>
       </x:c>
       <x:c r="V70" s="30" t="str">
-        <x:v>- Rower Z2 30m 3 RPE</x:v>
+        <x:v>- Rower Z2 30m 55-70% 85-95rpm</x:v>
       </x:c>
       <x:c r="W70" s="21" t="n">
         <x:v>0</x:v>
@@ -5473,7 +5429,7 @@
         <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Easy 6km 5:10/km-5:45/km Pace
 Rytm 4x
-- Rytm 15s 7–8 RPE
+- Rytm 15s 7-8 RPE
 - Trucht 90s open
 - Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
@@ -5810,7 +5766,7 @@
         <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Easy 3km 5:10/km-5:45/km Pace
 Rytm 4x
-- Rytm 15s 7–8 RPE
+- Rytm 15s 7-8 RPE
 - Trucht 90s open
 - Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
@@ -5945,7 +5901,7 @@
         <x:v>cc-v2-oslo-2026-2026-09-09-ride-alt</x:v>
       </x:c>
       <x:c r="V78" s="30" t="str">
-        <x:v>- Rower Z2 25m 3 RPE</x:v>
+        <x:v>- Rower Z2 25m 55-70% 85-95rpm</x:v>
       </x:c>
       <x:c r="W78" s="21" t="n">
         <x:v>0</x:v>
@@ -6021,7 +5977,7 @@
         <x:v>- Rozgrzewka 1km 5:30/km-6:05/km Pace
 - Easy 2km 5:10/km-5:45/km Pace
 Rytm 3x
-- Rytm 10s 7–8 RPE
+- Rytm 10s 7-8 RPE
 - Trucht 90s open
 - Schłodzenie 1km 5:35/km-6:15/km Pace</x:v>
       </x:c>
@@ -6156,10 +6112,9 @@
         <x:v>cc-v2-oslo-2026-2026-09-12-run-1</x:v>
       </x:c>
       <x:c r="V81" s="32" t="str">
-        <x:v>- Rozgrzewka 12m 5:30/km-6:05/km Pace
-- MP 42.195km 4:55/km-5:02/km Pace
-- Schłodzenie 12m open
-Plan B: Easy albo odpoczynek przy bólu lub wyraźnym zmęczeniu.</x:v>
+        <x:v>- Start 5km 4:58/km-5:02/km Pace
+- MP 32.195km 4:55/km-5:02/km Pace
+- Finisz 5km 5-8 RPE</x:v>
       </x:c>
       <x:c r="W81" s="26" t="n">
         <x:v>0</x:v>

</xml_diff>